<commit_message>
feat: tambah data bal tembakau tanggal 13 September 2026 (No Gud 991-1019) dan sinkronisasi realtime
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F729"/>
+  <dimension ref="A1:F757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15074,20 +15074,580 @@
       </c>
       <c r="F728" s="5" t="n"/>
     </row>
-    <row r="729" ht="22" customHeight="1">
-      <c r="A729" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (724 BAL)</t>
-        </is>
-      </c>
-      <c r="B729" s="4" t="n"/>
-      <c r="C729" s="4" t="n"/>
-      <c r="D729" s="4" t="n"/>
-      <c r="E729" s="4">
-        <f>SUM(E5:E728)</f>
+    <row r="729" ht="20.25" customHeight="1">
+      <c r="A729" s="5" t="n">
+        <v>991</v>
+      </c>
+      <c r="B729" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C729" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D729" s="6" t="inlineStr">
+        <is>
+          <t>280619</t>
+        </is>
+      </c>
+      <c r="E729" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F729" s="5" t="n"/>
+    </row>
+    <row r="730" ht="20.25" customHeight="1">
+      <c r="A730" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="B730" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C730" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D730" s="6" t="inlineStr">
+        <is>
+          <t>280763</t>
+        </is>
+      </c>
+      <c r="E730" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F730" s="5" t="n"/>
+    </row>
+    <row r="731" ht="20.25" customHeight="1">
+      <c r="A731" s="5" t="n">
+        <v>993</v>
+      </c>
+      <c r="B731" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C731" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D731" s="6" t="inlineStr">
+        <is>
+          <t>280618</t>
+        </is>
+      </c>
+      <c r="E731" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F731" s="5" t="n"/>
+    </row>
+    <row r="732" ht="20.25" customHeight="1">
+      <c r="A732" s="5" t="n">
+        <v>994</v>
+      </c>
+      <c r="B732" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C732" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D732" s="6" t="inlineStr">
+        <is>
+          <t>280762</t>
+        </is>
+      </c>
+      <c r="E732" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F732" s="5" t="n"/>
+    </row>
+    <row r="733" ht="20.25" customHeight="1">
+      <c r="A733" s="5" t="n">
+        <v>995</v>
+      </c>
+      <c r="B733" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C733" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D733" s="6" t="inlineStr">
+        <is>
+          <t>39844</t>
+        </is>
+      </c>
+      <c r="E733" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F733" s="5" t="n"/>
+    </row>
+    <row r="734" ht="20.25" customHeight="1">
+      <c r="A734" s="5" t="n">
+        <v>996</v>
+      </c>
+      <c r="B734" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C734" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D734" s="6" t="inlineStr">
+        <is>
+          <t>39843</t>
+        </is>
+      </c>
+      <c r="E734" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F734" s="5" t="n"/>
+    </row>
+    <row r="735" ht="20.25" customHeight="1">
+      <c r="A735" s="5" t="n">
+        <v>997</v>
+      </c>
+      <c r="B735" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C735" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D735" s="6" t="inlineStr">
+        <is>
+          <t>280617</t>
+        </is>
+      </c>
+      <c r="E735" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F735" s="5" t="n"/>
+    </row>
+    <row r="736" ht="20.25" customHeight="1">
+      <c r="A736" s="5" t="n">
+        <v>998</v>
+      </c>
+      <c r="B736" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C736" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D736" s="6" t="inlineStr">
+        <is>
+          <t>280761</t>
+        </is>
+      </c>
+      <c r="E736" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F736" s="5" t="n"/>
+    </row>
+    <row r="737" ht="20.25" customHeight="1">
+      <c r="A737" s="5" t="n">
+        <v>999</v>
+      </c>
+      <c r="B737" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C737" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D737" s="6" t="inlineStr">
+        <is>
+          <t>280616</t>
+        </is>
+      </c>
+      <c r="E737" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F737" s="5" t="n"/>
+    </row>
+    <row r="738" ht="20.25" customHeight="1">
+      <c r="A738" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B738" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C738" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D738" s="6" t="inlineStr">
+        <is>
+          <t>125833</t>
+        </is>
+      </c>
+      <c r="E738" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F738" s="5" t="n"/>
+    </row>
+    <row r="739" ht="20.25" customHeight="1">
+      <c r="A739" s="5" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B739" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C739" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D739" s="6" t="inlineStr">
+        <is>
+          <t>280613</t>
+        </is>
+      </c>
+      <c r="E739" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F739" s="5" t="n"/>
+    </row>
+    <row r="740" ht="20.25" customHeight="1">
+      <c r="A740" s="5" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B740" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C740" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D740" s="6" t="inlineStr">
+        <is>
+          <t>125832</t>
+        </is>
+      </c>
+      <c r="E740" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F740" s="5" t="n"/>
+    </row>
+    <row r="741" ht="20.25" customHeight="1">
+      <c r="A741" s="5" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B741" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C741" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D741" s="6" t="inlineStr">
+        <is>
+          <t>125862</t>
+        </is>
+      </c>
+      <c r="E741" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F741" s="5" t="n"/>
+    </row>
+    <row r="742" ht="20.25" customHeight="1">
+      <c r="A742" s="5" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B742" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C742" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D742" s="6" t="inlineStr">
+        <is>
+          <t>125866</t>
+        </is>
+      </c>
+      <c r="E742" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F742" s="5" t="n"/>
+    </row>
+    <row r="743" ht="20.25" customHeight="1">
+      <c r="A743" s="5" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B743" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C743" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D743" s="6" t="inlineStr">
+        <is>
+          <t>125863</t>
+        </is>
+      </c>
+      <c r="E743" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F743" s="5" t="n"/>
+    </row>
+    <row r="744" ht="20.25" customHeight="1">
+      <c r="A744" s="5" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B744" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C744" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D744" s="6" t="inlineStr">
+        <is>
+          <t>125864</t>
+        </is>
+      </c>
+      <c r="E744" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F744" s="5" t="n"/>
+    </row>
+    <row r="745" ht="20.25" customHeight="1">
+      <c r="A745" s="5" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B745" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C745" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D745" s="6" t="inlineStr">
+        <is>
+          <t>125865</t>
+        </is>
+      </c>
+      <c r="E745" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F745" s="5" t="n"/>
+    </row>
+    <row r="746" ht="20.25" customHeight="1">
+      <c r="A746" s="5" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B746" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C746" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D746" s="6" t="inlineStr">
+        <is>
+          <t>125831</t>
+        </is>
+      </c>
+      <c r="E746" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F746" s="5" t="n"/>
+    </row>
+    <row r="747" ht="20.25" customHeight="1">
+      <c r="A747" s="5" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B747" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C747" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D747" s="6" t="inlineStr">
+        <is>
+          <t>280760</t>
+        </is>
+      </c>
+      <c r="E747" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F747" s="5" t="n"/>
+    </row>
+    <row r="748" ht="20.25" customHeight="1">
+      <c r="A748" s="5" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B748" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C748" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D748" s="6" t="inlineStr">
+        <is>
+          <t>280614</t>
+        </is>
+      </c>
+      <c r="E748" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F748" s="5" t="n"/>
+    </row>
+    <row r="749" ht="20.25" customHeight="1">
+      <c r="A749" s="5" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B749" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C749" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D749" s="6" t="inlineStr">
+        <is>
+          <t>280612</t>
+        </is>
+      </c>
+      <c r="E749" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F749" s="5" t="n"/>
+    </row>
+    <row r="750" ht="20.25" customHeight="1">
+      <c r="A750" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B750" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C750" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D750" s="6" t="inlineStr">
+        <is>
+          <t>280759</t>
+        </is>
+      </c>
+      <c r="E750" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F750" s="5" t="n"/>
+    </row>
+    <row r="751" ht="20.25" customHeight="1">
+      <c r="A751" s="5" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B751" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C751" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D751" s="6" t="inlineStr">
+        <is>
+          <t>280615</t>
+        </is>
+      </c>
+      <c r="E751" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F751" s="5" t="n"/>
+    </row>
+    <row r="752" ht="20.25" customHeight="1">
+      <c r="A752" s="5" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B752" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C752" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D752" s="6" t="inlineStr">
+        <is>
+          <t>280620</t>
+        </is>
+      </c>
+      <c r="E752" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F752" s="5" t="n"/>
+    </row>
+    <row r="753" ht="20.25" customHeight="1">
+      <c r="A753" s="5" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B753" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C753" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D753" s="6" t="inlineStr">
+        <is>
+          <t>280611</t>
+        </is>
+      </c>
+      <c r="E753" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F753" s="5" t="n"/>
+    </row>
+    <row r="754" ht="20.25" customHeight="1">
+      <c r="A754" s="5" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B754" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C754" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D754" s="6" t="inlineStr">
+        <is>
+          <t>280412</t>
+        </is>
+      </c>
+      <c r="E754" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F754" s="5" t="n"/>
+    </row>
+    <row r="755" ht="20.25" customHeight="1">
+      <c r="A755" s="5" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B755" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C755" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D755" s="6" t="inlineStr">
+        <is>
+          <t>280299</t>
+        </is>
+      </c>
+      <c r="E755" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F755" s="5" t="n"/>
+    </row>
+    <row r="756" ht="20.25" customHeight="1">
+      <c r="A756" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B756" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C756" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D756" s="6" t="inlineStr">
+        <is>
+          <t>280300</t>
+        </is>
+      </c>
+      <c r="E756" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F756" s="5" t="n"/>
+    </row>
+    <row r="757" ht="22" customHeight="1">
+      <c r="A757" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (752 BAL)</t>
+        </is>
+      </c>
+      <c r="B757" s="4" t="n"/>
+      <c r="C757" s="4" t="n"/>
+      <c r="D757" s="4" t="n"/>
+      <c r="E757" s="4">
+        <f>SUM(E5:E756)</f>
         <v/>
       </c>
-      <c r="F729" s="4" t="inlineStr">
+      <c r="F757" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -15096,12 +15656,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A729:D729"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A757:D757"/>
     <mergeCell ref="B3:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15114,7 +15674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I729"/>
+  <dimension ref="A1:I757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15138,7 +15698,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 724 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 752 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -41977,23 +42537,1059 @@
         </is>
       </c>
     </row>
-    <row r="729">
-      <c r="A729" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (724 BAL)</t>
-        </is>
-      </c>
-      <c r="B729" s="4" t="n"/>
-      <c r="C729" s="4" t="n"/>
-      <c r="D729" s="4" t="n"/>
-      <c r="E729" s="4" t="n"/>
-      <c r="F729" s="4" t="n"/>
-      <c r="G729" s="4" t="n"/>
-      <c r="H729" s="4">
-        <f>SUM(H5:H728)</f>
+    <row r="729" ht="20" customHeight="1">
+      <c r="A729" s="9" t="n">
+        <v>725</v>
+      </c>
+      <c r="B729" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C729" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D729" s="9" t="n">
+        <v>991</v>
+      </c>
+      <c r="E729" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F729" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G729" s="10" t="inlineStr">
+        <is>
+          <t>280619</t>
+        </is>
+      </c>
+      <c r="H729" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I729" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="730" ht="20" customHeight="1">
+      <c r="A730" s="9" t="n">
+        <v>726</v>
+      </c>
+      <c r="B730" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C730" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D730" s="9" t="n">
+        <v>992</v>
+      </c>
+      <c r="E730" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F730" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G730" s="10" t="inlineStr">
+        <is>
+          <t>280763</t>
+        </is>
+      </c>
+      <c r="H730" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I730" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="731" ht="20" customHeight="1">
+      <c r="A731" s="9" t="n">
+        <v>727</v>
+      </c>
+      <c r="B731" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C731" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D731" s="9" t="n">
+        <v>993</v>
+      </c>
+      <c r="E731" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F731" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G731" s="10" t="inlineStr">
+        <is>
+          <t>280618</t>
+        </is>
+      </c>
+      <c r="H731" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I731" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="732" ht="20" customHeight="1">
+      <c r="A732" s="9" t="n">
+        <v>728</v>
+      </c>
+      <c r="B732" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C732" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D732" s="9" t="n">
+        <v>994</v>
+      </c>
+      <c r="E732" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F732" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G732" s="10" t="inlineStr">
+        <is>
+          <t>280762</t>
+        </is>
+      </c>
+      <c r="H732" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I732" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="733" ht="20" customHeight="1">
+      <c r="A733" s="9" t="n">
+        <v>729</v>
+      </c>
+      <c r="B733" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C733" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D733" s="9" t="n">
+        <v>995</v>
+      </c>
+      <c r="E733" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F733" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G733" s="10" t="inlineStr">
+        <is>
+          <t>39844</t>
+        </is>
+      </c>
+      <c r="H733" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I733" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="734" ht="20" customHeight="1">
+      <c r="A734" s="9" t="n">
+        <v>730</v>
+      </c>
+      <c r="B734" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C734" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D734" s="9" t="n">
+        <v>996</v>
+      </c>
+      <c r="E734" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F734" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G734" s="10" t="inlineStr">
+        <is>
+          <t>39843</t>
+        </is>
+      </c>
+      <c r="H734" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I734" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="735" ht="20" customHeight="1">
+      <c r="A735" s="9" t="n">
+        <v>731</v>
+      </c>
+      <c r="B735" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C735" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D735" s="9" t="n">
+        <v>997</v>
+      </c>
+      <c r="E735" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F735" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G735" s="10" t="inlineStr">
+        <is>
+          <t>280617</t>
+        </is>
+      </c>
+      <c r="H735" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I735" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="736" ht="20" customHeight="1">
+      <c r="A736" s="9" t="n">
+        <v>732</v>
+      </c>
+      <c r="B736" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C736" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D736" s="9" t="n">
+        <v>998</v>
+      </c>
+      <c r="E736" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F736" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G736" s="10" t="inlineStr">
+        <is>
+          <t>280761</t>
+        </is>
+      </c>
+      <c r="H736" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I736" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="737" ht="20" customHeight="1">
+      <c r="A737" s="9" t="n">
+        <v>733</v>
+      </c>
+      <c r="B737" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C737" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D737" s="9" t="n">
+        <v>999</v>
+      </c>
+      <c r="E737" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F737" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G737" s="10" t="inlineStr">
+        <is>
+          <t>280616</t>
+        </is>
+      </c>
+      <c r="H737" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I737" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="738" ht="20" customHeight="1">
+      <c r="A738" s="9" t="n">
+        <v>734</v>
+      </c>
+      <c r="B738" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C738" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D738" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E738" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F738" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G738" s="10" t="inlineStr">
+        <is>
+          <t>125833</t>
+        </is>
+      </c>
+      <c r="H738" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I738" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="739" ht="20" customHeight="1">
+      <c r="A739" s="9" t="n">
+        <v>735</v>
+      </c>
+      <c r="B739" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C739" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D739" s="9" t="n">
+        <v>1001</v>
+      </c>
+      <c r="E739" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F739" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G739" s="10" t="inlineStr">
+        <is>
+          <t>280613</t>
+        </is>
+      </c>
+      <c r="H739" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I739" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="740" ht="20" customHeight="1">
+      <c r="A740" s="9" t="n">
+        <v>736</v>
+      </c>
+      <c r="B740" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C740" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D740" s="9" t="n">
+        <v>1003</v>
+      </c>
+      <c r="E740" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F740" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G740" s="10" t="inlineStr">
+        <is>
+          <t>125832</t>
+        </is>
+      </c>
+      <c r="H740" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I740" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="741" ht="20" customHeight="1">
+      <c r="A741" s="9" t="n">
+        <v>737</v>
+      </c>
+      <c r="B741" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C741" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D741" s="9" t="n">
+        <v>1004</v>
+      </c>
+      <c r="E741" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F741" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G741" s="10" t="inlineStr">
+        <is>
+          <t>125862</t>
+        </is>
+      </c>
+      <c r="H741" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I741" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="742" ht="20" customHeight="1">
+      <c r="A742" s="9" t="n">
+        <v>738</v>
+      </c>
+      <c r="B742" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C742" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D742" s="9" t="n">
+        <v>1005</v>
+      </c>
+      <c r="E742" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F742" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G742" s="10" t="inlineStr">
+        <is>
+          <t>125866</t>
+        </is>
+      </c>
+      <c r="H742" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I742" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="743" ht="20" customHeight="1">
+      <c r="A743" s="9" t="n">
+        <v>739</v>
+      </c>
+      <c r="B743" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C743" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D743" s="9" t="n">
+        <v>1006</v>
+      </c>
+      <c r="E743" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F743" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G743" s="10" t="inlineStr">
+        <is>
+          <t>125863</t>
+        </is>
+      </c>
+      <c r="H743" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I743" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="744" ht="20" customHeight="1">
+      <c r="A744" s="9" t="n">
+        <v>740</v>
+      </c>
+      <c r="B744" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C744" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D744" s="9" t="n">
+        <v>1007</v>
+      </c>
+      <c r="E744" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F744" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G744" s="10" t="inlineStr">
+        <is>
+          <t>125864</t>
+        </is>
+      </c>
+      <c r="H744" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I744" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="745" ht="20" customHeight="1">
+      <c r="A745" s="9" t="n">
+        <v>741</v>
+      </c>
+      <c r="B745" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C745" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D745" s="9" t="n">
+        <v>1008</v>
+      </c>
+      <c r="E745" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F745" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G745" s="10" t="inlineStr">
+        <is>
+          <t>125865</t>
+        </is>
+      </c>
+      <c r="H745" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I745" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="746" ht="20" customHeight="1">
+      <c r="A746" s="9" t="n">
+        <v>742</v>
+      </c>
+      <c r="B746" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C746" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D746" s="9" t="n">
+        <v>1009</v>
+      </c>
+      <c r="E746" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F746" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G746" s="10" t="inlineStr">
+        <is>
+          <t>125831</t>
+        </is>
+      </c>
+      <c r="H746" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I746" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="747" ht="20" customHeight="1">
+      <c r="A747" s="9" t="n">
+        <v>743</v>
+      </c>
+      <c r="B747" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C747" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D747" s="9" t="n">
+        <v>1010</v>
+      </c>
+      <c r="E747" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F747" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G747" s="10" t="inlineStr">
+        <is>
+          <t>280760</t>
+        </is>
+      </c>
+      <c r="H747" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I747" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="748" ht="20" customHeight="1">
+      <c r="A748" s="9" t="n">
+        <v>744</v>
+      </c>
+      <c r="B748" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C748" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D748" s="9" t="n">
+        <v>1011</v>
+      </c>
+      <c r="E748" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F748" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G748" s="10" t="inlineStr">
+        <is>
+          <t>280614</t>
+        </is>
+      </c>
+      <c r="H748" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I748" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="749" ht="20" customHeight="1">
+      <c r="A749" s="9" t="n">
+        <v>745</v>
+      </c>
+      <c r="B749" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C749" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D749" s="9" t="n">
+        <v>1012</v>
+      </c>
+      <c r="E749" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F749" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G749" s="10" t="inlineStr">
+        <is>
+          <t>280612</t>
+        </is>
+      </c>
+      <c r="H749" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I749" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="750" ht="20" customHeight="1">
+      <c r="A750" s="9" t="n">
+        <v>746</v>
+      </c>
+      <c r="B750" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C750" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D750" s="9" t="n">
+        <v>1013</v>
+      </c>
+      <c r="E750" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F750" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G750" s="10" t="inlineStr">
+        <is>
+          <t>280759</t>
+        </is>
+      </c>
+      <c r="H750" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I750" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="751" ht="20" customHeight="1">
+      <c r="A751" s="9" t="n">
+        <v>747</v>
+      </c>
+      <c r="B751" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C751" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D751" s="9" t="n">
+        <v>1014</v>
+      </c>
+      <c r="E751" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F751" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G751" s="10" t="inlineStr">
+        <is>
+          <t>280615</t>
+        </is>
+      </c>
+      <c r="H751" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I751" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="752" ht="20" customHeight="1">
+      <c r="A752" s="9" t="n">
+        <v>748</v>
+      </c>
+      <c r="B752" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C752" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D752" s="9" t="n">
+        <v>1015</v>
+      </c>
+      <c r="E752" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F752" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G752" s="10" t="inlineStr">
+        <is>
+          <t>280620</t>
+        </is>
+      </c>
+      <c r="H752" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I752" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="753" ht="20" customHeight="1">
+      <c r="A753" s="9" t="n">
+        <v>749</v>
+      </c>
+      <c r="B753" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C753" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D753" s="9" t="n">
+        <v>1016</v>
+      </c>
+      <c r="E753" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F753" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G753" s="10" t="inlineStr">
+        <is>
+          <t>280611</t>
+        </is>
+      </c>
+      <c r="H753" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I753" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="754" ht="20" customHeight="1">
+      <c r="A754" s="9" t="n">
+        <v>750</v>
+      </c>
+      <c r="B754" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C754" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D754" s="9" t="n">
+        <v>1017</v>
+      </c>
+      <c r="E754" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F754" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G754" s="10" t="inlineStr">
+        <is>
+          <t>280412</t>
+        </is>
+      </c>
+      <c r="H754" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I754" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="755" ht="20" customHeight="1">
+      <c r="A755" s="9" t="n">
+        <v>751</v>
+      </c>
+      <c r="B755" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C755" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D755" s="9" t="n">
+        <v>1018</v>
+      </c>
+      <c r="E755" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F755" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G755" s="10" t="inlineStr">
+        <is>
+          <t>280299</t>
+        </is>
+      </c>
+      <c r="H755" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I755" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="756" ht="20" customHeight="1">
+      <c r="A756" s="9" t="n">
+        <v>752</v>
+      </c>
+      <c r="B756" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C756" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D756" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="E756" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F756" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G756" s="10" t="inlineStr">
+        <is>
+          <t>280300</t>
+        </is>
+      </c>
+      <c r="H756" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I756" s="11" t="inlineStr">
+        <is>
+          <t>grade 13 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (752 BAL)</t>
+        </is>
+      </c>
+      <c r="B757" s="4" t="n"/>
+      <c r="C757" s="4" t="n"/>
+      <c r="D757" s="4" t="n"/>
+      <c r="E757" s="4" t="n"/>
+      <c r="F757" s="4" t="n"/>
+      <c r="G757" s="4" t="n"/>
+      <c r="H757" s="4">
+        <f>SUM(H5:H756)</f>
         <v/>
       </c>
-      <c r="I729" s="4" t="inlineStr">
+      <c r="I757" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -42002,8 +43598,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A729:G729"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A757:G757"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -42015,7 +43611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -42716,35 +44312,64 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>1066</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>38.07</v>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>991 - 1019</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4">
-        <f>SUM(D5:D26)</f>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4">
+        <f>SUM(D5:D27)</f>
         <v/>
       </c>
-      <c r="E27" s="4">
-        <f>SUM(E5:E26)</f>
+      <c r="E28" s="4">
+        <f>SUM(E5:E27)</f>
         <v/>
       </c>
-      <c r="F27" s="4">
-        <f>AVERAGE(F5:F26)</f>
+      <c r="F28" s="4">
+        <f>AVERAGE(F5:F27)</f>
         <v/>
       </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>3 - 987</t>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>3 - 1019</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: tambah data bal tembakau tanggal 14 September 2026 (No Gud 1020-1046) dan sinkronisasi realtime
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F757"/>
+  <dimension ref="A1:F784"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15634,20 +15634,560 @@
       </c>
       <c r="F756" s="5" t="n"/>
     </row>
-    <row r="757" ht="22" customHeight="1">
-      <c r="A757" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (752 BAL)</t>
-        </is>
-      </c>
-      <c r="B757" s="4" t="n"/>
-      <c r="C757" s="4" t="n"/>
-      <c r="D757" s="4" t="n"/>
-      <c r="E757" s="4">
-        <f>SUM(E5:E756)</f>
+    <row r="757" ht="20.25" customHeight="1">
+      <c r="A757" s="5" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B757" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C757" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D757" s="6" t="inlineStr">
+        <is>
+          <t>282168</t>
+        </is>
+      </c>
+      <c r="E757" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F757" s="5" t="n"/>
+    </row>
+    <row r="758" ht="20.25" customHeight="1">
+      <c r="A758" s="5" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B758" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C758" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D758" s="6" t="inlineStr">
+        <is>
+          <t>282096</t>
+        </is>
+      </c>
+      <c r="E758" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F758" s="5" t="n"/>
+    </row>
+    <row r="759" ht="20.25" customHeight="1">
+      <c r="A759" s="5" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B759" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C759" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D759" s="6" t="inlineStr">
+        <is>
+          <t>282097</t>
+        </is>
+      </c>
+      <c r="E759" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F759" s="5" t="n"/>
+    </row>
+    <row r="760" ht="20.25" customHeight="1">
+      <c r="A760" s="5" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B760" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C760" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D760" s="6" t="inlineStr">
+        <is>
+          <t>282098</t>
+        </is>
+      </c>
+      <c r="E760" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F760" s="5" t="n"/>
+    </row>
+    <row r="761" ht="20.25" customHeight="1">
+      <c r="A761" s="5" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B761" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C761" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D761" s="6" t="inlineStr">
+        <is>
+          <t>282171</t>
+        </is>
+      </c>
+      <c r="E761" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F761" s="5" t="n"/>
+    </row>
+    <row r="762" ht="20.25" customHeight="1">
+      <c r="A762" s="5" t="n">
+        <v>1025</v>
+      </c>
+      <c r="B762" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C762" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D762" s="6" t="inlineStr">
+        <is>
+          <t>282174</t>
+        </is>
+      </c>
+      <c r="E762" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F762" s="5" t="n"/>
+    </row>
+    <row r="763" ht="20.25" customHeight="1">
+      <c r="A763" s="5" t="n">
+        <v>1026</v>
+      </c>
+      <c r="B763" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C763" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D763" s="6" t="inlineStr">
+        <is>
+          <t>282173</t>
+        </is>
+      </c>
+      <c r="E763" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F763" s="5" t="n"/>
+    </row>
+    <row r="764" ht="20.25" customHeight="1">
+      <c r="A764" s="5" t="n">
+        <v>1027</v>
+      </c>
+      <c r="B764" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C764" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D764" s="6" t="inlineStr">
+        <is>
+          <t>282176</t>
+        </is>
+      </c>
+      <c r="E764" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F764" s="5" t="n"/>
+    </row>
+    <row r="765" ht="20.25" customHeight="1">
+      <c r="A765" s="5" t="n">
+        <v>1028</v>
+      </c>
+      <c r="B765" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C765" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D765" s="6" t="inlineStr">
+        <is>
+          <t>282169</t>
+        </is>
+      </c>
+      <c r="E765" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F765" s="5" t="n"/>
+    </row>
+    <row r="766" ht="20.25" customHeight="1">
+      <c r="A766" s="5" t="n">
+        <v>1029</v>
+      </c>
+      <c r="B766" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C766" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D766" s="6" t="inlineStr">
+        <is>
+          <t>282170</t>
+        </is>
+      </c>
+      <c r="E766" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F766" s="5" t="n"/>
+    </row>
+    <row r="767" ht="20.25" customHeight="1">
+      <c r="A767" s="5" t="n">
+        <v>1030</v>
+      </c>
+      <c r="B767" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C767" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D767" s="6" t="inlineStr">
+        <is>
+          <t>282175</t>
+        </is>
+      </c>
+      <c r="E767" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F767" s="5" t="n"/>
+    </row>
+    <row r="768" ht="20.25" customHeight="1">
+      <c r="A768" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="B768" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C768" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D768" s="6" t="inlineStr">
+        <is>
+          <t>282252</t>
+        </is>
+      </c>
+      <c r="E768" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F768" s="5" t="n"/>
+    </row>
+    <row r="769" ht="20.25" customHeight="1">
+      <c r="A769" s="5" t="n">
+        <v>1032</v>
+      </c>
+      <c r="B769" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C769" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D769" s="6" t="inlineStr">
+        <is>
+          <t>282228</t>
+        </is>
+      </c>
+      <c r="E769" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F769" s="5" t="n"/>
+    </row>
+    <row r="770" ht="20.25" customHeight="1">
+      <c r="A770" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="B770" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C770" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D770" s="6" t="inlineStr">
+        <is>
+          <t>282099</t>
+        </is>
+      </c>
+      <c r="E770" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F770" s="5" t="n"/>
+    </row>
+    <row r="771" ht="20.25" customHeight="1">
+      <c r="A771" s="5" t="n">
+        <v>1034</v>
+      </c>
+      <c r="B771" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C771" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D771" s="6" t="inlineStr">
+        <is>
+          <t>282251</t>
+        </is>
+      </c>
+      <c r="E771" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F771" s="5" t="n"/>
+    </row>
+    <row r="772" ht="20.25" customHeight="1">
+      <c r="A772" s="5" t="n">
+        <v>1035</v>
+      </c>
+      <c r="B772" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C772" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D772" s="6" t="inlineStr">
+        <is>
+          <t>282100</t>
+        </is>
+      </c>
+      <c r="E772" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F772" s="5" t="n"/>
+    </row>
+    <row r="773" ht="20.25" customHeight="1">
+      <c r="A773" s="5" t="n">
+        <v>1036</v>
+      </c>
+      <c r="B773" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C773" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="D773" s="6" t="inlineStr">
+        <is>
+          <t>280315</t>
+        </is>
+      </c>
+      <c r="E773" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F773" s="5" t="n"/>
+    </row>
+    <row r="774" ht="20.25" customHeight="1">
+      <c r="A774" s="5" t="n">
+        <v>1037</v>
+      </c>
+      <c r="B774" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C774" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="D774" s="6" t="inlineStr">
+        <is>
+          <t>280314</t>
+        </is>
+      </c>
+      <c r="E774" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F774" s="5" t="n"/>
+    </row>
+    <row r="775" ht="20.25" customHeight="1">
+      <c r="A775" s="5" t="n">
+        <v>1038</v>
+      </c>
+      <c r="B775" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C775" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D775" s="6" t="inlineStr">
+        <is>
+          <t>282172</t>
+        </is>
+      </c>
+      <c r="E775" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F775" s="5" t="n"/>
+    </row>
+    <row r="776" ht="20.25" customHeight="1">
+      <c r="A776" s="5" t="n">
+        <v>1039</v>
+      </c>
+      <c r="B776" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C776" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D776" s="6" t="inlineStr">
+        <is>
+          <t>282229</t>
+        </is>
+      </c>
+      <c r="E776" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F776" s="5" t="n"/>
+    </row>
+    <row r="777" ht="20.25" customHeight="1">
+      <c r="A777" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="B777" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C777" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D777" s="6" t="inlineStr">
+        <is>
+          <t>282253</t>
+        </is>
+      </c>
+      <c r="E777" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F777" s="5" t="n"/>
+    </row>
+    <row r="778" ht="20.25" customHeight="1">
+      <c r="A778" s="5" t="n">
+        <v>1041</v>
+      </c>
+      <c r="B778" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C778" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D778" s="6" t="inlineStr">
+        <is>
+          <t>282230</t>
+        </is>
+      </c>
+      <c r="E778" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F778" s="5" t="n"/>
+    </row>
+    <row r="779" ht="20.25" customHeight="1">
+      <c r="A779" s="5" t="n">
+        <v>1042</v>
+      </c>
+      <c r="B779" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C779" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D779" s="6" t="inlineStr">
+        <is>
+          <t>282231</t>
+        </is>
+      </c>
+      <c r="E779" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F779" s="5" t="n"/>
+    </row>
+    <row r="780" ht="20.25" customHeight="1">
+      <c r="A780" s="5" t="n">
+        <v>1043</v>
+      </c>
+      <c r="B780" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C780" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D780" s="6" t="inlineStr">
+        <is>
+          <t>282167</t>
+        </is>
+      </c>
+      <c r="E780" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F780" s="5" t="n"/>
+    </row>
+    <row r="781" ht="20.25" customHeight="1">
+      <c r="A781" s="5" t="n">
+        <v>1044</v>
+      </c>
+      <c r="B781" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C781" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D781" s="6" t="inlineStr">
+        <is>
+          <t>282166</t>
+        </is>
+      </c>
+      <c r="E781" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F781" s="5" t="n"/>
+    </row>
+    <row r="782" ht="20.25" customHeight="1">
+      <c r="A782" s="5" t="n">
+        <v>1045</v>
+      </c>
+      <c r="B782" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C782" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D782" s="6" t="inlineStr">
+        <is>
+          <t>282416</t>
+        </is>
+      </c>
+      <c r="E782" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F782" s="5" t="n"/>
+    </row>
+    <row r="783" ht="20.25" customHeight="1">
+      <c r="A783" s="5" t="n">
+        <v>1046</v>
+      </c>
+      <c r="B783" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C783" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D783" s="6" t="inlineStr">
+        <is>
+          <t>282095</t>
+        </is>
+      </c>
+      <c r="E783" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F783" s="5" t="n"/>
+    </row>
+    <row r="784" ht="22" customHeight="1">
+      <c r="A784" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (779 BAL)</t>
+        </is>
+      </c>
+      <c r="B784" s="4" t="n"/>
+      <c r="C784" s="4" t="n"/>
+      <c r="D784" s="4" t="n"/>
+      <c r="E784" s="4">
+        <f>SUM(E5:E783)</f>
         <v/>
       </c>
-      <c r="F757" s="4" t="inlineStr">
+      <c r="F784" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -15661,7 +16201,7 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A757:D757"/>
+    <mergeCell ref="A784:D784"/>
     <mergeCell ref="B3:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15674,7 +16214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I757"/>
+  <dimension ref="A1:I784"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15698,7 +16238,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 752 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 779 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -43573,23 +44113,1022 @@
         </is>
       </c>
     </row>
-    <row r="757">
-      <c r="A757" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (752 BAL)</t>
-        </is>
-      </c>
-      <c r="B757" s="4" t="n"/>
-      <c r="C757" s="4" t="n"/>
-      <c r="D757" s="4" t="n"/>
-      <c r="E757" s="4" t="n"/>
-      <c r="F757" s="4" t="n"/>
-      <c r="G757" s="4" t="n"/>
-      <c r="H757" s="4">
-        <f>SUM(H5:H756)</f>
+    <row r="757" ht="20" customHeight="1">
+      <c r="A757" s="9" t="n">
+        <v>753</v>
+      </c>
+      <c r="B757" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C757" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D757" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="E757" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F757" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G757" s="10" t="inlineStr">
+        <is>
+          <t>282168</t>
+        </is>
+      </c>
+      <c r="H757" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I757" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="758" ht="20" customHeight="1">
+      <c r="A758" s="9" t="n">
+        <v>754</v>
+      </c>
+      <c r="B758" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C758" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D758" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="E758" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F758" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G758" s="10" t="inlineStr">
+        <is>
+          <t>282096</t>
+        </is>
+      </c>
+      <c r="H758" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I758" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="759" ht="20" customHeight="1">
+      <c r="A759" s="9" t="n">
+        <v>755</v>
+      </c>
+      <c r="B759" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C759" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D759" s="9" t="n">
+        <v>1022</v>
+      </c>
+      <c r="E759" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F759" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G759" s="10" t="inlineStr">
+        <is>
+          <t>282097</t>
+        </is>
+      </c>
+      <c r="H759" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I759" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="760" ht="20" customHeight="1">
+      <c r="A760" s="9" t="n">
+        <v>756</v>
+      </c>
+      <c r="B760" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C760" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D760" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="E760" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F760" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G760" s="10" t="inlineStr">
+        <is>
+          <t>282098</t>
+        </is>
+      </c>
+      <c r="H760" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I760" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="761" ht="20" customHeight="1">
+      <c r="A761" s="9" t="n">
+        <v>757</v>
+      </c>
+      <c r="B761" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C761" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D761" s="9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E761" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F761" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G761" s="10" t="inlineStr">
+        <is>
+          <t>282171</t>
+        </is>
+      </c>
+      <c r="H761" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I761" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="762" ht="20" customHeight="1">
+      <c r="A762" s="9" t="n">
+        <v>758</v>
+      </c>
+      <c r="B762" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C762" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D762" s="9" t="n">
+        <v>1025</v>
+      </c>
+      <c r="E762" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F762" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G762" s="10" t="inlineStr">
+        <is>
+          <t>282174</t>
+        </is>
+      </c>
+      <c r="H762" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I762" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="763" ht="20" customHeight="1">
+      <c r="A763" s="9" t="n">
+        <v>759</v>
+      </c>
+      <c r="B763" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C763" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D763" s="9" t="n">
+        <v>1026</v>
+      </c>
+      <c r="E763" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F763" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G763" s="10" t="inlineStr">
+        <is>
+          <t>282173</t>
+        </is>
+      </c>
+      <c r="H763" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I763" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="764" ht="20" customHeight="1">
+      <c r="A764" s="9" t="n">
+        <v>760</v>
+      </c>
+      <c r="B764" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C764" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D764" s="9" t="n">
+        <v>1027</v>
+      </c>
+      <c r="E764" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F764" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G764" s="10" t="inlineStr">
+        <is>
+          <t>282176</t>
+        </is>
+      </c>
+      <c r="H764" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I764" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="765" ht="20" customHeight="1">
+      <c r="A765" s="9" t="n">
+        <v>761</v>
+      </c>
+      <c r="B765" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C765" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D765" s="9" t="n">
+        <v>1028</v>
+      </c>
+      <c r="E765" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F765" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G765" s="10" t="inlineStr">
+        <is>
+          <t>282169</t>
+        </is>
+      </c>
+      <c r="H765" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I765" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="766" ht="20" customHeight="1">
+      <c r="A766" s="9" t="n">
+        <v>762</v>
+      </c>
+      <c r="B766" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C766" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D766" s="9" t="n">
+        <v>1029</v>
+      </c>
+      <c r="E766" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F766" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G766" s="10" t="inlineStr">
+        <is>
+          <t>282170</t>
+        </is>
+      </c>
+      <c r="H766" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I766" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="767" ht="20" customHeight="1">
+      <c r="A767" s="9" t="n">
+        <v>763</v>
+      </c>
+      <c r="B767" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C767" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D767" s="9" t="n">
+        <v>1030</v>
+      </c>
+      <c r="E767" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F767" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G767" s="10" t="inlineStr">
+        <is>
+          <t>282175</t>
+        </is>
+      </c>
+      <c r="H767" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I767" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="768" ht="20" customHeight="1">
+      <c r="A768" s="9" t="n">
+        <v>764</v>
+      </c>
+      <c r="B768" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C768" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D768" s="9" t="n">
+        <v>1031</v>
+      </c>
+      <c r="E768" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F768" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G768" s="10" t="inlineStr">
+        <is>
+          <t>282252</t>
+        </is>
+      </c>
+      <c r="H768" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I768" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="769" ht="20" customHeight="1">
+      <c r="A769" s="9" t="n">
+        <v>765</v>
+      </c>
+      <c r="B769" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C769" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D769" s="9" t="n">
+        <v>1032</v>
+      </c>
+      <c r="E769" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F769" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G769" s="10" t="inlineStr">
+        <is>
+          <t>282228</t>
+        </is>
+      </c>
+      <c r="H769" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I769" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="770" ht="20" customHeight="1">
+      <c r="A770" s="9" t="n">
+        <v>766</v>
+      </c>
+      <c r="B770" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C770" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D770" s="9" t="n">
+        <v>1033</v>
+      </c>
+      <c r="E770" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F770" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G770" s="10" t="inlineStr">
+        <is>
+          <t>282099</t>
+        </is>
+      </c>
+      <c r="H770" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I770" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="771" ht="20" customHeight="1">
+      <c r="A771" s="9" t="n">
+        <v>767</v>
+      </c>
+      <c r="B771" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C771" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D771" s="9" t="n">
+        <v>1034</v>
+      </c>
+      <c r="E771" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F771" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G771" s="10" t="inlineStr">
+        <is>
+          <t>282251</t>
+        </is>
+      </c>
+      <c r="H771" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I771" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="772" ht="20" customHeight="1">
+      <c r="A772" s="9" t="n">
+        <v>768</v>
+      </c>
+      <c r="B772" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C772" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D772" s="9" t="n">
+        <v>1035</v>
+      </c>
+      <c r="E772" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F772" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G772" s="10" t="inlineStr">
+        <is>
+          <t>282100</t>
+        </is>
+      </c>
+      <c r="H772" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I772" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="773" ht="20" customHeight="1">
+      <c r="A773" s="9" t="n">
+        <v>769</v>
+      </c>
+      <c r="B773" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C773" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D773" s="9" t="n">
+        <v>1036</v>
+      </c>
+      <c r="E773" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F773" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="G773" s="10" t="inlineStr">
+        <is>
+          <t>280315</t>
+        </is>
+      </c>
+      <c r="H773" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I773" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="774" ht="20" customHeight="1">
+      <c r="A774" s="9" t="n">
+        <v>770</v>
+      </c>
+      <c r="B774" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C774" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D774" s="9" t="n">
+        <v>1037</v>
+      </c>
+      <c r="E774" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F774" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="G774" s="10" t="inlineStr">
+        <is>
+          <t>280314</t>
+        </is>
+      </c>
+      <c r="H774" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I774" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="775" ht="20" customHeight="1">
+      <c r="A775" s="9" t="n">
+        <v>771</v>
+      </c>
+      <c r="B775" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C775" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D775" s="9" t="n">
+        <v>1038</v>
+      </c>
+      <c r="E775" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F775" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G775" s="10" t="inlineStr">
+        <is>
+          <t>282172</t>
+        </is>
+      </c>
+      <c r="H775" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I775" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="776" ht="20" customHeight="1">
+      <c r="A776" s="9" t="n">
+        <v>772</v>
+      </c>
+      <c r="B776" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C776" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D776" s="9" t="n">
+        <v>1039</v>
+      </c>
+      <c r="E776" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F776" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G776" s="10" t="inlineStr">
+        <is>
+          <t>282229</t>
+        </is>
+      </c>
+      <c r="H776" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I776" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="777" ht="20" customHeight="1">
+      <c r="A777" s="9" t="n">
+        <v>773</v>
+      </c>
+      <c r="B777" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C777" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D777" s="9" t="n">
+        <v>1040</v>
+      </c>
+      <c r="E777" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F777" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G777" s="10" t="inlineStr">
+        <is>
+          <t>282253</t>
+        </is>
+      </c>
+      <c r="H777" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I777" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="778" ht="20" customHeight="1">
+      <c r="A778" s="9" t="n">
+        <v>774</v>
+      </c>
+      <c r="B778" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C778" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D778" s="9" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E778" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F778" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G778" s="10" t="inlineStr">
+        <is>
+          <t>282230</t>
+        </is>
+      </c>
+      <c r="H778" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I778" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="779" ht="20" customHeight="1">
+      <c r="A779" s="9" t="n">
+        <v>775</v>
+      </c>
+      <c r="B779" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C779" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D779" s="9" t="n">
+        <v>1042</v>
+      </c>
+      <c r="E779" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F779" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G779" s="10" t="inlineStr">
+        <is>
+          <t>282231</t>
+        </is>
+      </c>
+      <c r="H779" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I779" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="780" ht="20" customHeight="1">
+      <c r="A780" s="9" t="n">
+        <v>776</v>
+      </c>
+      <c r="B780" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C780" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D780" s="9" t="n">
+        <v>1043</v>
+      </c>
+      <c r="E780" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F780" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G780" s="10" t="inlineStr">
+        <is>
+          <t>282167</t>
+        </is>
+      </c>
+      <c r="H780" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I780" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="781" ht="20" customHeight="1">
+      <c r="A781" s="9" t="n">
+        <v>777</v>
+      </c>
+      <c r="B781" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C781" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D781" s="9" t="n">
+        <v>1044</v>
+      </c>
+      <c r="E781" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F781" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G781" s="10" t="inlineStr">
+        <is>
+          <t>282166</t>
+        </is>
+      </c>
+      <c r="H781" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I781" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="782" ht="20" customHeight="1">
+      <c r="A782" s="9" t="n">
+        <v>778</v>
+      </c>
+      <c r="B782" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C782" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D782" s="9" t="n">
+        <v>1045</v>
+      </c>
+      <c r="E782" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F782" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G782" s="10" t="inlineStr">
+        <is>
+          <t>282416</t>
+        </is>
+      </c>
+      <c r="H782" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I782" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="783" ht="20" customHeight="1">
+      <c r="A783" s="9" t="n">
+        <v>779</v>
+      </c>
+      <c r="B783" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C783" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D783" s="9" t="n">
+        <v>1046</v>
+      </c>
+      <c r="E783" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F783" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G783" s="10" t="inlineStr">
+        <is>
+          <t>282095</t>
+        </is>
+      </c>
+      <c r="H783" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I783" s="11" t="inlineStr">
+        <is>
+          <t>grade 14 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (779 BAL)</t>
+        </is>
+      </c>
+      <c r="B784" s="4" t="n"/>
+      <c r="C784" s="4" t="n"/>
+      <c r="D784" s="4" t="n"/>
+      <c r="E784" s="4" t="n"/>
+      <c r="F784" s="4" t="n"/>
+      <c r="G784" s="4" t="n"/>
+      <c r="H784" s="4">
+        <f>SUM(H5:H783)</f>
         <v/>
       </c>
-      <c r="I757" s="4" t="inlineStr">
+      <c r="I784" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -43598,8 +45137,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A784:G784"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A757:G757"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -43611,7 +45150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -44341,35 +45880,64 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>1103</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>40.85</v>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>1020 - 1046</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4">
-        <f>SUM(D5:D27)</f>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4">
+        <f>SUM(D5:D28)</f>
         <v/>
       </c>
-      <c r="E28" s="4">
-        <f>SUM(E5:E27)</f>
+      <c r="E29" s="4">
+        <f>SUM(E5:E28)</f>
         <v/>
       </c>
-      <c r="F28" s="4">
-        <f>AVERAGE(F5:F27)</f>
+      <c r="F29" s="4">
+        <f>AVERAGE(F5:F28)</f>
         <v/>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>3 - 1019</t>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>3 - 1046</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: tambah data bal tembakau tanggal 17 September 2026 (71 bal, No Gud 1047-1154) dan sinkronisasi realtime
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F784"/>
+  <dimension ref="A1:F855"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16174,20 +16174,1440 @@
       </c>
       <c r="F783" s="5" t="n"/>
     </row>
-    <row r="784" ht="22" customHeight="1">
-      <c r="A784" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (779 BAL)</t>
-        </is>
-      </c>
-      <c r="B784" s="4" t="n"/>
-      <c r="C784" s="4" t="n"/>
-      <c r="D784" s="4" t="n"/>
-      <c r="E784" s="4">
-        <f>SUM(E5:E783)</f>
+    <row r="784" ht="20.25" customHeight="1">
+      <c r="A784" s="5" t="n">
+        <v>1047</v>
+      </c>
+      <c r="B784" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C784" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D784" s="6" t="inlineStr">
+        <is>
+          <t>284912</t>
+        </is>
+      </c>
+      <c r="E784" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F784" s="5" t="n"/>
+    </row>
+    <row r="785" ht="20.25" customHeight="1">
+      <c r="A785" s="5" t="n">
+        <v>1048</v>
+      </c>
+      <c r="B785" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C785" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D785" s="6" t="inlineStr">
+        <is>
+          <t>284626</t>
+        </is>
+      </c>
+      <c r="E785" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F785" s="5" t="n"/>
+    </row>
+    <row r="786" ht="20.25" customHeight="1">
+      <c r="A786" s="5" t="n">
+        <v>1049</v>
+      </c>
+      <c r="B786" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C786" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D786" s="6" t="inlineStr">
+        <is>
+          <t>284906</t>
+        </is>
+      </c>
+      <c r="E786" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F786" s="5" t="n"/>
+    </row>
+    <row r="787" ht="20.25" customHeight="1">
+      <c r="A787" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="B787" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C787" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D787" s="6" t="inlineStr">
+        <is>
+          <t>284908</t>
+        </is>
+      </c>
+      <c r="E787" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F787" s="5" t="n"/>
+    </row>
+    <row r="788" ht="20.25" customHeight="1">
+      <c r="A788" s="5" t="n">
+        <v>1051</v>
+      </c>
+      <c r="B788" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C788" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D788" s="6" t="inlineStr">
+        <is>
+          <t>284721</t>
+        </is>
+      </c>
+      <c r="E788" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F788" s="5" t="n"/>
+    </row>
+    <row r="789" ht="20.25" customHeight="1">
+      <c r="A789" s="5" t="n">
+        <v>1052</v>
+      </c>
+      <c r="B789" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C789" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D789" s="6" t="inlineStr">
+        <is>
+          <t>284627</t>
+        </is>
+      </c>
+      <c r="E789" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F789" s="5" t="n"/>
+    </row>
+    <row r="790" ht="20.25" customHeight="1">
+      <c r="A790" s="5" t="n">
+        <v>1053</v>
+      </c>
+      <c r="B790" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C790" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D790" s="6" t="inlineStr">
+        <is>
+          <t>284628</t>
+        </is>
+      </c>
+      <c r="E790" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F790" s="5" t="n"/>
+    </row>
+    <row r="791" ht="20.25" customHeight="1">
+      <c r="A791" s="5" t="n">
+        <v>1054</v>
+      </c>
+      <c r="B791" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C791" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D791" s="6" t="inlineStr">
+        <is>
+          <t>284911</t>
+        </is>
+      </c>
+      <c r="E791" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F791" s="5" t="n"/>
+    </row>
+    <row r="792" ht="20.25" customHeight="1">
+      <c r="A792" s="5" t="n">
+        <v>1055</v>
+      </c>
+      <c r="B792" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C792" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D792" s="6" t="inlineStr">
+        <is>
+          <t>284909</t>
+        </is>
+      </c>
+      <c r="E792" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F792" s="5" t="n"/>
+    </row>
+    <row r="793" ht="20.25" customHeight="1">
+      <c r="A793" s="5" t="n">
+        <v>1056</v>
+      </c>
+      <c r="B793" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C793" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D793" s="6" t="inlineStr">
+        <is>
+          <t>284910</t>
+        </is>
+      </c>
+      <c r="E793" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F793" s="5" t="n"/>
+    </row>
+    <row r="794" ht="20.25" customHeight="1">
+      <c r="A794" s="5" t="n">
+        <v>1057</v>
+      </c>
+      <c r="B794" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C794" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D794" s="6" t="inlineStr">
+        <is>
+          <t>284914</t>
+        </is>
+      </c>
+      <c r="E794" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F794" s="5" t="n"/>
+    </row>
+    <row r="795" ht="20.25" customHeight="1">
+      <c r="A795" s="5" t="n">
+        <v>1058</v>
+      </c>
+      <c r="B795" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C795" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D795" s="6" t="inlineStr">
+        <is>
+          <t>284913</t>
+        </is>
+      </c>
+      <c r="E795" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F795" s="5" t="n"/>
+    </row>
+    <row r="796" ht="20.25" customHeight="1">
+      <c r="A796" s="5" t="n">
+        <v>1059</v>
+      </c>
+      <c r="B796" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C796" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D796" s="6" t="inlineStr">
+        <is>
+          <t>284717</t>
+        </is>
+      </c>
+      <c r="E796" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F796" s="5" t="n"/>
+    </row>
+    <row r="797" ht="20.25" customHeight="1">
+      <c r="A797" s="5" t="n">
+        <v>1060</v>
+      </c>
+      <c r="B797" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C797" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D797" s="6" t="inlineStr">
+        <is>
+          <t>284718</t>
+        </is>
+      </c>
+      <c r="E797" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F797" s="5" t="n"/>
+    </row>
+    <row r="798" ht="20.25" customHeight="1">
+      <c r="A798" s="5" t="n">
+        <v>1093</v>
+      </c>
+      <c r="B798" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C798" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D798" s="6" t="inlineStr">
+        <is>
+          <t>284907</t>
+        </is>
+      </c>
+      <c r="E798" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F798" s="5" t="n"/>
+    </row>
+    <row r="799" ht="20.25" customHeight="1">
+      <c r="A799" s="5" t="n">
+        <v>1094</v>
+      </c>
+      <c r="B799" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C799" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D799" s="6" t="inlineStr">
+        <is>
+          <t>284637</t>
+        </is>
+      </c>
+      <c r="E799" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F799" s="5" t="n"/>
+    </row>
+    <row r="800" ht="20.25" customHeight="1">
+      <c r="A800" s="5" t="n">
+        <v>1095</v>
+      </c>
+      <c r="B800" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C800" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D800" s="6" t="inlineStr">
+        <is>
+          <t>284282</t>
+        </is>
+      </c>
+      <c r="E800" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F800" s="5" t="n"/>
+    </row>
+    <row r="801" ht="20.25" customHeight="1">
+      <c r="A801" s="5" t="n">
+        <v>1096</v>
+      </c>
+      <c r="B801" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C801" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D801" s="6" t="inlineStr">
+        <is>
+          <t>284715</t>
+        </is>
+      </c>
+      <c r="E801" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F801" s="5" t="n"/>
+    </row>
+    <row r="802" ht="20.25" customHeight="1">
+      <c r="A802" s="5" t="n">
+        <v>1097</v>
+      </c>
+      <c r="B802" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C802" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D802" s="6" t="inlineStr">
+        <is>
+          <t>284716</t>
+        </is>
+      </c>
+      <c r="E802" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F802" s="5" t="n"/>
+    </row>
+    <row r="803" ht="20.25" customHeight="1">
+      <c r="A803" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="B803" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C803" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D803" s="6" t="inlineStr">
+        <is>
+          <t>284283</t>
+        </is>
+      </c>
+      <c r="E803" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F803" s="5" t="n"/>
+    </row>
+    <row r="804" ht="20.25" customHeight="1">
+      <c r="A804" s="5" t="n">
+        <v>1099</v>
+      </c>
+      <c r="B804" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C804" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D804" s="6" t="inlineStr">
+        <is>
+          <t>284904</t>
+        </is>
+      </c>
+      <c r="E804" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F804" s="5" t="n"/>
+    </row>
+    <row r="805" ht="20.25" customHeight="1">
+      <c r="A805" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="B805" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C805" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D805" s="6" t="inlineStr">
+        <is>
+          <t>284905</t>
+        </is>
+      </c>
+      <c r="E805" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F805" s="5" t="n"/>
+    </row>
+    <row r="806" ht="20.25" customHeight="1">
+      <c r="A806" s="5" t="n">
+        <v>1101</v>
+      </c>
+      <c r="B806" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C806" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D806" s="6" t="inlineStr">
+        <is>
+          <t>284901</t>
+        </is>
+      </c>
+      <c r="E806" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F806" s="5" t="n"/>
+    </row>
+    <row r="807" ht="20.25" customHeight="1">
+      <c r="A807" s="5" t="n">
+        <v>1102</v>
+      </c>
+      <c r="B807" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C807" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D807" s="6" t="inlineStr">
+        <is>
+          <t>284902</t>
+        </is>
+      </c>
+      <c r="E807" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F807" s="5" t="n"/>
+    </row>
+    <row r="808" ht="20.25" customHeight="1">
+      <c r="A808" s="5" t="n">
+        <v>1103</v>
+      </c>
+      <c r="B808" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C808" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D808" s="6" t="inlineStr">
+        <is>
+          <t>284903</t>
+        </is>
+      </c>
+      <c r="E808" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F808" s="5" t="n"/>
+    </row>
+    <row r="809" ht="20.25" customHeight="1">
+      <c r="A809" s="5" t="n">
+        <v>1104</v>
+      </c>
+      <c r="B809" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C809" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D809" s="6" t="inlineStr">
+        <is>
+          <t>284636</t>
+        </is>
+      </c>
+      <c r="E809" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F809" s="5" t="n"/>
+    </row>
+    <row r="810" ht="20.25" customHeight="1">
+      <c r="A810" s="5" t="n">
+        <v>1105</v>
+      </c>
+      <c r="B810" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C810" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D810" s="6" t="inlineStr">
+        <is>
+          <t>284919</t>
+        </is>
+      </c>
+      <c r="E810" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F810" s="5" t="n"/>
+    </row>
+    <row r="811" ht="20.25" customHeight="1">
+      <c r="A811" s="5" t="n">
+        <v>1106</v>
+      </c>
+      <c r="B811" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="C811" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D811" s="6" t="inlineStr">
+        <is>
+          <t>284635</t>
+        </is>
+      </c>
+      <c r="E811" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F811" s="5" t="n"/>
+    </row>
+    <row r="812" ht="20.25" customHeight="1">
+      <c r="A812" s="5" t="n">
+        <v>1107</v>
+      </c>
+      <c r="B812" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C812" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D812" s="6" t="inlineStr">
+        <is>
+          <t>284634</t>
+        </is>
+      </c>
+      <c r="E812" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F812" s="5" t="n"/>
+    </row>
+    <row r="813" ht="20.25" customHeight="1">
+      <c r="A813" s="5" t="n">
+        <v>1108</v>
+      </c>
+      <c r="B813" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C813" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D813" s="6" t="inlineStr">
+        <is>
+          <t>284920</t>
+        </is>
+      </c>
+      <c r="E813" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F813" s="5" t="n"/>
+    </row>
+    <row r="814" ht="20.25" customHeight="1">
+      <c r="A814" s="5" t="n">
+        <v>1109</v>
+      </c>
+      <c r="B814" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C814" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D814" s="6" t="inlineStr">
+        <is>
+          <t>284629</t>
+        </is>
+      </c>
+      <c r="E814" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F814" s="5" t="n"/>
+    </row>
+    <row r="815" ht="20.25" customHeight="1">
+      <c r="A815" s="5" t="n">
+        <v>1110</v>
+      </c>
+      <c r="B815" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C815" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D815" s="6" t="inlineStr">
+        <is>
+          <t>284633</t>
+        </is>
+      </c>
+      <c r="E815" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F815" s="5" t="n"/>
+    </row>
+    <row r="816" ht="20.25" customHeight="1">
+      <c r="A816" s="5" t="n">
+        <v>1111</v>
+      </c>
+      <c r="B816" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C816" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D816" s="6" t="inlineStr">
+        <is>
+          <t>284632</t>
+        </is>
+      </c>
+      <c r="E816" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F816" s="5" t="n"/>
+    </row>
+    <row r="817" ht="20.25" customHeight="1">
+      <c r="A817" s="5" t="n">
+        <v>1112</v>
+      </c>
+      <c r="B817" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C817" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D817" s="6" t="inlineStr">
+        <is>
+          <t>284630</t>
+        </is>
+      </c>
+      <c r="E817" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F817" s="5" t="n"/>
+    </row>
+    <row r="818" ht="20.25" customHeight="1">
+      <c r="A818" s="5" t="n">
+        <v>1113</v>
+      </c>
+      <c r="B818" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C818" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D818" s="6" t="inlineStr">
+        <is>
+          <t>284631</t>
+        </is>
+      </c>
+      <c r="E818" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F818" s="5" t="n"/>
+    </row>
+    <row r="819" ht="20.25" customHeight="1">
+      <c r="A819" s="5" t="n">
+        <v>1114</v>
+      </c>
+      <c r="B819" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C819" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D819" s="6" t="inlineStr">
+        <is>
+          <t>284918</t>
+        </is>
+      </c>
+      <c r="E819" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F819" s="5" t="n"/>
+    </row>
+    <row r="820" ht="20.25" customHeight="1">
+      <c r="A820" s="5" t="n">
+        <v>1115</v>
+      </c>
+      <c r="B820" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C820" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D820" s="6" t="inlineStr">
+        <is>
+          <t>284916</t>
+        </is>
+      </c>
+      <c r="E820" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F820" s="5" t="n"/>
+    </row>
+    <row r="821" ht="20.25" customHeight="1">
+      <c r="A821" s="5" t="n">
+        <v>1116</v>
+      </c>
+      <c r="B821" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C821" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D821" s="6" t="inlineStr">
+        <is>
+          <t>284915</t>
+        </is>
+      </c>
+      <c r="E821" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F821" s="5" t="n"/>
+    </row>
+    <row r="822" ht="20.25" customHeight="1">
+      <c r="A822" s="5" t="n">
+        <v>1117</v>
+      </c>
+      <c r="B822" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C822" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D822" s="6" t="inlineStr">
+        <is>
+          <t>284917</t>
+        </is>
+      </c>
+      <c r="E822" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F822" s="5" t="n"/>
+    </row>
+    <row r="823" ht="20.25" customHeight="1">
+      <c r="A823" s="5" t="n">
+        <v>1118</v>
+      </c>
+      <c r="B823" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C823" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D823" s="6" t="inlineStr">
+        <is>
+          <t>284720</t>
+        </is>
+      </c>
+      <c r="E823" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F823" s="5" t="n"/>
+    </row>
+    <row r="824" ht="20.25" customHeight="1">
+      <c r="A824" s="5" t="n">
+        <v>1119</v>
+      </c>
+      <c r="B824" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C824" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D824" s="6" t="inlineStr">
+        <is>
+          <t>284719</t>
+        </is>
+      </c>
+      <c r="E824" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F824" s="5" t="n"/>
+    </row>
+    <row r="825" ht="20.25" customHeight="1">
+      <c r="A825" s="5" t="n">
+        <v>1120</v>
+      </c>
+      <c r="B825" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C825" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D825" s="6" t="inlineStr">
+        <is>
+          <t>284922</t>
+        </is>
+      </c>
+      <c r="E825" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F825" s="5" t="n"/>
+    </row>
+    <row r="826" ht="20.25" customHeight="1">
+      <c r="A826" s="5" t="n">
+        <v>1121</v>
+      </c>
+      <c r="B826" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C826" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D826" s="6" t="inlineStr">
+        <is>
+          <t>284823</t>
+        </is>
+      </c>
+      <c r="E826" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F826" s="5" t="n"/>
+    </row>
+    <row r="827" ht="20.25" customHeight="1">
+      <c r="A827" s="5" t="n">
+        <v>1122</v>
+      </c>
+      <c r="B827" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C827" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D827" s="6" t="inlineStr">
+        <is>
+          <t>280336</t>
+        </is>
+      </c>
+      <c r="E827" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F827" s="5" t="n"/>
+    </row>
+    <row r="828" ht="20.25" customHeight="1">
+      <c r="A828" s="5" t="n">
+        <v>1123</v>
+      </c>
+      <c r="B828" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C828" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D828" s="6" t="inlineStr">
+        <is>
+          <t>284822</t>
+        </is>
+      </c>
+      <c r="E828" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F828" s="5" t="n"/>
+    </row>
+    <row r="829" ht="20.25" customHeight="1">
+      <c r="A829" s="5" t="n">
+        <v>1124</v>
+      </c>
+      <c r="B829" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C829" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D829" s="6" t="inlineStr">
+        <is>
+          <t>284820</t>
+        </is>
+      </c>
+      <c r="E829" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F829" s="5" t="n"/>
+    </row>
+    <row r="830" ht="20.25" customHeight="1">
+      <c r="A830" s="5" t="n">
+        <v>1125</v>
+      </c>
+      <c r="B830" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C830" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D830" s="6" t="inlineStr">
+        <is>
+          <t>284819</t>
+        </is>
+      </c>
+      <c r="E830" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F830" s="5" t="n"/>
+    </row>
+    <row r="831" ht="20.25" customHeight="1">
+      <c r="A831" s="5" t="n">
+        <v>1127</v>
+      </c>
+      <c r="B831" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C831" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D831" s="6" t="inlineStr">
+        <is>
+          <t>284821</t>
+        </is>
+      </c>
+      <c r="E831" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F831" s="5" t="n"/>
+    </row>
+    <row r="832" ht="20.25" customHeight="1">
+      <c r="A832" s="5" t="n">
+        <v>1128</v>
+      </c>
+      <c r="B832" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C832" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D832" s="6" t="inlineStr">
+        <is>
+          <t>284422</t>
+        </is>
+      </c>
+      <c r="E832" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F832" s="5" t="n"/>
+    </row>
+    <row r="833" ht="20.25" customHeight="1">
+      <c r="A833" s="5" t="n">
+        <v>1131</v>
+      </c>
+      <c r="B833" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C833" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D833" s="6" t="inlineStr">
+        <is>
+          <t>284833</t>
+        </is>
+      </c>
+      <c r="E833" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F833" s="5" t="n"/>
+    </row>
+    <row r="834" ht="20.25" customHeight="1">
+      <c r="A834" s="5" t="n">
+        <v>1132</v>
+      </c>
+      <c r="B834" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C834" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D834" s="6" t="inlineStr">
+        <is>
+          <t>284922</t>
+        </is>
+      </c>
+      <c r="E834" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F834" s="5" t="n"/>
+    </row>
+    <row r="835" ht="20.25" customHeight="1">
+      <c r="A835" s="5" t="n">
+        <v>1133</v>
+      </c>
+      <c r="B835" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C835" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D835" s="6" t="inlineStr">
+        <is>
+          <t>284921</t>
+        </is>
+      </c>
+      <c r="E835" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F835" s="5" t="n"/>
+    </row>
+    <row r="836" ht="20.25" customHeight="1">
+      <c r="A836" s="5" t="n">
+        <v>1134</v>
+      </c>
+      <c r="B836" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C836" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D836" s="6" t="inlineStr">
+        <is>
+          <t>284830</t>
+        </is>
+      </c>
+      <c r="E836" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F836" s="5" t="n"/>
+    </row>
+    <row r="837" ht="20.25" customHeight="1">
+      <c r="A837" s="5" t="n">
+        <v>1135</v>
+      </c>
+      <c r="B837" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C837" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D837" s="6" t="inlineStr">
+        <is>
+          <t>280338</t>
+        </is>
+      </c>
+      <c r="E837" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F837" s="5" t="n"/>
+    </row>
+    <row r="838" ht="20.25" customHeight="1">
+      <c r="A838" s="5" t="n">
+        <v>1136</v>
+      </c>
+      <c r="B838" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C838" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D838" s="6" t="inlineStr">
+        <is>
+          <t>282923</t>
+        </is>
+      </c>
+      <c r="E838" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F838" s="5" t="n"/>
+    </row>
+    <row r="839" ht="20.25" customHeight="1">
+      <c r="A839" s="5" t="n">
+        <v>1137</v>
+      </c>
+      <c r="B839" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C839" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D839" s="6" t="inlineStr">
+        <is>
+          <t>284831</t>
+        </is>
+      </c>
+      <c r="E839" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F839" s="5" t="n"/>
+    </row>
+    <row r="840" ht="20.25" customHeight="1">
+      <c r="A840" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="B840" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C840" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D840" s="6" t="inlineStr">
+        <is>
+          <t>284832</t>
+        </is>
+      </c>
+      <c r="E840" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F840" s="5" t="n"/>
+    </row>
+    <row r="841" ht="20.25" customHeight="1">
+      <c r="A841" s="5" t="n">
+        <v>1139</v>
+      </c>
+      <c r="B841" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C841" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D841" s="6" t="inlineStr">
+        <is>
+          <t>284427</t>
+        </is>
+      </c>
+      <c r="E841" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F841" s="5" t="n"/>
+    </row>
+    <row r="842" ht="20.25" customHeight="1">
+      <c r="A842" s="5" t="n">
+        <v>1140</v>
+      </c>
+      <c r="B842" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C842" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D842" s="6" t="inlineStr">
+        <is>
+          <t>280337</t>
+        </is>
+      </c>
+      <c r="E842" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F842" s="5" t="n"/>
+    </row>
+    <row r="843" ht="20.25" customHeight="1">
+      <c r="A843" s="5" t="n">
+        <v>1141</v>
+      </c>
+      <c r="B843" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C843" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D843" s="6" t="inlineStr">
+        <is>
+          <t>284426</t>
+        </is>
+      </c>
+      <c r="E843" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F843" s="5" t="n"/>
+    </row>
+    <row r="844" ht="20.25" customHeight="1">
+      <c r="A844" s="5" t="n">
+        <v>1142</v>
+      </c>
+      <c r="B844" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C844" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D844" s="6" t="inlineStr">
+        <is>
+          <t>284425</t>
+        </is>
+      </c>
+      <c r="E844" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F844" s="5" t="n"/>
+    </row>
+    <row r="845" ht="20.25" customHeight="1">
+      <c r="A845" s="5" t="n">
+        <v>1143</v>
+      </c>
+      <c r="B845" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C845" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D845" s="6" t="inlineStr">
+        <is>
+          <t>284829</t>
+        </is>
+      </c>
+      <c r="E845" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F845" s="5" t="n"/>
+    </row>
+    <row r="846" ht="20.25" customHeight="1">
+      <c r="A846" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="B846" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C846" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D846" s="6" t="inlineStr">
+        <is>
+          <t>284824</t>
+        </is>
+      </c>
+      <c r="E846" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F846" s="5" t="n"/>
+    </row>
+    <row r="847" ht="20.25" customHeight="1">
+      <c r="A847" s="5" t="n">
+        <v>1145</v>
+      </c>
+      <c r="B847" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C847" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D847" s="6" t="inlineStr">
+        <is>
+          <t>284825</t>
+        </is>
+      </c>
+      <c r="E847" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F847" s="5" t="n"/>
+    </row>
+    <row r="848" ht="20.25" customHeight="1">
+      <c r="A848" s="5" t="n">
+        <v>1146</v>
+      </c>
+      <c r="B848" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C848" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D848" s="6" t="inlineStr">
+        <is>
+          <t>284828</t>
+        </is>
+      </c>
+      <c r="E848" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F848" s="5" t="n"/>
+    </row>
+    <row r="849" ht="20.25" customHeight="1">
+      <c r="A849" s="5" t="n">
+        <v>1147</v>
+      </c>
+      <c r="B849" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C849" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D849" s="6" t="inlineStr">
+        <is>
+          <t>284826</t>
+        </is>
+      </c>
+      <c r="E849" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F849" s="5" t="n"/>
+    </row>
+    <row r="850" ht="20.25" customHeight="1">
+      <c r="A850" s="5" t="n">
+        <v>1148</v>
+      </c>
+      <c r="B850" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C850" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D850" s="6" t="inlineStr">
+        <is>
+          <t>284827</t>
+        </is>
+      </c>
+      <c r="E850" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F850" s="5" t="n"/>
+    </row>
+    <row r="851" ht="20.25" customHeight="1">
+      <c r="A851" s="5" t="n">
+        <v>1150</v>
+      </c>
+      <c r="B851" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C851" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D851" s="6" t="inlineStr">
+        <is>
+          <t>284424</t>
+        </is>
+      </c>
+      <c r="E851" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F851" s="5" t="n"/>
+    </row>
+    <row r="852" ht="20.25" customHeight="1">
+      <c r="A852" s="5" t="n">
+        <v>1151</v>
+      </c>
+      <c r="B852" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C852" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D852" s="6" t="inlineStr">
+        <is>
+          <t>284423</t>
+        </is>
+      </c>
+      <c r="E852" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F852" s="5" t="n"/>
+    </row>
+    <row r="853" ht="20.25" customHeight="1">
+      <c r="A853" s="5" t="n">
+        <v>1153</v>
+      </c>
+      <c r="B853" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C853" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D853" s="6" t="inlineStr">
+        <is>
+          <t>284722</t>
+        </is>
+      </c>
+      <c r="E853" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F853" s="5" t="n"/>
+    </row>
+    <row r="854" ht="20.25" customHeight="1">
+      <c r="A854" s="5" t="n">
+        <v>1154</v>
+      </c>
+      <c r="B854" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C854" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D854" s="6" t="inlineStr">
+        <is>
+          <t>284284</t>
+        </is>
+      </c>
+      <c r="E854" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F854" s="5" t="n"/>
+    </row>
+    <row r="855" ht="22" customHeight="1">
+      <c r="A855" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (850 BAL)</t>
+        </is>
+      </c>
+      <c r="B855" s="4" t="n"/>
+      <c r="C855" s="4" t="n"/>
+      <c r="D855" s="4" t="n"/>
+      <c r="E855" s="4">
+        <f>SUM(E5:E854)</f>
         <v/>
       </c>
-      <c r="F784" s="4" t="inlineStr">
+      <c r="F855" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -16201,8 +17621,8 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A784:D784"/>
     <mergeCell ref="B3:C4"/>
+    <mergeCell ref="A855:D855"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16214,7 +17634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I784"/>
+  <dimension ref="A1:I855"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -16238,7 +17658,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 779 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 850 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -45112,23 +46532,2650 @@
         </is>
       </c>
     </row>
-    <row r="784">
-      <c r="A784" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (779 BAL)</t>
-        </is>
-      </c>
-      <c r="B784" s="4" t="n"/>
-      <c r="C784" s="4" t="n"/>
-      <c r="D784" s="4" t="n"/>
-      <c r="E784" s="4" t="n"/>
-      <c r="F784" s="4" t="n"/>
-      <c r="G784" s="4" t="n"/>
-      <c r="H784" s="4">
-        <f>SUM(H5:H783)</f>
+    <row r="784" ht="20" customHeight="1">
+      <c r="A784" s="9" t="n">
+        <v>780</v>
+      </c>
+      <c r="B784" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C784" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D784" s="9" t="n">
+        <v>1047</v>
+      </c>
+      <c r="E784" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F784" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G784" s="10" t="inlineStr">
+        <is>
+          <t>284912</t>
+        </is>
+      </c>
+      <c r="H784" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I784" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="785" ht="20" customHeight="1">
+      <c r="A785" s="9" t="n">
+        <v>781</v>
+      </c>
+      <c r="B785" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C785" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D785" s="9" t="n">
+        <v>1048</v>
+      </c>
+      <c r="E785" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F785" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G785" s="10" t="inlineStr">
+        <is>
+          <t>284626</t>
+        </is>
+      </c>
+      <c r="H785" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I785" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="786" ht="20" customHeight="1">
+      <c r="A786" s="9" t="n">
+        <v>782</v>
+      </c>
+      <c r="B786" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C786" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D786" s="9" t="n">
+        <v>1049</v>
+      </c>
+      <c r="E786" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F786" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G786" s="10" t="inlineStr">
+        <is>
+          <t>284906</t>
+        </is>
+      </c>
+      <c r="H786" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I786" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="787" ht="20" customHeight="1">
+      <c r="A787" s="9" t="n">
+        <v>783</v>
+      </c>
+      <c r="B787" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C787" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D787" s="9" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E787" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F787" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G787" s="10" t="inlineStr">
+        <is>
+          <t>284908</t>
+        </is>
+      </c>
+      <c r="H787" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I787" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="788" ht="20" customHeight="1">
+      <c r="A788" s="9" t="n">
+        <v>784</v>
+      </c>
+      <c r="B788" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C788" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D788" s="9" t="n">
+        <v>1051</v>
+      </c>
+      <c r="E788" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F788" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G788" s="10" t="inlineStr">
+        <is>
+          <t>284721</t>
+        </is>
+      </c>
+      <c r="H788" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I788" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="789" ht="20" customHeight="1">
+      <c r="A789" s="9" t="n">
+        <v>785</v>
+      </c>
+      <c r="B789" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C789" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D789" s="9" t="n">
+        <v>1052</v>
+      </c>
+      <c r="E789" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F789" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G789" s="10" t="inlineStr">
+        <is>
+          <t>284627</t>
+        </is>
+      </c>
+      <c r="H789" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I789" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="790" ht="20" customHeight="1">
+      <c r="A790" s="9" t="n">
+        <v>786</v>
+      </c>
+      <c r="B790" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C790" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D790" s="9" t="n">
+        <v>1053</v>
+      </c>
+      <c r="E790" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F790" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G790" s="10" t="inlineStr">
+        <is>
+          <t>284628</t>
+        </is>
+      </c>
+      <c r="H790" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I790" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="791" ht="20" customHeight="1">
+      <c r="A791" s="9" t="n">
+        <v>787</v>
+      </c>
+      <c r="B791" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C791" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D791" s="9" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E791" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F791" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G791" s="10" t="inlineStr">
+        <is>
+          <t>284911</t>
+        </is>
+      </c>
+      <c r="H791" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I791" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="792" ht="20" customHeight="1">
+      <c r="A792" s="9" t="n">
+        <v>788</v>
+      </c>
+      <c r="B792" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C792" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D792" s="9" t="n">
+        <v>1055</v>
+      </c>
+      <c r="E792" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F792" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G792" s="10" t="inlineStr">
+        <is>
+          <t>284909</t>
+        </is>
+      </c>
+      <c r="H792" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I792" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="793" ht="20" customHeight="1">
+      <c r="A793" s="9" t="n">
+        <v>789</v>
+      </c>
+      <c r="B793" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C793" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D793" s="9" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E793" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F793" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G793" s="10" t="inlineStr">
+        <is>
+          <t>284910</t>
+        </is>
+      </c>
+      <c r="H793" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I793" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="794" ht="20" customHeight="1">
+      <c r="A794" s="9" t="n">
+        <v>790</v>
+      </c>
+      <c r="B794" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C794" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D794" s="9" t="n">
+        <v>1057</v>
+      </c>
+      <c r="E794" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F794" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G794" s="10" t="inlineStr">
+        <is>
+          <t>284914</t>
+        </is>
+      </c>
+      <c r="H794" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I794" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="795" ht="20" customHeight="1">
+      <c r="A795" s="9" t="n">
+        <v>791</v>
+      </c>
+      <c r="B795" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C795" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D795" s="9" t="n">
+        <v>1058</v>
+      </c>
+      <c r="E795" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F795" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G795" s="10" t="inlineStr">
+        <is>
+          <t>284913</t>
+        </is>
+      </c>
+      <c r="H795" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I795" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="796" ht="20" customHeight="1">
+      <c r="A796" s="9" t="n">
+        <v>792</v>
+      </c>
+      <c r="B796" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C796" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D796" s="9" t="n">
+        <v>1059</v>
+      </c>
+      <c r="E796" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F796" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G796" s="10" t="inlineStr">
+        <is>
+          <t>284717</t>
+        </is>
+      </c>
+      <c r="H796" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I796" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="797" ht="20" customHeight="1">
+      <c r="A797" s="9" t="n">
+        <v>793</v>
+      </c>
+      <c r="B797" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C797" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D797" s="9" t="n">
+        <v>1060</v>
+      </c>
+      <c r="E797" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F797" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G797" s="10" t="inlineStr">
+        <is>
+          <t>284718</t>
+        </is>
+      </c>
+      <c r="H797" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I797" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="798" ht="20" customHeight="1">
+      <c r="A798" s="9" t="n">
+        <v>794</v>
+      </c>
+      <c r="B798" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C798" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D798" s="9" t="n">
+        <v>1093</v>
+      </c>
+      <c r="E798" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F798" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G798" s="10" t="inlineStr">
+        <is>
+          <t>284907</t>
+        </is>
+      </c>
+      <c r="H798" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I798" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="799" ht="20" customHeight="1">
+      <c r="A799" s="9" t="n">
+        <v>795</v>
+      </c>
+      <c r="B799" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C799" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D799" s="9" t="n">
+        <v>1094</v>
+      </c>
+      <c r="E799" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F799" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G799" s="10" t="inlineStr">
+        <is>
+          <t>284637</t>
+        </is>
+      </c>
+      <c r="H799" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I799" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="800" ht="20" customHeight="1">
+      <c r="A800" s="9" t="n">
+        <v>796</v>
+      </c>
+      <c r="B800" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C800" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D800" s="9" t="n">
+        <v>1095</v>
+      </c>
+      <c r="E800" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F800" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G800" s="10" t="inlineStr">
+        <is>
+          <t>284282</t>
+        </is>
+      </c>
+      <c r="H800" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I800" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="801" ht="20" customHeight="1">
+      <c r="A801" s="9" t="n">
+        <v>797</v>
+      </c>
+      <c r="B801" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C801" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D801" s="9" t="n">
+        <v>1096</v>
+      </c>
+      <c r="E801" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F801" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G801" s="10" t="inlineStr">
+        <is>
+          <t>284715</t>
+        </is>
+      </c>
+      <c r="H801" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I801" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="802" ht="20" customHeight="1">
+      <c r="A802" s="9" t="n">
+        <v>798</v>
+      </c>
+      <c r="B802" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C802" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D802" s="9" t="n">
+        <v>1097</v>
+      </c>
+      <c r="E802" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F802" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G802" s="10" t="inlineStr">
+        <is>
+          <t>284716</t>
+        </is>
+      </c>
+      <c r="H802" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I802" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="803" ht="20" customHeight="1">
+      <c r="A803" s="9" t="n">
+        <v>799</v>
+      </c>
+      <c r="B803" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C803" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D803" s="9" t="n">
+        <v>1098</v>
+      </c>
+      <c r="E803" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F803" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G803" s="10" t="inlineStr">
+        <is>
+          <t>284283</t>
+        </is>
+      </c>
+      <c r="H803" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I803" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="804" ht="20" customHeight="1">
+      <c r="A804" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="B804" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C804" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D804" s="9" t="n">
+        <v>1099</v>
+      </c>
+      <c r="E804" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F804" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G804" s="10" t="inlineStr">
+        <is>
+          <t>284904</t>
+        </is>
+      </c>
+      <c r="H804" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I804" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="805" ht="20" customHeight="1">
+      <c r="A805" s="9" t="n">
+        <v>801</v>
+      </c>
+      <c r="B805" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C805" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D805" s="9" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E805" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F805" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G805" s="10" t="inlineStr">
+        <is>
+          <t>284905</t>
+        </is>
+      </c>
+      <c r="H805" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I805" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="806" ht="20" customHeight="1">
+      <c r="A806" s="9" t="n">
+        <v>802</v>
+      </c>
+      <c r="B806" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C806" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D806" s="9" t="n">
+        <v>1101</v>
+      </c>
+      <c r="E806" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F806" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G806" s="10" t="inlineStr">
+        <is>
+          <t>284901</t>
+        </is>
+      </c>
+      <c r="H806" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I806" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="807" ht="20" customHeight="1">
+      <c r="A807" s="9" t="n">
+        <v>803</v>
+      </c>
+      <c r="B807" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C807" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D807" s="9" t="n">
+        <v>1102</v>
+      </c>
+      <c r="E807" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F807" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G807" s="10" t="inlineStr">
+        <is>
+          <t>284902</t>
+        </is>
+      </c>
+      <c r="H807" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I807" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="808" ht="20" customHeight="1">
+      <c r="A808" s="9" t="n">
+        <v>804</v>
+      </c>
+      <c r="B808" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C808" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D808" s="9" t="n">
+        <v>1103</v>
+      </c>
+      <c r="E808" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F808" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G808" s="10" t="inlineStr">
+        <is>
+          <t>284903</t>
+        </is>
+      </c>
+      <c r="H808" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I808" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="809" ht="20" customHeight="1">
+      <c r="A809" s="9" t="n">
+        <v>805</v>
+      </c>
+      <c r="B809" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C809" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D809" s="9" t="n">
+        <v>1104</v>
+      </c>
+      <c r="E809" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F809" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G809" s="10" t="inlineStr">
+        <is>
+          <t>284636</t>
+        </is>
+      </c>
+      <c r="H809" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I809" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="810" ht="20" customHeight="1">
+      <c r="A810" s="9" t="n">
+        <v>806</v>
+      </c>
+      <c r="B810" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C810" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D810" s="9" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E810" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F810" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G810" s="10" t="inlineStr">
+        <is>
+          <t>284919</t>
+        </is>
+      </c>
+      <c r="H810" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I810" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="811" ht="20" customHeight="1">
+      <c r="A811" s="9" t="n">
+        <v>807</v>
+      </c>
+      <c r="B811" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C811" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D811" s="9" t="n">
+        <v>1106</v>
+      </c>
+      <c r="E811" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F811" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G811" s="10" t="inlineStr">
+        <is>
+          <t>284635</t>
+        </is>
+      </c>
+      <c r="H811" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I811" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="812" ht="20" customHeight="1">
+      <c r="A812" s="9" t="n">
+        <v>808</v>
+      </c>
+      <c r="B812" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C812" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D812" s="9" t="n">
+        <v>1107</v>
+      </c>
+      <c r="E812" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F812" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G812" s="10" t="inlineStr">
+        <is>
+          <t>284634</t>
+        </is>
+      </c>
+      <c r="H812" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I812" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="813" ht="20" customHeight="1">
+      <c r="A813" s="9" t="n">
+        <v>809</v>
+      </c>
+      <c r="B813" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C813" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D813" s="9" t="n">
+        <v>1108</v>
+      </c>
+      <c r="E813" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F813" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G813" s="10" t="inlineStr">
+        <is>
+          <t>284920</t>
+        </is>
+      </c>
+      <c r="H813" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I813" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="814" ht="20" customHeight="1">
+      <c r="A814" s="9" t="n">
+        <v>810</v>
+      </c>
+      <c r="B814" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C814" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D814" s="9" t="n">
+        <v>1109</v>
+      </c>
+      <c r="E814" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F814" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G814" s="10" t="inlineStr">
+        <is>
+          <t>284629</t>
+        </is>
+      </c>
+      <c r="H814" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I814" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="815" ht="20" customHeight="1">
+      <c r="A815" s="9" t="n">
+        <v>811</v>
+      </c>
+      <c r="B815" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C815" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D815" s="9" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E815" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F815" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G815" s="10" t="inlineStr">
+        <is>
+          <t>284633</t>
+        </is>
+      </c>
+      <c r="H815" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I815" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="816" ht="20" customHeight="1">
+      <c r="A816" s="9" t="n">
+        <v>812</v>
+      </c>
+      <c r="B816" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C816" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D816" s="9" t="n">
+        <v>1111</v>
+      </c>
+      <c r="E816" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F816" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G816" s="10" t="inlineStr">
+        <is>
+          <t>284632</t>
+        </is>
+      </c>
+      <c r="H816" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I816" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="817" ht="20" customHeight="1">
+      <c r="A817" s="9" t="n">
+        <v>813</v>
+      </c>
+      <c r="B817" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C817" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D817" s="9" t="n">
+        <v>1112</v>
+      </c>
+      <c r="E817" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F817" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G817" s="10" t="inlineStr">
+        <is>
+          <t>284630</t>
+        </is>
+      </c>
+      <c r="H817" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I817" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="818" ht="20" customHeight="1">
+      <c r="A818" s="9" t="n">
+        <v>814</v>
+      </c>
+      <c r="B818" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C818" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D818" s="9" t="n">
+        <v>1113</v>
+      </c>
+      <c r="E818" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F818" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G818" s="10" t="inlineStr">
+        <is>
+          <t>284631</t>
+        </is>
+      </c>
+      <c r="H818" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I818" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="819" ht="20" customHeight="1">
+      <c r="A819" s="9" t="n">
+        <v>815</v>
+      </c>
+      <c r="B819" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C819" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D819" s="9" t="n">
+        <v>1114</v>
+      </c>
+      <c r="E819" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F819" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G819" s="10" t="inlineStr">
+        <is>
+          <t>284918</t>
+        </is>
+      </c>
+      <c r="H819" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I819" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="820" ht="20" customHeight="1">
+      <c r="A820" s="9" t="n">
+        <v>816</v>
+      </c>
+      <c r="B820" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C820" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D820" s="9" t="n">
+        <v>1115</v>
+      </c>
+      <c r="E820" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F820" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G820" s="10" t="inlineStr">
+        <is>
+          <t>284916</t>
+        </is>
+      </c>
+      <c r="H820" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I820" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="821" ht="20" customHeight="1">
+      <c r="A821" s="9" t="n">
+        <v>817</v>
+      </c>
+      <c r="B821" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C821" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D821" s="9" t="n">
+        <v>1116</v>
+      </c>
+      <c r="E821" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F821" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G821" s="10" t="inlineStr">
+        <is>
+          <t>284915</t>
+        </is>
+      </c>
+      <c r="H821" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I821" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="822" ht="20" customHeight="1">
+      <c r="A822" s="9" t="n">
+        <v>818</v>
+      </c>
+      <c r="B822" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C822" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D822" s="9" t="n">
+        <v>1117</v>
+      </c>
+      <c r="E822" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F822" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G822" s="10" t="inlineStr">
+        <is>
+          <t>284917</t>
+        </is>
+      </c>
+      <c r="H822" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I822" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="823" ht="20" customHeight="1">
+      <c r="A823" s="9" t="n">
+        <v>819</v>
+      </c>
+      <c r="B823" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C823" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D823" s="9" t="n">
+        <v>1118</v>
+      </c>
+      <c r="E823" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F823" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G823" s="10" t="inlineStr">
+        <is>
+          <t>284720</t>
+        </is>
+      </c>
+      <c r="H823" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I823" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="824" ht="20" customHeight="1">
+      <c r="A824" s="9" t="n">
+        <v>820</v>
+      </c>
+      <c r="B824" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C824" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D824" s="9" t="n">
+        <v>1119</v>
+      </c>
+      <c r="E824" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F824" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G824" s="10" t="inlineStr">
+        <is>
+          <t>284719</t>
+        </is>
+      </c>
+      <c r="H824" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I824" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="825" ht="20" customHeight="1">
+      <c r="A825" s="9" t="n">
+        <v>821</v>
+      </c>
+      <c r="B825" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C825" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D825" s="9" t="n">
+        <v>1120</v>
+      </c>
+      <c r="E825" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F825" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G825" s="10" t="inlineStr">
+        <is>
+          <t>284922</t>
+        </is>
+      </c>
+      <c r="H825" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I825" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="826" ht="20" customHeight="1">
+      <c r="A826" s="9" t="n">
+        <v>822</v>
+      </c>
+      <c r="B826" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C826" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D826" s="9" t="n">
+        <v>1121</v>
+      </c>
+      <c r="E826" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F826" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G826" s="10" t="inlineStr">
+        <is>
+          <t>284823</t>
+        </is>
+      </c>
+      <c r="H826" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I826" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="827" ht="20" customHeight="1">
+      <c r="A827" s="9" t="n">
+        <v>823</v>
+      </c>
+      <c r="B827" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C827" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D827" s="9" t="n">
+        <v>1122</v>
+      </c>
+      <c r="E827" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F827" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G827" s="10" t="inlineStr">
+        <is>
+          <t>280336</t>
+        </is>
+      </c>
+      <c r="H827" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I827" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="828" ht="20" customHeight="1">
+      <c r="A828" s="9" t="n">
+        <v>824</v>
+      </c>
+      <c r="B828" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C828" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D828" s="9" t="n">
+        <v>1123</v>
+      </c>
+      <c r="E828" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F828" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G828" s="10" t="inlineStr">
+        <is>
+          <t>284822</t>
+        </is>
+      </c>
+      <c r="H828" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I828" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="829" ht="20" customHeight="1">
+      <c r="A829" s="9" t="n">
+        <v>825</v>
+      </c>
+      <c r="B829" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C829" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D829" s="9" t="n">
+        <v>1124</v>
+      </c>
+      <c r="E829" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F829" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G829" s="10" t="inlineStr">
+        <is>
+          <t>284820</t>
+        </is>
+      </c>
+      <c r="H829" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I829" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="830" ht="20" customHeight="1">
+      <c r="A830" s="9" t="n">
+        <v>826</v>
+      </c>
+      <c r="B830" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C830" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D830" s="9" t="n">
+        <v>1125</v>
+      </c>
+      <c r="E830" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F830" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G830" s="10" t="inlineStr">
+        <is>
+          <t>284819</t>
+        </is>
+      </c>
+      <c r="H830" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I830" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="831" ht="20" customHeight="1">
+      <c r="A831" s="9" t="n">
+        <v>827</v>
+      </c>
+      <c r="B831" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C831" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D831" s="9" t="n">
+        <v>1127</v>
+      </c>
+      <c r="E831" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F831" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G831" s="10" t="inlineStr">
+        <is>
+          <t>284821</t>
+        </is>
+      </c>
+      <c r="H831" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I831" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="832" ht="20" customHeight="1">
+      <c r="A832" s="9" t="n">
+        <v>828</v>
+      </c>
+      <c r="B832" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C832" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D832" s="9" t="n">
+        <v>1128</v>
+      </c>
+      <c r="E832" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F832" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G832" s="10" t="inlineStr">
+        <is>
+          <t>284422</t>
+        </is>
+      </c>
+      <c r="H832" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I832" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="833" ht="20" customHeight="1">
+      <c r="A833" s="9" t="n">
+        <v>829</v>
+      </c>
+      <c r="B833" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C833" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D833" s="9" t="n">
+        <v>1131</v>
+      </c>
+      <c r="E833" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F833" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G833" s="10" t="inlineStr">
+        <is>
+          <t>284833</t>
+        </is>
+      </c>
+      <c r="H833" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I833" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="834" ht="20" customHeight="1">
+      <c r="A834" s="9" t="n">
+        <v>830</v>
+      </c>
+      <c r="B834" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C834" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D834" s="9" t="n">
+        <v>1132</v>
+      </c>
+      <c r="E834" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F834" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G834" s="10" t="inlineStr">
+        <is>
+          <t>284922</t>
+        </is>
+      </c>
+      <c r="H834" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I834" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="835" ht="20" customHeight="1">
+      <c r="A835" s="9" t="n">
+        <v>831</v>
+      </c>
+      <c r="B835" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C835" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D835" s="9" t="n">
+        <v>1133</v>
+      </c>
+      <c r="E835" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F835" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G835" s="10" t="inlineStr">
+        <is>
+          <t>284921</t>
+        </is>
+      </c>
+      <c r="H835" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I835" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="836" ht="20" customHeight="1">
+      <c r="A836" s="9" t="n">
+        <v>832</v>
+      </c>
+      <c r="B836" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C836" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D836" s="9" t="n">
+        <v>1134</v>
+      </c>
+      <c r="E836" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F836" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G836" s="10" t="inlineStr">
+        <is>
+          <t>284830</t>
+        </is>
+      </c>
+      <c r="H836" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I836" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="837" ht="20" customHeight="1">
+      <c r="A837" s="9" t="n">
+        <v>833</v>
+      </c>
+      <c r="B837" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C837" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D837" s="9" t="n">
+        <v>1135</v>
+      </c>
+      <c r="E837" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F837" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G837" s="10" t="inlineStr">
+        <is>
+          <t>280338</t>
+        </is>
+      </c>
+      <c r="H837" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I837" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="838" ht="20" customHeight="1">
+      <c r="A838" s="9" t="n">
+        <v>834</v>
+      </c>
+      <c r="B838" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C838" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D838" s="9" t="n">
+        <v>1136</v>
+      </c>
+      <c r="E838" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F838" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G838" s="10" t="inlineStr">
+        <is>
+          <t>282923</t>
+        </is>
+      </c>
+      <c r="H838" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I838" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="839" ht="20" customHeight="1">
+      <c r="A839" s="9" t="n">
+        <v>835</v>
+      </c>
+      <c r="B839" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C839" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D839" s="9" t="n">
+        <v>1137</v>
+      </c>
+      <c r="E839" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F839" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G839" s="10" t="inlineStr">
+        <is>
+          <t>284831</t>
+        </is>
+      </c>
+      <c r="H839" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I839" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="840" ht="20" customHeight="1">
+      <c r="A840" s="9" t="n">
+        <v>836</v>
+      </c>
+      <c r="B840" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C840" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D840" s="9" t="n">
+        <v>1138</v>
+      </c>
+      <c r="E840" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F840" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G840" s="10" t="inlineStr">
+        <is>
+          <t>284832</t>
+        </is>
+      </c>
+      <c r="H840" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I840" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="841" ht="20" customHeight="1">
+      <c r="A841" s="9" t="n">
+        <v>837</v>
+      </c>
+      <c r="B841" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C841" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D841" s="9" t="n">
+        <v>1139</v>
+      </c>
+      <c r="E841" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F841" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G841" s="10" t="inlineStr">
+        <is>
+          <t>284427</t>
+        </is>
+      </c>
+      <c r="H841" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I841" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="842" ht="20" customHeight="1">
+      <c r="A842" s="9" t="n">
+        <v>838</v>
+      </c>
+      <c r="B842" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C842" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D842" s="9" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E842" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F842" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G842" s="10" t="inlineStr">
+        <is>
+          <t>280337</t>
+        </is>
+      </c>
+      <c r="H842" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I842" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="843" ht="20" customHeight="1">
+      <c r="A843" s="9" t="n">
+        <v>839</v>
+      </c>
+      <c r="B843" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C843" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D843" s="9" t="n">
+        <v>1141</v>
+      </c>
+      <c r="E843" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F843" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G843" s="10" t="inlineStr">
+        <is>
+          <t>284426</t>
+        </is>
+      </c>
+      <c r="H843" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I843" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="844" ht="20" customHeight="1">
+      <c r="A844" s="9" t="n">
+        <v>840</v>
+      </c>
+      <c r="B844" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C844" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D844" s="9" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E844" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F844" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G844" s="10" t="inlineStr">
+        <is>
+          <t>284425</t>
+        </is>
+      </c>
+      <c r="H844" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I844" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="845" ht="20" customHeight="1">
+      <c r="A845" s="9" t="n">
+        <v>841</v>
+      </c>
+      <c r="B845" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C845" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D845" s="9" t="n">
+        <v>1143</v>
+      </c>
+      <c r="E845" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F845" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G845" s="10" t="inlineStr">
+        <is>
+          <t>284829</t>
+        </is>
+      </c>
+      <c r="H845" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I845" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="846" ht="20" customHeight="1">
+      <c r="A846" s="9" t="n">
+        <v>842</v>
+      </c>
+      <c r="B846" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C846" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D846" s="9" t="n">
+        <v>1144</v>
+      </c>
+      <c r="E846" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F846" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G846" s="10" t="inlineStr">
+        <is>
+          <t>284824</t>
+        </is>
+      </c>
+      <c r="H846" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I846" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="847" ht="20" customHeight="1">
+      <c r="A847" s="9" t="n">
+        <v>843</v>
+      </c>
+      <c r="B847" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C847" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D847" s="9" t="n">
+        <v>1145</v>
+      </c>
+      <c r="E847" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F847" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G847" s="10" t="inlineStr">
+        <is>
+          <t>284825</t>
+        </is>
+      </c>
+      <c r="H847" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I847" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="848" ht="20" customHeight="1">
+      <c r="A848" s="9" t="n">
+        <v>844</v>
+      </c>
+      <c r="B848" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C848" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D848" s="9" t="n">
+        <v>1146</v>
+      </c>
+      <c r="E848" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F848" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G848" s="10" t="inlineStr">
+        <is>
+          <t>284828</t>
+        </is>
+      </c>
+      <c r="H848" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I848" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="849" ht="20" customHeight="1">
+      <c r="A849" s="9" t="n">
+        <v>845</v>
+      </c>
+      <c r="B849" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C849" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D849" s="9" t="n">
+        <v>1147</v>
+      </c>
+      <c r="E849" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F849" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G849" s="10" t="inlineStr">
+        <is>
+          <t>284826</t>
+        </is>
+      </c>
+      <c r="H849" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I849" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="850" ht="20" customHeight="1">
+      <c r="A850" s="9" t="n">
+        <v>846</v>
+      </c>
+      <c r="B850" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C850" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D850" s="9" t="n">
+        <v>1148</v>
+      </c>
+      <c r="E850" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F850" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G850" s="10" t="inlineStr">
+        <is>
+          <t>284827</t>
+        </is>
+      </c>
+      <c r="H850" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I850" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="851" ht="20" customHeight="1">
+      <c r="A851" s="9" t="n">
+        <v>847</v>
+      </c>
+      <c r="B851" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C851" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D851" s="9" t="n">
+        <v>1150</v>
+      </c>
+      <c r="E851" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F851" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G851" s="10" t="inlineStr">
+        <is>
+          <t>284424</t>
+        </is>
+      </c>
+      <c r="H851" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I851" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="852" ht="20" customHeight="1">
+      <c r="A852" s="9" t="n">
+        <v>848</v>
+      </c>
+      <c r="B852" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C852" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D852" s="9" t="n">
+        <v>1151</v>
+      </c>
+      <c r="E852" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F852" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G852" s="10" t="inlineStr">
+        <is>
+          <t>284423</t>
+        </is>
+      </c>
+      <c r="H852" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I852" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="853" ht="20" customHeight="1">
+      <c r="A853" s="9" t="n">
+        <v>849</v>
+      </c>
+      <c r="B853" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C853" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D853" s="9" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E853" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F853" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G853" s="10" t="inlineStr">
+        <is>
+          <t>284722</t>
+        </is>
+      </c>
+      <c r="H853" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I853" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="854" ht="20" customHeight="1">
+      <c r="A854" s="9" t="n">
+        <v>850</v>
+      </c>
+      <c r="B854" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C854" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D854" s="9" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E854" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F854" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G854" s="10" t="inlineStr">
+        <is>
+          <t>284284</t>
+        </is>
+      </c>
+      <c r="H854" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I854" s="11" t="inlineStr">
+        <is>
+          <t>grade 17 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (850 BAL)</t>
+        </is>
+      </c>
+      <c r="B855" s="4" t="n"/>
+      <c r="C855" s="4" t="n"/>
+      <c r="D855" s="4" t="n"/>
+      <c r="E855" s="4" t="n"/>
+      <c r="F855" s="4" t="n"/>
+      <c r="G855" s="4" t="n"/>
+      <c r="H855" s="4">
+        <f>SUM(H5:H854)</f>
         <v/>
       </c>
-      <c r="I784" s="4" t="inlineStr">
+      <c r="I855" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -45137,7 +49184,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A784:G784"/>
+    <mergeCell ref="A855:G855"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -45150,7 +49197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -45909,36 +49956,65 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>3014</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>1047 - 1154</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4">
-        <f>SUM(D5:D28)</f>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4">
+        <f>SUM(D5:D29)</f>
         <v/>
       </c>
-      <c r="E29" s="4">
-        <f>SUM(E5:E28)</f>
+      <c r="E30" s="4">
+        <f>SUM(E5:E29)</f>
         <v/>
       </c>
-      <c r="F29" s="4">
-        <f>AVERAGE(F5:F28)</f>
+      <c r="F30" s="4">
+        <f>AVERAGE(F5:F29)</f>
         <v/>
       </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>3 - 1046</t>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>3 - 1154</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A30:C30"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix nomor barkot tgl 17 & 19 September (No Gud 1120 & 1208), update rekap excel, seed_data, supabase schema, dan bump cache version v=6.2
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -17046,7 +17046,7 @@
       </c>
       <c r="D827" s="6" t="inlineStr">
         <is>
-          <t>284922</t>
+          <t>282922</t>
         </is>
       </c>
       <c r="E827" s="5" t="n">
@@ -18626,7 +18626,7 @@
       </c>
       <c r="D906" s="6" t="inlineStr">
         <is>
-          <t>374179</t>
+          <t>374139</t>
         </is>
       </c>
       <c r="E906" s="5" t="n">
@@ -49388,7 +49388,7 @@
       </c>
       <c r="G827" s="10" t="inlineStr">
         <is>
-          <t>284922</t>
+          <t>282922</t>
         </is>
       </c>
       <c r="H827" s="9" t="n">
@@ -52311,7 +52311,7 @@
       </c>
       <c r="G906" s="10" t="inlineStr">
         <is>
-          <t>374179</t>
+          <t>374139</t>
         </is>
       </c>
       <c r="H906" s="9" t="n">

</xml_diff>

<commit_message>
feat: tambah data bal tembakau tanggal 21 September 2026 (68 bal, No Gud 1283-1374), update rekap excel, dan bump cache version v=6.4
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F944"/>
+  <dimension ref="A1:F1003"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19374,20 +19374,1200 @@
       </c>
       <c r="F943" s="5" t="n"/>
     </row>
-    <row r="944" ht="22" customHeight="1">
-      <c r="A944" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (939 BAL)</t>
-        </is>
-      </c>
-      <c r="B944" s="4" t="n"/>
-      <c r="C944" s="4" t="n"/>
-      <c r="D944" s="4" t="n"/>
-      <c r="E944" s="4">
-        <f>SUM(E5:E943)</f>
+    <row r="944" ht="20.25" customHeight="1">
+      <c r="A944" s="5" t="n">
+        <v>1283</v>
+      </c>
+      <c r="B944" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C944" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D944" s="6" t="inlineStr">
+        <is>
+          <t>375596</t>
+        </is>
+      </c>
+      <c r="E944" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F944" s="5" t="n"/>
+    </row>
+    <row r="945" ht="20.25" customHeight="1">
+      <c r="A945" s="5" t="n">
+        <v>1284</v>
+      </c>
+      <c r="B945" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C945" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D945" s="6" t="inlineStr">
+        <is>
+          <t>375597</t>
+        </is>
+      </c>
+      <c r="E945" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F945" s="5" t="n"/>
+    </row>
+    <row r="946" ht="20.25" customHeight="1">
+      <c r="A946" s="5" t="n">
+        <v>1285</v>
+      </c>
+      <c r="B946" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C946" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D946" s="6" t="inlineStr">
+        <is>
+          <t>375595</t>
+        </is>
+      </c>
+      <c r="E946" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F946" s="5" t="n"/>
+    </row>
+    <row r="947" ht="20.25" customHeight="1">
+      <c r="A947" s="5" t="n">
+        <v>1286</v>
+      </c>
+      <c r="B947" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C947" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D947" s="6" t="inlineStr">
+        <is>
+          <t>375808</t>
+        </is>
+      </c>
+      <c r="E947" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F947" s="5" t="n"/>
+    </row>
+    <row r="948" ht="20.25" customHeight="1">
+      <c r="A948" s="5" t="n">
+        <v>1287</v>
+      </c>
+      <c r="B948" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C948" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D948" s="6" t="inlineStr">
+        <is>
+          <t>375622</t>
+        </is>
+      </c>
+      <c r="E948" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F948" s="5" t="n"/>
+    </row>
+    <row r="949" ht="20.25" customHeight="1">
+      <c r="A949" s="5" t="n">
+        <v>1288</v>
+      </c>
+      <c r="B949" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C949" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D949" s="6" t="inlineStr">
+        <is>
+          <t>375809</t>
+        </is>
+      </c>
+      <c r="E949" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F949" s="5" t="n"/>
+    </row>
+    <row r="950" ht="20.25" customHeight="1">
+      <c r="A950" s="5" t="n">
+        <v>1289</v>
+      </c>
+      <c r="B950" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C950" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D950" s="6" t="inlineStr">
+        <is>
+          <t>375763</t>
+        </is>
+      </c>
+      <c r="E950" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F950" s="5" t="n"/>
+    </row>
+    <row r="951" ht="20.25" customHeight="1">
+      <c r="A951" s="5" t="n">
+        <v>1290</v>
+      </c>
+      <c r="B951" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C951" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D951" s="6" t="inlineStr">
+        <is>
+          <t>375422</t>
+        </is>
+      </c>
+      <c r="E951" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F951" s="5" t="n"/>
+    </row>
+    <row r="952" ht="20.25" customHeight="1">
+      <c r="A952" s="5" t="n">
+        <v>1291</v>
+      </c>
+      <c r="B952" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C952" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D952" s="6" t="inlineStr">
+        <is>
+          <t>375423</t>
+        </is>
+      </c>
+      <c r="E952" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F952" s="5" t="n"/>
+    </row>
+    <row r="953" ht="20.25" customHeight="1">
+      <c r="A953" s="5" t="n">
+        <v>1292</v>
+      </c>
+      <c r="B953" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C953" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D953" s="6" t="inlineStr">
+        <is>
+          <t>375421</t>
+        </is>
+      </c>
+      <c r="E953" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F953" s="5" t="n"/>
+    </row>
+    <row r="954" ht="20.25" customHeight="1">
+      <c r="A954" s="5" t="n">
+        <v>1293</v>
+      </c>
+      <c r="B954" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C954" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D954" s="6" t="inlineStr">
+        <is>
+          <t>375424</t>
+        </is>
+      </c>
+      <c r="E954" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F954" s="5" t="n"/>
+    </row>
+    <row r="955" ht="20.25" customHeight="1">
+      <c r="A955" s="5" t="n">
+        <v>1294</v>
+      </c>
+      <c r="B955" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C955" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D955" s="6" t="inlineStr">
+        <is>
+          <t>375811</t>
+        </is>
+      </c>
+      <c r="E955" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F955" s="5" t="n"/>
+    </row>
+    <row r="956" ht="20.25" customHeight="1">
+      <c r="A956" s="5" t="n">
+        <v>1295</v>
+      </c>
+      <c r="B956" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C956" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D956" s="6" t="inlineStr">
+        <is>
+          <t>375810</t>
+        </is>
+      </c>
+      <c r="E956" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F956" s="5" t="n"/>
+    </row>
+    <row r="957" ht="20.25" customHeight="1">
+      <c r="A957" s="5" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B957" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C957" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D957" s="6" t="inlineStr">
+        <is>
+          <t>375852</t>
+        </is>
+      </c>
+      <c r="E957" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F957" s="5" t="n"/>
+    </row>
+    <row r="958" ht="20.25" customHeight="1">
+      <c r="A958" s="5" t="n">
+        <v>1304</v>
+      </c>
+      <c r="B958" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C958" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D958" s="6" t="inlineStr">
+        <is>
+          <t>375600</t>
+        </is>
+      </c>
+      <c r="E958" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F958" s="5" t="n"/>
+    </row>
+    <row r="959" ht="20.25" customHeight="1">
+      <c r="A959" s="5" t="n">
+        <v>1305</v>
+      </c>
+      <c r="B959" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="C959" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D959" s="6" t="inlineStr">
+        <is>
+          <t>375854</t>
+        </is>
+      </c>
+      <c r="E959" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F959" s="5" t="n"/>
+    </row>
+    <row r="960" ht="20.25" customHeight="1">
+      <c r="A960" s="5" t="n">
+        <v>1306</v>
+      </c>
+      <c r="B960" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C960" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D960" s="6" t="inlineStr">
+        <is>
+          <t>375599</t>
+        </is>
+      </c>
+      <c r="E960" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F960" s="5" t="n"/>
+    </row>
+    <row r="961" ht="20.25" customHeight="1">
+      <c r="A961" s="5" t="n">
+        <v>1307</v>
+      </c>
+      <c r="B961" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C961" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D961" s="6" t="inlineStr">
+        <is>
+          <t>375598</t>
+        </is>
+      </c>
+      <c r="E961" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F961" s="5" t="n"/>
+    </row>
+    <row r="962" ht="20.25" customHeight="1">
+      <c r="A962" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="B962" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C962" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D962" s="6" t="inlineStr">
+        <is>
+          <t>375851</t>
+        </is>
+      </c>
+      <c r="E962" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F962" s="5" t="n"/>
+    </row>
+    <row r="963" ht="20.25" customHeight="1">
+      <c r="A963" s="5" t="n">
+        <v>1309</v>
+      </c>
+      <c r="B963" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C963" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D963" s="6" t="inlineStr">
+        <is>
+          <t>375853</t>
+        </is>
+      </c>
+      <c r="E963" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F963" s="5" t="n"/>
+    </row>
+    <row r="964" ht="20.25" customHeight="1">
+      <c r="A964" s="5" t="n">
+        <v>1310</v>
+      </c>
+      <c r="B964" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C964" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D964" s="6" t="inlineStr">
+        <is>
+          <t>375637</t>
+        </is>
+      </c>
+      <c r="E964" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F964" s="5" t="n"/>
+    </row>
+    <row r="965" ht="20.25" customHeight="1">
+      <c r="A965" s="5" t="n">
+        <v>1311</v>
+      </c>
+      <c r="B965" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C965" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D965" s="6" t="inlineStr">
+        <is>
+          <t>375638</t>
+        </is>
+      </c>
+      <c r="E965" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F965" s="5" t="n"/>
+    </row>
+    <row r="966" ht="20.25" customHeight="1">
+      <c r="A966" s="5" t="n">
+        <v>1314</v>
+      </c>
+      <c r="B966" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C966" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D966" s="6" t="inlineStr">
+        <is>
+          <t>375639</t>
+        </is>
+      </c>
+      <c r="E966" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F966" s="5" t="n"/>
+    </row>
+    <row r="967" ht="20.25" customHeight="1">
+      <c r="A967" s="5" t="n">
+        <v>1315</v>
+      </c>
+      <c r="B967" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C967" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D967" s="6" t="inlineStr">
+        <is>
+          <t>375806</t>
+        </is>
+      </c>
+      <c r="E967" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F967" s="5" t="n"/>
+    </row>
+    <row r="968" ht="20.25" customHeight="1">
+      <c r="A968" s="5" t="n">
+        <v>1316</v>
+      </c>
+      <c r="B968" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C968" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D968" s="6" t="inlineStr">
+        <is>
+          <t>375812</t>
+        </is>
+      </c>
+      <c r="E968" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F968" s="5" t="n"/>
+    </row>
+    <row r="969" ht="20.25" customHeight="1">
+      <c r="A969" s="5" t="n">
+        <v>1317</v>
+      </c>
+      <c r="B969" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C969" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D969" s="6" t="inlineStr">
+        <is>
+          <t>375814</t>
+        </is>
+      </c>
+      <c r="E969" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F969" s="5" t="n"/>
+    </row>
+    <row r="970" ht="20.25" customHeight="1">
+      <c r="A970" s="5" t="n">
+        <v>1318</v>
+      </c>
+      <c r="B970" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C970" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D970" s="6" t="inlineStr">
+        <is>
+          <t>375813</t>
+        </is>
+      </c>
+      <c r="E970" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F970" s="5" t="n"/>
+    </row>
+    <row r="971" ht="20.25" customHeight="1">
+      <c r="A971" s="5" t="n">
+        <v>1319</v>
+      </c>
+      <c r="B971" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C971" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D971" s="6" t="inlineStr">
+        <is>
+          <t>375306</t>
+        </is>
+      </c>
+      <c r="E971" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F971" s="5" t="n"/>
+    </row>
+    <row r="972" ht="20.25" customHeight="1">
+      <c r="A972" s="5" t="n">
+        <v>1320</v>
+      </c>
+      <c r="B972" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C972" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D972" s="6" t="inlineStr">
+        <is>
+          <t>375805</t>
+        </is>
+      </c>
+      <c r="E972" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F972" s="5" t="n"/>
+    </row>
+    <row r="973" ht="20.25" customHeight="1">
+      <c r="A973" s="5" t="n">
+        <v>1321</v>
+      </c>
+      <c r="B973" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C973" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D973" s="6" t="inlineStr">
+        <is>
+          <t>375807</t>
+        </is>
+      </c>
+      <c r="E973" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F973" s="5" t="n"/>
+    </row>
+    <row r="974" ht="20.25" customHeight="1">
+      <c r="A974" s="5" t="n">
+        <v>1322</v>
+      </c>
+      <c r="B974" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C974" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D974" s="6" t="inlineStr">
+        <is>
+          <t>375307</t>
+        </is>
+      </c>
+      <c r="E974" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F974" s="5" t="n"/>
+    </row>
+    <row r="975" ht="20.25" customHeight="1">
+      <c r="A975" s="5" t="n">
+        <v>1328</v>
+      </c>
+      <c r="B975" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C975" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D975" s="6" t="inlineStr">
+        <is>
+          <t>375120</t>
+        </is>
+      </c>
+      <c r="E975" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F975" s="5" t="n"/>
+    </row>
+    <row r="976" ht="20.25" customHeight="1">
+      <c r="A976" s="5" t="n">
+        <v>1329</v>
+      </c>
+      <c r="B976" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C976" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D976" s="6" t="inlineStr">
+        <is>
+          <t>375626</t>
+        </is>
+      </c>
+      <c r="E976" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F976" s="5" t="n"/>
+    </row>
+    <row r="977" ht="20.25" customHeight="1">
+      <c r="A977" s="5" t="n">
+        <v>1330</v>
+      </c>
+      <c r="B977" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C977" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D977" s="6" t="inlineStr">
+        <is>
+          <t>375628</t>
+        </is>
+      </c>
+      <c r="E977" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F977" s="5" t="n"/>
+    </row>
+    <row r="978" ht="20.25" customHeight="1">
+      <c r="A978" s="5" t="n">
+        <v>1331</v>
+      </c>
+      <c r="B978" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C978" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D978" s="6" t="inlineStr">
+        <is>
+          <t>375625</t>
+        </is>
+      </c>
+      <c r="E978" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F978" s="5" t="n"/>
+    </row>
+    <row r="979" ht="20.25" customHeight="1">
+      <c r="A979" s="5" t="n">
+        <v>1333</v>
+      </c>
+      <c r="B979" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C979" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D979" s="6" t="inlineStr">
+        <is>
+          <t>375629</t>
+        </is>
+      </c>
+      <c r="E979" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F979" s="5" t="n"/>
+    </row>
+    <row r="980" ht="20.25" customHeight="1">
+      <c r="A980" s="5" t="n">
+        <v>1338</v>
+      </c>
+      <c r="B980" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C980" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D980" s="6" t="inlineStr">
+        <is>
+          <t>375630</t>
+        </is>
+      </c>
+      <c r="E980" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F980" s="5" t="n"/>
+    </row>
+    <row r="981" ht="20.25" customHeight="1">
+      <c r="A981" s="5" t="n">
+        <v>1339</v>
+      </c>
+      <c r="B981" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C981" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D981" s="6" t="inlineStr">
+        <is>
+          <t>375631</t>
+        </is>
+      </c>
+      <c r="E981" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F981" s="5" t="n"/>
+    </row>
+    <row r="982" ht="20.25" customHeight="1">
+      <c r="A982" s="5" t="n">
+        <v>1341</v>
+      </c>
+      <c r="B982" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C982" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D982" s="6" t="inlineStr">
+        <is>
+          <t>375627</t>
+        </is>
+      </c>
+      <c r="E982" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F982" s="5" t="n"/>
+    </row>
+    <row r="983" ht="20.25" customHeight="1">
+      <c r="A983" s="5" t="n">
+        <v>1346</v>
+      </c>
+      <c r="B983" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C983" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D983" s="6" t="inlineStr">
+        <is>
+          <t>375632</t>
+        </is>
+      </c>
+      <c r="E983" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F983" s="5" t="n"/>
+    </row>
+    <row r="984" ht="20.25" customHeight="1">
+      <c r="A984" s="5" t="n">
+        <v>1352</v>
+      </c>
+      <c r="B984" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C984" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D984" s="6" t="inlineStr">
+        <is>
+          <t>375633</t>
+        </is>
+      </c>
+      <c r="E984" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F984" s="5" t="n"/>
+    </row>
+    <row r="985" ht="20.25" customHeight="1">
+      <c r="A985" s="5" t="n">
+        <v>1353</v>
+      </c>
+      <c r="B985" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C985" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D985" s="6" t="inlineStr">
+        <is>
+          <t>375122</t>
+        </is>
+      </c>
+      <c r="E985" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F985" s="5" t="n"/>
+    </row>
+    <row r="986" ht="20.25" customHeight="1">
+      <c r="A986" s="5" t="n">
+        <v>1354</v>
+      </c>
+      <c r="B986" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C986" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D986" s="6" t="inlineStr">
+        <is>
+          <t>375634</t>
+        </is>
+      </c>
+      <c r="E986" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F986" s="5" t="n"/>
+    </row>
+    <row r="987" ht="20.25" customHeight="1">
+      <c r="A987" s="5" t="n">
+        <v>1355</v>
+      </c>
+      <c r="B987" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C987" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D987" s="6" t="inlineStr">
+        <is>
+          <t>375121</t>
+        </is>
+      </c>
+      <c r="E987" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F987" s="5" t="n"/>
+    </row>
+    <row r="988" ht="20.25" customHeight="1">
+      <c r="A988" s="5" t="n">
+        <v>1356</v>
+      </c>
+      <c r="B988" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C988" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D988" s="6" t="inlineStr">
+        <is>
+          <t>375123</t>
+        </is>
+      </c>
+      <c r="E988" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F988" s="5" t="n"/>
+    </row>
+    <row r="989" ht="20.25" customHeight="1">
+      <c r="A989" s="5" t="n">
+        <v>1358</v>
+      </c>
+      <c r="B989" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C989" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D989" s="6" t="inlineStr">
+        <is>
+          <t>375124</t>
+        </is>
+      </c>
+      <c r="E989" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F989" s="5" t="n"/>
+    </row>
+    <row r="990" ht="20.25" customHeight="1">
+      <c r="A990" s="5" t="n">
+        <v>1359</v>
+      </c>
+      <c r="B990" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C990" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D990" s="6" t="inlineStr">
+        <is>
+          <t>375130</t>
+        </is>
+      </c>
+      <c r="E990" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F990" s="5" t="n"/>
+    </row>
+    <row r="991" ht="20.25" customHeight="1">
+      <c r="A991" s="5" t="n">
+        <v>1360</v>
+      </c>
+      <c r="B991" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C991" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D991" s="6" t="inlineStr">
+        <is>
+          <t>375125</t>
+        </is>
+      </c>
+      <c r="E991" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F991" s="5" t="n"/>
+    </row>
+    <row r="992" ht="20.25" customHeight="1">
+      <c r="A992" s="5" t="n">
+        <v>1361</v>
+      </c>
+      <c r="B992" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C992" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D992" s="6" t="inlineStr">
+        <is>
+          <t>375126</t>
+        </is>
+      </c>
+      <c r="E992" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F992" s="5" t="n"/>
+    </row>
+    <row r="993" ht="20.25" customHeight="1">
+      <c r="A993" s="5" t="n">
+        <v>1362</v>
+      </c>
+      <c r="B993" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C993" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D993" s="6" t="inlineStr">
+        <is>
+          <t>375129</t>
+        </is>
+      </c>
+      <c r="E993" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F993" s="5" t="n"/>
+    </row>
+    <row r="994" ht="20.25" customHeight="1">
+      <c r="A994" s="5" t="n">
+        <v>1363</v>
+      </c>
+      <c r="B994" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C994" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D994" s="6" t="inlineStr">
+        <is>
+          <t>375127</t>
+        </is>
+      </c>
+      <c r="E994" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F994" s="5" t="n"/>
+    </row>
+    <row r="995" ht="20.25" customHeight="1">
+      <c r="A995" s="5" t="n">
+        <v>1364</v>
+      </c>
+      <c r="B995" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C995" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D995" s="6" t="inlineStr">
+        <is>
+          <t>375636</t>
+        </is>
+      </c>
+      <c r="E995" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F995" s="5" t="n"/>
+    </row>
+    <row r="996" ht="20.25" customHeight="1">
+      <c r="A996" s="5" t="n">
+        <v>1365</v>
+      </c>
+      <c r="B996" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C996" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D996" s="6" t="inlineStr">
+        <is>
+          <t>375128</t>
+        </is>
+      </c>
+      <c r="E996" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F996" s="5" t="n"/>
+    </row>
+    <row r="997" ht="20.25" customHeight="1">
+      <c r="A997" s="5" t="n">
+        <v>1366</v>
+      </c>
+      <c r="B997" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C997" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D997" s="6" t="inlineStr">
+        <is>
+          <t>375635</t>
+        </is>
+      </c>
+      <c r="E997" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F997" s="5" t="n"/>
+    </row>
+    <row r="998" ht="20.25" customHeight="1">
+      <c r="A998" s="5" t="n">
+        <v>1370</v>
+      </c>
+      <c r="B998" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C998" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D998" s="6" t="inlineStr">
+        <is>
+          <t>375132</t>
+        </is>
+      </c>
+      <c r="E998" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F998" s="5" t="n"/>
+    </row>
+    <row r="999" ht="20.25" customHeight="1">
+      <c r="A999" s="5" t="n">
+        <v>1371</v>
+      </c>
+      <c r="B999" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C999" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D999" s="6" t="inlineStr">
+        <is>
+          <t>375131</t>
+        </is>
+      </c>
+      <c r="E999" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F999" s="5" t="n"/>
+    </row>
+    <row r="1000" ht="20.25" customHeight="1">
+      <c r="A1000" s="5" t="n">
+        <v>1372</v>
+      </c>
+      <c r="B1000" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1000" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1000" s="6" t="inlineStr">
+        <is>
+          <t>375133</t>
+        </is>
+      </c>
+      <c r="E1000" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F1000" s="5" t="n"/>
+    </row>
+    <row r="1001" ht="20.25" customHeight="1">
+      <c r="A1001" s="5" t="n">
+        <v>1373</v>
+      </c>
+      <c r="B1001" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1001" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1001" s="6" t="inlineStr">
+        <is>
+          <t>375623</t>
+        </is>
+      </c>
+      <c r="E1001" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F1001" s="5" t="n"/>
+    </row>
+    <row r="1002" ht="20.25" customHeight="1">
+      <c r="A1002" s="5" t="n">
+        <v>1374</v>
+      </c>
+      <c r="B1002" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1002" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D1002" s="6" t="inlineStr">
+        <is>
+          <t>375624</t>
+        </is>
+      </c>
+      <c r="E1002" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F1002" s="5" t="n"/>
+    </row>
+    <row r="1003" ht="22" customHeight="1">
+      <c r="A1003" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (998 BAL)</t>
+        </is>
+      </c>
+      <c r="B1003" s="4" t="n"/>
+      <c r="C1003" s="4" t="n"/>
+      <c r="D1003" s="4" t="n"/>
+      <c r="E1003" s="4">
+        <f>SUM(E5:E1002)</f>
         <v/>
       </c>
-      <c r="F944" s="4" t="inlineStr">
+      <c r="F1003" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -19396,10 +20576,10 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A944:D944"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="A1003:D1003"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:C4"/>
@@ -19414,7 +20594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I944"/>
+  <dimension ref="A1:I1003"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19438,7 +20618,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 939 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 998 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -54232,23 +55412,2206 @@
         </is>
       </c>
     </row>
-    <row r="944">
-      <c r="A944" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (939 BAL)</t>
-        </is>
-      </c>
-      <c r="B944" s="4" t="n"/>
-      <c r="C944" s="4" t="n"/>
-      <c r="D944" s="4" t="n"/>
-      <c r="E944" s="4" t="n"/>
-      <c r="F944" s="4" t="n"/>
-      <c r="G944" s="4" t="n"/>
-      <c r="H944" s="4">
-        <f>SUM(H5:H943)</f>
+    <row r="944" ht="20" customHeight="1">
+      <c r="A944" s="9" t="n">
+        <v>940</v>
+      </c>
+      <c r="B944" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C944" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D944" s="9" t="n">
+        <v>1283</v>
+      </c>
+      <c r="E944" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F944" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G944" s="10" t="inlineStr">
+        <is>
+          <t>375596</t>
+        </is>
+      </c>
+      <c r="H944" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I944" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="945" ht="20" customHeight="1">
+      <c r="A945" s="9" t="n">
+        <v>941</v>
+      </c>
+      <c r="B945" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C945" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D945" s="9" t="n">
+        <v>1284</v>
+      </c>
+      <c r="E945" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F945" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G945" s="10" t="inlineStr">
+        <is>
+          <t>375597</t>
+        </is>
+      </c>
+      <c r="H945" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I945" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="946" ht="20" customHeight="1">
+      <c r="A946" s="9" t="n">
+        <v>942</v>
+      </c>
+      <c r="B946" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C946" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D946" s="9" t="n">
+        <v>1285</v>
+      </c>
+      <c r="E946" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F946" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G946" s="10" t="inlineStr">
+        <is>
+          <t>375595</t>
+        </is>
+      </c>
+      <c r="H946" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I946" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="947" ht="20" customHeight="1">
+      <c r="A947" s="9" t="n">
+        <v>943</v>
+      </c>
+      <c r="B947" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C947" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D947" s="9" t="n">
+        <v>1286</v>
+      </c>
+      <c r="E947" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F947" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G947" s="10" t="inlineStr">
+        <is>
+          <t>375808</t>
+        </is>
+      </c>
+      <c r="H947" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I947" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="948" ht="20" customHeight="1">
+      <c r="A948" s="9" t="n">
+        <v>944</v>
+      </c>
+      <c r="B948" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C948" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D948" s="9" t="n">
+        <v>1287</v>
+      </c>
+      <c r="E948" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F948" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G948" s="10" t="inlineStr">
+        <is>
+          <t>375622</t>
+        </is>
+      </c>
+      <c r="H948" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I948" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="949" ht="20" customHeight="1">
+      <c r="A949" s="9" t="n">
+        <v>945</v>
+      </c>
+      <c r="B949" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C949" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D949" s="9" t="n">
+        <v>1288</v>
+      </c>
+      <c r="E949" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F949" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G949" s="10" t="inlineStr">
+        <is>
+          <t>375809</t>
+        </is>
+      </c>
+      <c r="H949" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I949" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="950" ht="20" customHeight="1">
+      <c r="A950" s="9" t="n">
+        <v>946</v>
+      </c>
+      <c r="B950" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C950" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D950" s="9" t="n">
+        <v>1289</v>
+      </c>
+      <c r="E950" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F950" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G950" s="10" t="inlineStr">
+        <is>
+          <t>375763</t>
+        </is>
+      </c>
+      <c r="H950" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I950" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="951" ht="20" customHeight="1">
+      <c r="A951" s="9" t="n">
+        <v>947</v>
+      </c>
+      <c r="B951" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C951" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D951" s="9" t="n">
+        <v>1290</v>
+      </c>
+      <c r="E951" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F951" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G951" s="10" t="inlineStr">
+        <is>
+          <t>375422</t>
+        </is>
+      </c>
+      <c r="H951" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I951" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="952" ht="20" customHeight="1">
+      <c r="A952" s="9" t="n">
+        <v>948</v>
+      </c>
+      <c r="B952" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C952" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D952" s="9" t="n">
+        <v>1291</v>
+      </c>
+      <c r="E952" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F952" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G952" s="10" t="inlineStr">
+        <is>
+          <t>375423</t>
+        </is>
+      </c>
+      <c r="H952" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I952" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="953" ht="20" customHeight="1">
+      <c r="A953" s="9" t="n">
+        <v>949</v>
+      </c>
+      <c r="B953" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C953" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D953" s="9" t="n">
+        <v>1292</v>
+      </c>
+      <c r="E953" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F953" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G953" s="10" t="inlineStr">
+        <is>
+          <t>375421</t>
+        </is>
+      </c>
+      <c r="H953" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I953" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="954" ht="20" customHeight="1">
+      <c r="A954" s="9" t="n">
+        <v>950</v>
+      </c>
+      <c r="B954" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C954" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D954" s="9" t="n">
+        <v>1293</v>
+      </c>
+      <c r="E954" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F954" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G954" s="10" t="inlineStr">
+        <is>
+          <t>375424</t>
+        </is>
+      </c>
+      <c r="H954" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I954" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="955" ht="20" customHeight="1">
+      <c r="A955" s="9" t="n">
+        <v>951</v>
+      </c>
+      <c r="B955" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C955" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D955" s="9" t="n">
+        <v>1294</v>
+      </c>
+      <c r="E955" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F955" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G955" s="10" t="inlineStr">
+        <is>
+          <t>375811</t>
+        </is>
+      </c>
+      <c r="H955" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I955" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="956" ht="20" customHeight="1">
+      <c r="A956" s="9" t="n">
+        <v>952</v>
+      </c>
+      <c r="B956" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C956" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D956" s="9" t="n">
+        <v>1295</v>
+      </c>
+      <c r="E956" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F956" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G956" s="10" t="inlineStr">
+        <is>
+          <t>375810</t>
+        </is>
+      </c>
+      <c r="H956" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I956" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="957" ht="20" customHeight="1">
+      <c r="A957" s="9" t="n">
+        <v>953</v>
+      </c>
+      <c r="B957" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C957" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D957" s="9" t="n">
+        <v>1303</v>
+      </c>
+      <c r="E957" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F957" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G957" s="10" t="inlineStr">
+        <is>
+          <t>375852</t>
+        </is>
+      </c>
+      <c r="H957" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I957" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="958" ht="20" customHeight="1">
+      <c r="A958" s="9" t="n">
+        <v>954</v>
+      </c>
+      <c r="B958" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C958" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D958" s="9" t="n">
+        <v>1304</v>
+      </c>
+      <c r="E958" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F958" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G958" s="10" t="inlineStr">
+        <is>
+          <t>375600</t>
+        </is>
+      </c>
+      <c r="H958" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I958" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="959" ht="20" customHeight="1">
+      <c r="A959" s="9" t="n">
+        <v>955</v>
+      </c>
+      <c r="B959" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C959" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D959" s="9" t="n">
+        <v>1305</v>
+      </c>
+      <c r="E959" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F959" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="G959" s="10" t="inlineStr">
+        <is>
+          <t>375854</t>
+        </is>
+      </c>
+      <c r="H959" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I959" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="960" ht="20" customHeight="1">
+      <c r="A960" s="9" t="n">
+        <v>956</v>
+      </c>
+      <c r="B960" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C960" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D960" s="9" t="n">
+        <v>1306</v>
+      </c>
+      <c r="E960" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F960" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G960" s="10" t="inlineStr">
+        <is>
+          <t>375599</t>
+        </is>
+      </c>
+      <c r="H960" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I960" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="961" ht="20" customHeight="1">
+      <c r="A961" s="9" t="n">
+        <v>957</v>
+      </c>
+      <c r="B961" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C961" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D961" s="9" t="n">
+        <v>1307</v>
+      </c>
+      <c r="E961" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F961" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G961" s="10" t="inlineStr">
+        <is>
+          <t>375598</t>
+        </is>
+      </c>
+      <c r="H961" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I961" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="962" ht="20" customHeight="1">
+      <c r="A962" s="9" t="n">
+        <v>958</v>
+      </c>
+      <c r="B962" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C962" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D962" s="9" t="n">
+        <v>1308</v>
+      </c>
+      <c r="E962" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F962" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G962" s="10" t="inlineStr">
+        <is>
+          <t>375851</t>
+        </is>
+      </c>
+      <c r="H962" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I962" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="963" ht="20" customHeight="1">
+      <c r="A963" s="9" t="n">
+        <v>959</v>
+      </c>
+      <c r="B963" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C963" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D963" s="9" t="n">
+        <v>1309</v>
+      </c>
+      <c r="E963" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F963" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G963" s="10" t="inlineStr">
+        <is>
+          <t>375853</t>
+        </is>
+      </c>
+      <c r="H963" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I963" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="964" ht="20" customHeight="1">
+      <c r="A964" s="9" t="n">
+        <v>960</v>
+      </c>
+      <c r="B964" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C964" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D964" s="9" t="n">
+        <v>1310</v>
+      </c>
+      <c r="E964" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F964" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G964" s="10" t="inlineStr">
+        <is>
+          <t>375637</t>
+        </is>
+      </c>
+      <c r="H964" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I964" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="965" ht="20" customHeight="1">
+      <c r="A965" s="9" t="n">
+        <v>961</v>
+      </c>
+      <c r="B965" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C965" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D965" s="9" t="n">
+        <v>1311</v>
+      </c>
+      <c r="E965" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F965" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G965" s="10" t="inlineStr">
+        <is>
+          <t>375638</t>
+        </is>
+      </c>
+      <c r="H965" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I965" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="966" ht="20" customHeight="1">
+      <c r="A966" s="9" t="n">
+        <v>962</v>
+      </c>
+      <c r="B966" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C966" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D966" s="9" t="n">
+        <v>1314</v>
+      </c>
+      <c r="E966" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F966" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G966" s="10" t="inlineStr">
+        <is>
+          <t>375639</t>
+        </is>
+      </c>
+      <c r="H966" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I966" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="967" ht="20" customHeight="1">
+      <c r="A967" s="9" t="n">
+        <v>963</v>
+      </c>
+      <c r="B967" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C967" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D967" s="9" t="n">
+        <v>1315</v>
+      </c>
+      <c r="E967" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F967" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G967" s="10" t="inlineStr">
+        <is>
+          <t>375806</t>
+        </is>
+      </c>
+      <c r="H967" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I967" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="968" ht="20" customHeight="1">
+      <c r="A968" s="9" t="n">
+        <v>964</v>
+      </c>
+      <c r="B968" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C968" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D968" s="9" t="n">
+        <v>1316</v>
+      </c>
+      <c r="E968" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F968" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G968" s="10" t="inlineStr">
+        <is>
+          <t>375812</t>
+        </is>
+      </c>
+      <c r="H968" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I968" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="969" ht="20" customHeight="1">
+      <c r="A969" s="9" t="n">
+        <v>965</v>
+      </c>
+      <c r="B969" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C969" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D969" s="9" t="n">
+        <v>1317</v>
+      </c>
+      <c r="E969" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F969" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G969" s="10" t="inlineStr">
+        <is>
+          <t>375814</t>
+        </is>
+      </c>
+      <c r="H969" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I969" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="970" ht="20" customHeight="1">
+      <c r="A970" s="9" t="n">
+        <v>966</v>
+      </c>
+      <c r="B970" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C970" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D970" s="9" t="n">
+        <v>1318</v>
+      </c>
+      <c r="E970" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F970" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G970" s="10" t="inlineStr">
+        <is>
+          <t>375813</t>
+        </is>
+      </c>
+      <c r="H970" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I970" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="971" ht="20" customHeight="1">
+      <c r="A971" s="9" t="n">
+        <v>967</v>
+      </c>
+      <c r="B971" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C971" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D971" s="9" t="n">
+        <v>1319</v>
+      </c>
+      <c r="E971" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F971" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G971" s="10" t="inlineStr">
+        <is>
+          <t>375306</t>
+        </is>
+      </c>
+      <c r="H971" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I971" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="972" ht="20" customHeight="1">
+      <c r="A972" s="9" t="n">
+        <v>968</v>
+      </c>
+      <c r="B972" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C972" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D972" s="9" t="n">
+        <v>1320</v>
+      </c>
+      <c r="E972" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F972" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G972" s="10" t="inlineStr">
+        <is>
+          <t>375805</t>
+        </is>
+      </c>
+      <c r="H972" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I972" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="973" ht="20" customHeight="1">
+      <c r="A973" s="9" t="n">
+        <v>969</v>
+      </c>
+      <c r="B973" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C973" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D973" s="9" t="n">
+        <v>1321</v>
+      </c>
+      <c r="E973" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F973" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G973" s="10" t="inlineStr">
+        <is>
+          <t>375807</t>
+        </is>
+      </c>
+      <c r="H973" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I973" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="974" ht="20" customHeight="1">
+      <c r="A974" s="9" t="n">
+        <v>970</v>
+      </c>
+      <c r="B974" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C974" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D974" s="9" t="n">
+        <v>1322</v>
+      </c>
+      <c r="E974" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F974" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G974" s="10" t="inlineStr">
+        <is>
+          <t>375307</t>
+        </is>
+      </c>
+      <c r="H974" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I974" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="975" ht="20" customHeight="1">
+      <c r="A975" s="9" t="n">
+        <v>971</v>
+      </c>
+      <c r="B975" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C975" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D975" s="9" t="n">
+        <v>1328</v>
+      </c>
+      <c r="E975" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F975" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G975" s="10" t="inlineStr">
+        <is>
+          <t>375120</t>
+        </is>
+      </c>
+      <c r="H975" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I975" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="976" ht="20" customHeight="1">
+      <c r="A976" s="9" t="n">
+        <v>972</v>
+      </c>
+      <c r="B976" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C976" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D976" s="9" t="n">
+        <v>1329</v>
+      </c>
+      <c r="E976" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F976" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G976" s="10" t="inlineStr">
+        <is>
+          <t>375626</t>
+        </is>
+      </c>
+      <c r="H976" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I976" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="977" ht="20" customHeight="1">
+      <c r="A977" s="9" t="n">
+        <v>973</v>
+      </c>
+      <c r="B977" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C977" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D977" s="9" t="n">
+        <v>1330</v>
+      </c>
+      <c r="E977" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F977" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G977" s="10" t="inlineStr">
+        <is>
+          <t>375628</t>
+        </is>
+      </c>
+      <c r="H977" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I977" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="978" ht="20" customHeight="1">
+      <c r="A978" s="9" t="n">
+        <v>974</v>
+      </c>
+      <c r="B978" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C978" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D978" s="9" t="n">
+        <v>1331</v>
+      </c>
+      <c r="E978" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F978" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G978" s="10" t="inlineStr">
+        <is>
+          <t>375625</t>
+        </is>
+      </c>
+      <c r="H978" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I978" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="979" ht="20" customHeight="1">
+      <c r="A979" s="9" t="n">
+        <v>975</v>
+      </c>
+      <c r="B979" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C979" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D979" s="9" t="n">
+        <v>1333</v>
+      </c>
+      <c r="E979" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F979" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G979" s="10" t="inlineStr">
+        <is>
+          <t>375629</t>
+        </is>
+      </c>
+      <c r="H979" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I979" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="980" ht="20" customHeight="1">
+      <c r="A980" s="9" t="n">
+        <v>976</v>
+      </c>
+      <c r="B980" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C980" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D980" s="9" t="n">
+        <v>1338</v>
+      </c>
+      <c r="E980" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F980" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G980" s="10" t="inlineStr">
+        <is>
+          <t>375630</t>
+        </is>
+      </c>
+      <c r="H980" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I980" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="981" ht="20" customHeight="1">
+      <c r="A981" s="9" t="n">
+        <v>977</v>
+      </c>
+      <c r="B981" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C981" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D981" s="9" t="n">
+        <v>1339</v>
+      </c>
+      <c r="E981" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F981" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G981" s="10" t="inlineStr">
+        <is>
+          <t>375631</t>
+        </is>
+      </c>
+      <c r="H981" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I981" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="982" ht="20" customHeight="1">
+      <c r="A982" s="9" t="n">
+        <v>978</v>
+      </c>
+      <c r="B982" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C982" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D982" s="9" t="n">
+        <v>1341</v>
+      </c>
+      <c r="E982" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F982" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G982" s="10" t="inlineStr">
+        <is>
+          <t>375627</t>
+        </is>
+      </c>
+      <c r="H982" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I982" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="983" ht="20" customHeight="1">
+      <c r="A983" s="9" t="n">
+        <v>979</v>
+      </c>
+      <c r="B983" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C983" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D983" s="9" t="n">
+        <v>1346</v>
+      </c>
+      <c r="E983" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F983" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G983" s="10" t="inlineStr">
+        <is>
+          <t>375632</t>
+        </is>
+      </c>
+      <c r="H983" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I983" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="984" ht="20" customHeight="1">
+      <c r="A984" s="9" t="n">
+        <v>980</v>
+      </c>
+      <c r="B984" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C984" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D984" s="9" t="n">
+        <v>1352</v>
+      </c>
+      <c r="E984" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F984" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G984" s="10" t="inlineStr">
+        <is>
+          <t>375633</t>
+        </is>
+      </c>
+      <c r="H984" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I984" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="985" ht="20" customHeight="1">
+      <c r="A985" s="9" t="n">
+        <v>981</v>
+      </c>
+      <c r="B985" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C985" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D985" s="9" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E985" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F985" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G985" s="10" t="inlineStr">
+        <is>
+          <t>375122</t>
+        </is>
+      </c>
+      <c r="H985" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I985" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="986" ht="20" customHeight="1">
+      <c r="A986" s="9" t="n">
+        <v>982</v>
+      </c>
+      <c r="B986" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C986" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D986" s="9" t="n">
+        <v>1354</v>
+      </c>
+      <c r="E986" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F986" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G986" s="10" t="inlineStr">
+        <is>
+          <t>375634</t>
+        </is>
+      </c>
+      <c r="H986" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I986" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="987" ht="20" customHeight="1">
+      <c r="A987" s="9" t="n">
+        <v>983</v>
+      </c>
+      <c r="B987" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C987" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D987" s="9" t="n">
+        <v>1355</v>
+      </c>
+      <c r="E987" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F987" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G987" s="10" t="inlineStr">
+        <is>
+          <t>375121</t>
+        </is>
+      </c>
+      <c r="H987" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I987" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="988" ht="20" customHeight="1">
+      <c r="A988" s="9" t="n">
+        <v>984</v>
+      </c>
+      <c r="B988" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C988" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D988" s="9" t="n">
+        <v>1356</v>
+      </c>
+      <c r="E988" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F988" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G988" s="10" t="inlineStr">
+        <is>
+          <t>375123</t>
+        </is>
+      </c>
+      <c r="H988" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I988" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="989" ht="20" customHeight="1">
+      <c r="A989" s="9" t="n">
+        <v>985</v>
+      </c>
+      <c r="B989" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C989" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D989" s="9" t="n">
+        <v>1358</v>
+      </c>
+      <c r="E989" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F989" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G989" s="10" t="inlineStr">
+        <is>
+          <t>375124</t>
+        </is>
+      </c>
+      <c r="H989" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I989" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="990" ht="20" customHeight="1">
+      <c r="A990" s="9" t="n">
+        <v>986</v>
+      </c>
+      <c r="B990" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C990" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D990" s="9" t="n">
+        <v>1359</v>
+      </c>
+      <c r="E990" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F990" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G990" s="10" t="inlineStr">
+        <is>
+          <t>375130</t>
+        </is>
+      </c>
+      <c r="H990" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I990" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="991" ht="20" customHeight="1">
+      <c r="A991" s="9" t="n">
+        <v>987</v>
+      </c>
+      <c r="B991" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C991" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D991" s="9" t="n">
+        <v>1360</v>
+      </c>
+      <c r="E991" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F991" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G991" s="10" t="inlineStr">
+        <is>
+          <t>375125</t>
+        </is>
+      </c>
+      <c r="H991" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I991" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="992" ht="20" customHeight="1">
+      <c r="A992" s="9" t="n">
+        <v>988</v>
+      </c>
+      <c r="B992" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C992" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D992" s="9" t="n">
+        <v>1361</v>
+      </c>
+      <c r="E992" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F992" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G992" s="10" t="inlineStr">
+        <is>
+          <t>375126</t>
+        </is>
+      </c>
+      <c r="H992" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I992" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="993" ht="20" customHeight="1">
+      <c r="A993" s="9" t="n">
+        <v>989</v>
+      </c>
+      <c r="B993" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C993" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D993" s="9" t="n">
+        <v>1362</v>
+      </c>
+      <c r="E993" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F993" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G993" s="10" t="inlineStr">
+        <is>
+          <t>375129</t>
+        </is>
+      </c>
+      <c r="H993" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I993" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="994" ht="20" customHeight="1">
+      <c r="A994" s="9" t="n">
+        <v>990</v>
+      </c>
+      <c r="B994" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C994" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D994" s="9" t="n">
+        <v>1363</v>
+      </c>
+      <c r="E994" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F994" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G994" s="10" t="inlineStr">
+        <is>
+          <t>375127</t>
+        </is>
+      </c>
+      <c r="H994" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I994" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="995" ht="20" customHeight="1">
+      <c r="A995" s="9" t="n">
+        <v>991</v>
+      </c>
+      <c r="B995" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C995" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D995" s="9" t="n">
+        <v>1364</v>
+      </c>
+      <c r="E995" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F995" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G995" s="10" t="inlineStr">
+        <is>
+          <t>375636</t>
+        </is>
+      </c>
+      <c r="H995" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I995" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="996" ht="20" customHeight="1">
+      <c r="A996" s="9" t="n">
+        <v>992</v>
+      </c>
+      <c r="B996" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C996" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D996" s="9" t="n">
+        <v>1365</v>
+      </c>
+      <c r="E996" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F996" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G996" s="10" t="inlineStr">
+        <is>
+          <t>375128</t>
+        </is>
+      </c>
+      <c r="H996" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I996" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="997" ht="20" customHeight="1">
+      <c r="A997" s="9" t="n">
+        <v>993</v>
+      </c>
+      <c r="B997" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C997" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D997" s="9" t="n">
+        <v>1366</v>
+      </c>
+      <c r="E997" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F997" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G997" s="10" t="inlineStr">
+        <is>
+          <t>375635</t>
+        </is>
+      </c>
+      <c r="H997" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I997" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="998" ht="20" customHeight="1">
+      <c r="A998" s="9" t="n">
+        <v>994</v>
+      </c>
+      <c r="B998" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C998" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D998" s="9" t="n">
+        <v>1370</v>
+      </c>
+      <c r="E998" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F998" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G998" s="10" t="inlineStr">
+        <is>
+          <t>375132</t>
+        </is>
+      </c>
+      <c r="H998" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I998" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="999" ht="20" customHeight="1">
+      <c r="A999" s="9" t="n">
+        <v>995</v>
+      </c>
+      <c r="B999" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C999" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D999" s="9" t="n">
+        <v>1371</v>
+      </c>
+      <c r="E999" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F999" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G999" s="10" t="inlineStr">
+        <is>
+          <t>375131</t>
+        </is>
+      </c>
+      <c r="H999" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I999" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000" ht="20" customHeight="1">
+      <c r="A1000" s="9" t="n">
+        <v>996</v>
+      </c>
+      <c r="B1000" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1000" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D1000" s="9" t="n">
+        <v>1372</v>
+      </c>
+      <c r="E1000" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1000" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1000" s="10" t="inlineStr">
+        <is>
+          <t>375133</t>
+        </is>
+      </c>
+      <c r="H1000" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I1000" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001" ht="20" customHeight="1">
+      <c r="A1001" s="9" t="n">
+        <v>997</v>
+      </c>
+      <c r="B1001" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1001" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D1001" s="9" t="n">
+        <v>1373</v>
+      </c>
+      <c r="E1001" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1001" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1001" s="10" t="inlineStr">
+        <is>
+          <t>375623</t>
+        </is>
+      </c>
+      <c r="H1001" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I1001" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002" ht="20" customHeight="1">
+      <c r="A1002" s="9" t="n">
+        <v>998</v>
+      </c>
+      <c r="B1002" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1002" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D1002" s="9" t="n">
+        <v>1374</v>
+      </c>
+      <c r="E1002" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1002" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G1002" s="10" t="inlineStr">
+        <is>
+          <t>375624</t>
+        </is>
+      </c>
+      <c r="H1002" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I1002" s="11" t="inlineStr">
+        <is>
+          <t>grade 21 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (998 BAL)</t>
+        </is>
+      </c>
+      <c r="B1003" s="4" t="n"/>
+      <c r="C1003" s="4" t="n"/>
+      <c r="D1003" s="4" t="n"/>
+      <c r="E1003" s="4" t="n"/>
+      <c r="F1003" s="4" t="n"/>
+      <c r="G1003" s="4" t="n"/>
+      <c r="H1003" s="4">
+        <f>SUM(H5:H1002)</f>
         <v/>
       </c>
-      <c r="I944" s="4" t="inlineStr">
+      <c r="I1003" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -54257,8 +57620,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1003:G1003"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A944:G944"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -54270,7 +57633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -55145,37 +58508,66 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>2459</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>41.68</v>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>1283 - 1374</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4">
-        <f>SUM(D5:D32)</f>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4">
+        <f>SUM(D5:D33)</f>
         <v/>
       </c>
-      <c r="E33" s="4">
-        <f>SUM(E5:E32)</f>
+      <c r="E34" s="4">
+        <f>SUM(E5:E33)</f>
         <v/>
       </c>
-      <c r="F33" s="4">
-        <f>AVERAGE(F5:F32)</f>
+      <c r="F34" s="4">
+        <f>AVERAGE(F5:F33)</f>
         <v/>
       </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>3 - 1282</t>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>3 - 1374</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A34:C34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: tambah data bal tembakau tanggal 22 September 2026 (58 bal, No Gud 1376-1477), update rekap excel, dan bump cache version v=6.5
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1003"/>
+  <dimension ref="A1:F1061"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20554,20 +20554,1180 @@
       </c>
       <c r="F1002" s="5" t="n"/>
     </row>
-    <row r="1003" ht="22" customHeight="1">
-      <c r="A1003" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (998 BAL)</t>
-        </is>
-      </c>
-      <c r="B1003" s="4" t="n"/>
-      <c r="C1003" s="4" t="n"/>
-      <c r="D1003" s="4" t="n"/>
-      <c r="E1003" s="4">
-        <f>SUM(E5:E1002)</f>
+    <row r="1003" ht="20.25" customHeight="1">
+      <c r="A1003" s="5" t="n">
+        <v>1376</v>
+      </c>
+      <c r="B1003" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1003" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D1003" s="6" t="inlineStr">
+        <is>
+          <t>375176</t>
+        </is>
+      </c>
+      <c r="E1003" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F1003" s="5" t="n"/>
+    </row>
+    <row r="1004" ht="20.25" customHeight="1">
+      <c r="A1004" s="5" t="n">
+        <v>1377</v>
+      </c>
+      <c r="B1004" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1004" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D1004" s="6" t="inlineStr">
+        <is>
+          <t>376200</t>
+        </is>
+      </c>
+      <c r="E1004" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F1004" s="5" t="n"/>
+    </row>
+    <row r="1005" ht="20.25" customHeight="1">
+      <c r="A1005" s="5" t="n">
+        <v>1378</v>
+      </c>
+      <c r="B1005" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1005" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1005" s="6" t="inlineStr">
+        <is>
+          <t>376268</t>
+        </is>
+      </c>
+      <c r="E1005" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F1005" s="5" t="n"/>
+    </row>
+    <row r="1006" ht="20.25" customHeight="1">
+      <c r="A1006" s="5" t="n">
+        <v>1379</v>
+      </c>
+      <c r="B1006" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C1006" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D1006" s="6" t="inlineStr">
+        <is>
+          <t>376199</t>
+        </is>
+      </c>
+      <c r="E1006" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1006" s="5" t="n"/>
+    </row>
+    <row r="1007" ht="20.25" customHeight="1">
+      <c r="A1007" s="5" t="n">
+        <v>1383</v>
+      </c>
+      <c r="B1007" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1007" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1007" s="6" t="inlineStr">
+        <is>
+          <t>376269</t>
+        </is>
+      </c>
+      <c r="E1007" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F1007" s="5" t="n"/>
+    </row>
+    <row r="1008" ht="20.25" customHeight="1">
+      <c r="A1008" s="5" t="n">
+        <v>1384</v>
+      </c>
+      <c r="B1008" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1008" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1008" s="6" t="inlineStr">
+        <is>
+          <t>376270</t>
+        </is>
+      </c>
+      <c r="E1008" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F1008" s="5" t="n"/>
+    </row>
+    <row r="1009" ht="20.25" customHeight="1">
+      <c r="A1009" s="5" t="n">
+        <v>1386</v>
+      </c>
+      <c r="B1009" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1009" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D1009" s="6" t="inlineStr">
+        <is>
+          <t>375177</t>
+        </is>
+      </c>
+      <c r="E1009" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F1009" s="5" t="n"/>
+    </row>
+    <row r="1010" ht="20.25" customHeight="1">
+      <c r="A1010" s="5" t="n">
+        <v>1393</v>
+      </c>
+      <c r="B1010" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C1010" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D1010" s="6" t="inlineStr">
+        <is>
+          <t>376601</t>
+        </is>
+      </c>
+      <c r="E1010" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F1010" s="5" t="n"/>
+    </row>
+    <row r="1011" ht="20.25" customHeight="1">
+      <c r="A1011" s="5" t="n">
+        <v>1396</v>
+      </c>
+      <c r="B1011" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1011" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1011" s="6" t="inlineStr">
+        <is>
+          <t>375178</t>
+        </is>
+      </c>
+      <c r="E1011" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F1011" s="5" t="n"/>
+    </row>
+    <row r="1012" ht="20.25" customHeight="1">
+      <c r="A1012" s="5" t="n">
+        <v>1397</v>
+      </c>
+      <c r="B1012" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1012" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D1012" s="6" t="inlineStr">
+        <is>
+          <t>374379</t>
+        </is>
+      </c>
+      <c r="E1012" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F1012" s="5" t="n"/>
+    </row>
+    <row r="1013" ht="20.25" customHeight="1">
+      <c r="A1013" s="5" t="n">
+        <v>1398</v>
+      </c>
+      <c r="B1013" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1013" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1013" s="6" t="inlineStr">
+        <is>
+          <t>375179</t>
+        </is>
+      </c>
+      <c r="E1013" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F1013" s="5" t="n"/>
+    </row>
+    <row r="1014" ht="20.25" customHeight="1">
+      <c r="A1014" s="5" t="n">
+        <v>1399</v>
+      </c>
+      <c r="B1014" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C1014" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="D1014" s="6" t="inlineStr">
+        <is>
+          <t>374378</t>
+        </is>
+      </c>
+      <c r="E1014" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F1014" s="5" t="n"/>
+    </row>
+    <row r="1015" ht="20.25" customHeight="1">
+      <c r="A1015" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="B1015" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C1015" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D1015" s="6" t="inlineStr">
+        <is>
+          <t>125881</t>
+        </is>
+      </c>
+      <c r="E1015" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1015" s="5" t="n"/>
+    </row>
+    <row r="1016" ht="20.25" customHeight="1">
+      <c r="A1016" s="5" t="n">
+        <v>1401</v>
+      </c>
+      <c r="B1016" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1016" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1016" s="6" t="inlineStr">
+        <is>
+          <t>376343</t>
+        </is>
+      </c>
+      <c r="E1016" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F1016" s="5" t="n"/>
+    </row>
+    <row r="1017" ht="20.25" customHeight="1">
+      <c r="A1017" s="5" t="n">
+        <v>1407</v>
+      </c>
+      <c r="B1017" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1017" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D1017" s="6" t="inlineStr">
+        <is>
+          <t>375180</t>
+        </is>
+      </c>
+      <c r="E1017" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F1017" s="5" t="n"/>
+    </row>
+    <row r="1018" ht="20.25" customHeight="1">
+      <c r="A1018" s="5" t="n">
+        <v>1409</v>
+      </c>
+      <c r="B1018" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1018" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1018" s="6" t="inlineStr">
+        <is>
+          <t>375181</t>
+        </is>
+      </c>
+      <c r="E1018" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F1018" s="5" t="n"/>
+    </row>
+    <row r="1019" ht="20.25" customHeight="1">
+      <c r="A1019" s="5" t="n">
+        <v>1410</v>
+      </c>
+      <c r="B1019" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1019" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1019" s="6" t="inlineStr">
+        <is>
+          <t>376277</t>
+        </is>
+      </c>
+      <c r="E1019" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F1019" s="5" t="n"/>
+    </row>
+    <row r="1020" ht="20.25" customHeight="1">
+      <c r="A1020" s="5" t="n">
+        <v>1411</v>
+      </c>
+      <c r="B1020" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1020" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1020" s="6" t="inlineStr">
+        <is>
+          <t>376278</t>
+        </is>
+      </c>
+      <c r="E1020" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F1020" s="5" t="n"/>
+    </row>
+    <row r="1021" ht="20.25" customHeight="1">
+      <c r="A1021" s="5" t="n">
+        <v>1412</v>
+      </c>
+      <c r="B1021" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1021" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1021" s="6" t="inlineStr">
+        <is>
+          <t>375191</t>
+        </is>
+      </c>
+      <c r="E1021" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F1021" s="5" t="n"/>
+    </row>
+    <row r="1022" ht="20.25" customHeight="1">
+      <c r="A1022" s="5" t="n">
+        <v>1413</v>
+      </c>
+      <c r="B1022" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1022" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1022" s="6" t="inlineStr">
+        <is>
+          <t>375192</t>
+        </is>
+      </c>
+      <c r="E1022" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F1022" s="5" t="n"/>
+    </row>
+    <row r="1023" ht="20.25" customHeight="1">
+      <c r="A1023" s="5" t="n">
+        <v>1414</v>
+      </c>
+      <c r="B1023" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1023" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1023" s="6" t="inlineStr">
+        <is>
+          <t>376344</t>
+        </is>
+      </c>
+      <c r="E1023" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F1023" s="5" t="n"/>
+    </row>
+    <row r="1024" ht="20.25" customHeight="1">
+      <c r="A1024" s="5" t="n">
+        <v>1415</v>
+      </c>
+      <c r="B1024" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1024" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1024" s="6" t="inlineStr">
+        <is>
+          <t>376347</t>
+        </is>
+      </c>
+      <c r="E1024" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F1024" s="5" t="n"/>
+    </row>
+    <row r="1025" ht="20.25" customHeight="1">
+      <c r="A1025" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="B1025" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1025" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1025" s="6" t="inlineStr">
+        <is>
+          <t>376345</t>
+        </is>
+      </c>
+      <c r="E1025" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F1025" s="5" t="n"/>
+    </row>
+    <row r="1026" ht="20.25" customHeight="1">
+      <c r="A1026" s="5" t="n">
+        <v>1417</v>
+      </c>
+      <c r="B1026" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1026" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D1026" s="6" t="inlineStr">
+        <is>
+          <t>376346</t>
+        </is>
+      </c>
+      <c r="E1026" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F1026" s="5" t="n"/>
+    </row>
+    <row r="1027" ht="20.25" customHeight="1">
+      <c r="A1027" s="5" t="n">
+        <v>1420</v>
+      </c>
+      <c r="B1027" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C1027" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D1027" s="6" t="inlineStr">
+        <is>
+          <t>374382</t>
+        </is>
+      </c>
+      <c r="E1027" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F1027" s="5" t="n"/>
+    </row>
+    <row r="1028" ht="20.25" customHeight="1">
+      <c r="A1028" s="5" t="n">
+        <v>1421</v>
+      </c>
+      <c r="B1028" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C1028" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D1028" s="6" t="inlineStr">
+        <is>
+          <t>374380</t>
+        </is>
+      </c>
+      <c r="E1028" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F1028" s="5" t="n"/>
+    </row>
+    <row r="1029" ht="20.25" customHeight="1">
+      <c r="A1029" s="5" t="n">
+        <v>1422</v>
+      </c>
+      <c r="B1029" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C1029" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D1029" s="6" t="inlineStr">
+        <is>
+          <t>374381</t>
+        </is>
+      </c>
+      <c r="E1029" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F1029" s="5" t="n"/>
+    </row>
+    <row r="1030" ht="20.25" customHeight="1">
+      <c r="A1030" s="5" t="n">
+        <v>1423</v>
+      </c>
+      <c r="B1030" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C1030" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D1030" s="6" t="inlineStr">
+        <is>
+          <t>375320</t>
+        </is>
+      </c>
+      <c r="E1030" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F1030" s="5" t="n"/>
+    </row>
+    <row r="1031" ht="20.25" customHeight="1">
+      <c r="A1031" s="5" t="n">
+        <v>1424</v>
+      </c>
+      <c r="B1031" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C1031" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D1031" s="6" t="inlineStr">
+        <is>
+          <t>375321</t>
+        </is>
+      </c>
+      <c r="E1031" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F1031" s="5" t="n"/>
+    </row>
+    <row r="1032" ht="20.25" customHeight="1">
+      <c r="A1032" s="5" t="n">
+        <v>1425</v>
+      </c>
+      <c r="B1032" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C1032" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D1032" s="6" t="inlineStr">
+        <is>
+          <t>375324</t>
+        </is>
+      </c>
+      <c r="E1032" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F1032" s="5" t="n"/>
+    </row>
+    <row r="1033" ht="20.25" customHeight="1">
+      <c r="A1033" s="5" t="n">
+        <v>1426</v>
+      </c>
+      <c r="B1033" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C1033" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D1033" s="6" t="inlineStr">
+        <is>
+          <t>375323</t>
+        </is>
+      </c>
+      <c r="E1033" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F1033" s="5" t="n"/>
+    </row>
+    <row r="1034" ht="20.25" customHeight="1">
+      <c r="A1034" s="5" t="n">
+        <v>1427</v>
+      </c>
+      <c r="B1034" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C1034" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D1034" s="6" t="inlineStr">
+        <is>
+          <t>375322</t>
+        </is>
+      </c>
+      <c r="E1034" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F1034" s="5" t="n"/>
+    </row>
+    <row r="1035" ht="20.25" customHeight="1">
+      <c r="A1035" s="5" t="n">
+        <v>1432</v>
+      </c>
+      <c r="B1035" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1035" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1035" s="6" t="inlineStr">
+        <is>
+          <t>375182</t>
+        </is>
+      </c>
+      <c r="E1035" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F1035" s="5" t="n"/>
+    </row>
+    <row r="1036" ht="20.25" customHeight="1">
+      <c r="A1036" s="5" t="n">
+        <v>1433</v>
+      </c>
+      <c r="B1036" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1036" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1036" s="6" t="inlineStr">
+        <is>
+          <t>375183</t>
+        </is>
+      </c>
+      <c r="E1036" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F1036" s="5" t="n"/>
+    </row>
+    <row r="1037" ht="20.25" customHeight="1">
+      <c r="A1037" s="5" t="n">
+        <v>1436</v>
+      </c>
+      <c r="B1037" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C1037" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D1037" s="6" t="inlineStr">
+        <is>
+          <t>376605</t>
+        </is>
+      </c>
+      <c r="E1037" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1037" s="5" t="n"/>
+    </row>
+    <row r="1038" ht="20.25" customHeight="1">
+      <c r="A1038" s="5" t="n">
+        <v>1437</v>
+      </c>
+      <c r="B1038" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C1038" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D1038" s="6" t="inlineStr">
+        <is>
+          <t>376603</t>
+        </is>
+      </c>
+      <c r="E1038" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F1038" s="5" t="n"/>
+    </row>
+    <row r="1039" ht="20.25" customHeight="1">
+      <c r="A1039" s="5" t="n">
+        <v>1438</v>
+      </c>
+      <c r="B1039" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C1039" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D1039" s="6" t="inlineStr">
+        <is>
+          <t>376604</t>
+        </is>
+      </c>
+      <c r="E1039" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1039" s="5" t="n"/>
+    </row>
+    <row r="1040" ht="20.25" customHeight="1">
+      <c r="A1040" s="5" t="n">
+        <v>1439</v>
+      </c>
+      <c r="B1040" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C1040" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D1040" s="6" t="inlineStr">
+        <is>
+          <t>376602</t>
+        </is>
+      </c>
+      <c r="E1040" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F1040" s="5" t="n"/>
+    </row>
+    <row r="1041" ht="20.25" customHeight="1">
+      <c r="A1041" s="5" t="n">
+        <v>1445</v>
+      </c>
+      <c r="B1041" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1041" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1041" s="6" t="inlineStr">
+        <is>
+          <t>375187</t>
+        </is>
+      </c>
+      <c r="E1041" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F1041" s="5" t="n"/>
+    </row>
+    <row r="1042" ht="20.25" customHeight="1">
+      <c r="A1042" s="5" t="n">
+        <v>1446</v>
+      </c>
+      <c r="B1042" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1042" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1042" s="6" t="inlineStr">
+        <is>
+          <t>375184</t>
+        </is>
+      </c>
+      <c r="E1042" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F1042" s="5" t="n"/>
+    </row>
+    <row r="1043" ht="20.25" customHeight="1">
+      <c r="A1043" s="5" t="n">
+        <v>1447</v>
+      </c>
+      <c r="B1043" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1043" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1043" s="6" t="inlineStr">
+        <is>
+          <t>375186</t>
+        </is>
+      </c>
+      <c r="E1043" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1043" s="5" t="n"/>
+    </row>
+    <row r="1044" ht="20.25" customHeight="1">
+      <c r="A1044" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="B1044" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1044" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1044" s="6" t="inlineStr">
+        <is>
+          <t>375185</t>
+        </is>
+      </c>
+      <c r="E1044" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F1044" s="5" t="n"/>
+    </row>
+    <row r="1045" ht="20.25" customHeight="1">
+      <c r="A1045" s="5" t="n">
+        <v>1449</v>
+      </c>
+      <c r="B1045" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1045" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D1045" s="6" t="inlineStr">
+        <is>
+          <t>376271</t>
+        </is>
+      </c>
+      <c r="E1045" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1045" s="5" t="n"/>
+    </row>
+    <row r="1046" ht="20.25" customHeight="1">
+      <c r="A1046" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="B1046" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1046" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1046" s="6" t="inlineStr">
+        <is>
+          <t>375190</t>
+        </is>
+      </c>
+      <c r="E1046" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F1046" s="5" t="n"/>
+    </row>
+    <row r="1047" ht="20.25" customHeight="1">
+      <c r="A1047" s="5" t="n">
+        <v>1451</v>
+      </c>
+      <c r="B1047" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1047" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1047" s="6" t="inlineStr">
+        <is>
+          <t>376272</t>
+        </is>
+      </c>
+      <c r="E1047" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F1047" s="5" t="n"/>
+    </row>
+    <row r="1048" ht="20.25" customHeight="1">
+      <c r="A1048" s="5" t="n">
+        <v>1453</v>
+      </c>
+      <c r="B1048" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1048" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1048" s="6" t="inlineStr">
+        <is>
+          <t>375189</t>
+        </is>
+      </c>
+      <c r="E1048" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1048" s="5" t="n"/>
+    </row>
+    <row r="1049" ht="20.25" customHeight="1">
+      <c r="A1049" s="5" t="n">
+        <v>1454</v>
+      </c>
+      <c r="B1049" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1049" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1049" s="6" t="inlineStr">
+        <is>
+          <t>375188</t>
+        </is>
+      </c>
+      <c r="E1049" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1049" s="5" t="n"/>
+    </row>
+    <row r="1050" ht="20.25" customHeight="1">
+      <c r="A1050" s="5" t="n">
+        <v>1455</v>
+      </c>
+      <c r="B1050" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1050" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1050" s="6" t="inlineStr">
+        <is>
+          <t>376274</t>
+        </is>
+      </c>
+      <c r="E1050" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F1050" s="5" t="n"/>
+    </row>
+    <row r="1051" ht="20.25" customHeight="1">
+      <c r="A1051" s="5" t="n">
+        <v>1456</v>
+      </c>
+      <c r="B1051" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1051" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="D1051" s="6" t="inlineStr">
+        <is>
+          <t>376276</t>
+        </is>
+      </c>
+      <c r="E1051" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1051" s="5" t="n"/>
+    </row>
+    <row r="1052" ht="20.25" customHeight="1">
+      <c r="A1052" s="5" t="n">
+        <v>1457</v>
+      </c>
+      <c r="B1052" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1052" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1052" s="6" t="inlineStr">
+        <is>
+          <t>376275</t>
+        </is>
+      </c>
+      <c r="E1052" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F1052" s="5" t="n"/>
+    </row>
+    <row r="1053" ht="20.25" customHeight="1">
+      <c r="A1053" s="5" t="n">
+        <v>1458</v>
+      </c>
+      <c r="B1053" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1053" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D1053" s="6" t="inlineStr">
+        <is>
+          <t>376273</t>
+        </is>
+      </c>
+      <c r="E1053" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F1053" s="5" t="n"/>
+    </row>
+    <row r="1054" ht="20.25" customHeight="1">
+      <c r="A1054" s="5" t="n">
+        <v>1460</v>
+      </c>
+      <c r="B1054" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C1054" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D1054" s="6" t="inlineStr">
+        <is>
+          <t>375193</t>
+        </is>
+      </c>
+      <c r="E1054" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F1054" s="5" t="n"/>
+    </row>
+    <row r="1055" ht="20.25" customHeight="1">
+      <c r="A1055" s="5" t="n">
+        <v>1470</v>
+      </c>
+      <c r="B1055" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C1055" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D1055" s="6" t="inlineStr">
+        <is>
+          <t>376349</t>
+        </is>
+      </c>
+      <c r="E1055" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F1055" s="5" t="n"/>
+    </row>
+    <row r="1056" ht="20.25" customHeight="1">
+      <c r="A1056" s="5" t="n">
+        <v>1471</v>
+      </c>
+      <c r="B1056" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C1056" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D1056" s="6" t="inlineStr">
+        <is>
+          <t>376348</t>
+        </is>
+      </c>
+      <c r="E1056" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F1056" s="5" t="n"/>
+    </row>
+    <row r="1057" ht="20.25" customHeight="1">
+      <c r="A1057" s="5" t="n">
+        <v>1474</v>
+      </c>
+      <c r="B1057" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C1057" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D1057" s="6" t="inlineStr">
+        <is>
+          <t>375319</t>
+        </is>
+      </c>
+      <c r="E1057" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F1057" s="5" t="n"/>
+    </row>
+    <row r="1058" ht="20.25" customHeight="1">
+      <c r="A1058" s="5" t="n">
+        <v>1475</v>
+      </c>
+      <c r="B1058" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C1058" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D1058" s="6" t="inlineStr">
+        <is>
+          <t>375318</t>
+        </is>
+      </c>
+      <c r="E1058" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1058" s="5" t="n"/>
+    </row>
+    <row r="1059" ht="20.25" customHeight="1">
+      <c r="A1059" s="5" t="n">
+        <v>1476</v>
+      </c>
+      <c r="B1059" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="C1059" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D1059" s="6" t="inlineStr">
+        <is>
+          <t>376606</t>
+        </is>
+      </c>
+      <c r="E1059" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F1059" s="5" t="n"/>
+    </row>
+    <row r="1060" ht="20.25" customHeight="1">
+      <c r="A1060" s="5" t="n">
+        <v>1477</v>
+      </c>
+      <c r="B1060" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="C1060" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D1060" s="6" t="inlineStr">
+        <is>
+          <t>376607</t>
+        </is>
+      </c>
+      <c r="E1060" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F1060" s="5" t="n"/>
+    </row>
+    <row r="1061" ht="22" customHeight="1">
+      <c r="A1061" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (1056 BAL)</t>
+        </is>
+      </c>
+      <c r="B1061" s="4" t="n"/>
+      <c r="C1061" s="4" t="n"/>
+      <c r="D1061" s="4" t="n"/>
+      <c r="E1061" s="4">
+        <f>SUM(E5:E1060)</f>
         <v/>
       </c>
-      <c r="F1003" s="4" t="inlineStr">
+      <c r="F1061" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -20579,7 +21739,7 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A1003:D1003"/>
+    <mergeCell ref="A1061:D1061"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:C4"/>
@@ -20594,7 +21754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1003"/>
+  <dimension ref="A1:I1061"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -20618,7 +21778,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 998 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 1056 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -57595,23 +58755,2169 @@
         </is>
       </c>
     </row>
-    <row r="1003">
-      <c r="A1003" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (998 BAL)</t>
-        </is>
-      </c>
-      <c r="B1003" s="4" t="n"/>
-      <c r="C1003" s="4" t="n"/>
-      <c r="D1003" s="4" t="n"/>
-      <c r="E1003" s="4" t="n"/>
-      <c r="F1003" s="4" t="n"/>
-      <c r="G1003" s="4" t="n"/>
-      <c r="H1003" s="4">
-        <f>SUM(H5:H1002)</f>
+    <row r="1003" ht="20" customHeight="1">
+      <c r="A1003" s="9" t="n">
+        <v>999</v>
+      </c>
+      <c r="B1003" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1003" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1003" s="9" t="n">
+        <v>1376</v>
+      </c>
+      <c r="E1003" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1003" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1003" s="10" t="inlineStr">
+        <is>
+          <t>375176</t>
+        </is>
+      </c>
+      <c r="H1003" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I1003" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004" ht="20" customHeight="1">
+      <c r="A1004" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B1004" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1004" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1004" s="9" t="n">
+        <v>1377</v>
+      </c>
+      <c r="E1004" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1004" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G1004" s="10" t="inlineStr">
+        <is>
+          <t>376200</t>
+        </is>
+      </c>
+      <c r="H1004" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1004" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005" ht="20" customHeight="1">
+      <c r="A1005" s="9" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B1005" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1005" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1005" s="9" t="n">
+        <v>1378</v>
+      </c>
+      <c r="E1005" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1005" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1005" s="10" t="inlineStr">
+        <is>
+          <t>376268</t>
+        </is>
+      </c>
+      <c r="H1005" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I1005" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006" ht="20" customHeight="1">
+      <c r="A1006" s="9" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B1006" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1006" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1006" s="9" t="n">
+        <v>1379</v>
+      </c>
+      <c r="E1006" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F1006" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G1006" s="10" t="inlineStr">
+        <is>
+          <t>376199</t>
+        </is>
+      </c>
+      <c r="H1006" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1006" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007" ht="20" customHeight="1">
+      <c r="A1007" s="9" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B1007" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1007" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1007" s="9" t="n">
+        <v>1383</v>
+      </c>
+      <c r="E1007" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1007" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1007" s="10" t="inlineStr">
+        <is>
+          <t>376269</t>
+        </is>
+      </c>
+      <c r="H1007" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1007" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008" ht="20" customHeight="1">
+      <c r="A1008" s="9" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B1008" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1008" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1008" s="9" t="n">
+        <v>1384</v>
+      </c>
+      <c r="E1008" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1008" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1008" s="10" t="inlineStr">
+        <is>
+          <t>376270</t>
+        </is>
+      </c>
+      <c r="H1008" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1008" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009" ht="20" customHeight="1">
+      <c r="A1009" s="9" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B1009" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1009" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1009" s="9" t="n">
+        <v>1386</v>
+      </c>
+      <c r="E1009" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1009" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1009" s="10" t="inlineStr">
+        <is>
+          <t>375177</t>
+        </is>
+      </c>
+      <c r="H1009" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1009" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010" ht="20" customHeight="1">
+      <c r="A1010" s="9" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B1010" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1010" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1010" s="9" t="n">
+        <v>1393</v>
+      </c>
+      <c r="E1010" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F1010" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G1010" s="10" t="inlineStr">
+        <is>
+          <t>376601</t>
+        </is>
+      </c>
+      <c r="H1010" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I1010" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011" ht="20" customHeight="1">
+      <c r="A1011" s="9" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B1011" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1011" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1011" s="9" t="n">
+        <v>1396</v>
+      </c>
+      <c r="E1011" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1011" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1011" s="10" t="inlineStr">
+        <is>
+          <t>375178</t>
+        </is>
+      </c>
+      <c r="H1011" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I1011" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012" ht="20" customHeight="1">
+      <c r="A1012" s="9" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B1012" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1012" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1012" s="9" t="n">
+        <v>1397</v>
+      </c>
+      <c r="E1012" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1012" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1012" s="10" t="inlineStr">
+        <is>
+          <t>374379</t>
+        </is>
+      </c>
+      <c r="H1012" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I1012" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013" ht="20" customHeight="1">
+      <c r="A1013" s="9" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B1013" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1013" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1013" s="9" t="n">
+        <v>1398</v>
+      </c>
+      <c r="E1013" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1013" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1013" s="10" t="inlineStr">
+        <is>
+          <t>375179</t>
+        </is>
+      </c>
+      <c r="H1013" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I1013" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014" ht="20" customHeight="1">
+      <c r="A1014" s="9" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B1014" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1014" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1014" s="9" t="n">
+        <v>1399</v>
+      </c>
+      <c r="E1014" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F1014" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="G1014" s="10" t="inlineStr">
+        <is>
+          <t>374378</t>
+        </is>
+      </c>
+      <c r="H1014" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I1014" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015" ht="20" customHeight="1">
+      <c r="A1015" s="9" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B1015" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1015" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1015" s="9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E1015" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F1015" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1015" s="10" t="inlineStr">
+        <is>
+          <t>125881</t>
+        </is>
+      </c>
+      <c r="H1015" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1015" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016" ht="20" customHeight="1">
+      <c r="A1016" s="9" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B1016" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1016" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1016" s="9" t="n">
+        <v>1401</v>
+      </c>
+      <c r="E1016" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1016" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1016" s="10" t="inlineStr">
+        <is>
+          <t>376343</t>
+        </is>
+      </c>
+      <c r="H1016" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1016" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017" ht="20" customHeight="1">
+      <c r="A1017" s="9" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B1017" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1017" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1017" s="9" t="n">
+        <v>1407</v>
+      </c>
+      <c r="E1017" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1017" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1017" s="10" t="inlineStr">
+        <is>
+          <t>375180</t>
+        </is>
+      </c>
+      <c r="H1017" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I1017" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018" ht="20" customHeight="1">
+      <c r="A1018" s="9" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B1018" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1018" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1018" s="9" t="n">
+        <v>1409</v>
+      </c>
+      <c r="E1018" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1018" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1018" s="10" t="inlineStr">
+        <is>
+          <t>375181</t>
+        </is>
+      </c>
+      <c r="H1018" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1018" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019" ht="20" customHeight="1">
+      <c r="A1019" s="9" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B1019" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1019" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1019" s="9" t="n">
+        <v>1410</v>
+      </c>
+      <c r="E1019" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1019" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1019" s="10" t="inlineStr">
+        <is>
+          <t>376277</t>
+        </is>
+      </c>
+      <c r="H1019" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1019" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020" ht="20" customHeight="1">
+      <c r="A1020" s="9" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B1020" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1020" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1020" s="9" t="n">
+        <v>1411</v>
+      </c>
+      <c r="E1020" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1020" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1020" s="10" t="inlineStr">
+        <is>
+          <t>376278</t>
+        </is>
+      </c>
+      <c r="H1020" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1020" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021" ht="20" customHeight="1">
+      <c r="A1021" s="9" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B1021" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1021" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1021" s="9" t="n">
+        <v>1412</v>
+      </c>
+      <c r="E1021" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1021" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1021" s="10" t="inlineStr">
+        <is>
+          <t>375191</t>
+        </is>
+      </c>
+      <c r="H1021" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I1021" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022" ht="20" customHeight="1">
+      <c r="A1022" s="9" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B1022" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1022" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1022" s="9" t="n">
+        <v>1413</v>
+      </c>
+      <c r="E1022" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1022" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1022" s="10" t="inlineStr">
+        <is>
+          <t>375192</t>
+        </is>
+      </c>
+      <c r="H1022" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1022" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023" ht="20" customHeight="1">
+      <c r="A1023" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B1023" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1023" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1023" s="9" t="n">
+        <v>1414</v>
+      </c>
+      <c r="E1023" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1023" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1023" s="10" t="inlineStr">
+        <is>
+          <t>376344</t>
+        </is>
+      </c>
+      <c r="H1023" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1023" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024" ht="20" customHeight="1">
+      <c r="A1024" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B1024" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1024" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1024" s="9" t="n">
+        <v>1415</v>
+      </c>
+      <c r="E1024" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1024" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1024" s="10" t="inlineStr">
+        <is>
+          <t>376347</t>
+        </is>
+      </c>
+      <c r="H1024" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I1024" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025" ht="20" customHeight="1">
+      <c r="A1025" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B1025" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1025" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1025" s="9" t="n">
+        <v>1416</v>
+      </c>
+      <c r="E1025" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1025" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1025" s="10" t="inlineStr">
+        <is>
+          <t>376345</t>
+        </is>
+      </c>
+      <c r="H1025" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1025" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026" ht="20" customHeight="1">
+      <c r="A1026" s="9" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B1026" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1026" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1026" s="9" t="n">
+        <v>1417</v>
+      </c>
+      <c r="E1026" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1026" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1026" s="10" t="inlineStr">
+        <is>
+          <t>376346</t>
+        </is>
+      </c>
+      <c r="H1026" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I1026" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027" ht="20" customHeight="1">
+      <c r="A1027" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B1027" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1027" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1027" s="9" t="n">
+        <v>1420</v>
+      </c>
+      <c r="E1027" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F1027" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1027" s="10" t="inlineStr">
+        <is>
+          <t>374382</t>
+        </is>
+      </c>
+      <c r="H1027" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1027" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028" ht="20" customHeight="1">
+      <c r="A1028" s="9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B1028" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1028" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1028" s="9" t="n">
+        <v>1421</v>
+      </c>
+      <c r="E1028" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F1028" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1028" s="10" t="inlineStr">
+        <is>
+          <t>374380</t>
+        </is>
+      </c>
+      <c r="H1028" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I1028" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029" ht="20" customHeight="1">
+      <c r="A1029" s="9" t="n">
+        <v>1025</v>
+      </c>
+      <c r="B1029" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1029" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1029" s="9" t="n">
+        <v>1422</v>
+      </c>
+      <c r="E1029" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F1029" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1029" s="10" t="inlineStr">
+        <is>
+          <t>374381</t>
+        </is>
+      </c>
+      <c r="H1029" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I1029" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030" ht="20" customHeight="1">
+      <c r="A1030" s="9" t="n">
+        <v>1026</v>
+      </c>
+      <c r="B1030" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1030" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1030" s="9" t="n">
+        <v>1423</v>
+      </c>
+      <c r="E1030" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F1030" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1030" s="10" t="inlineStr">
+        <is>
+          <t>375320</t>
+        </is>
+      </c>
+      <c r="H1030" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I1030" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031" ht="20" customHeight="1">
+      <c r="A1031" s="9" t="n">
+        <v>1027</v>
+      </c>
+      <c r="B1031" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1031" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1031" s="9" t="n">
+        <v>1424</v>
+      </c>
+      <c r="E1031" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F1031" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1031" s="10" t="inlineStr">
+        <is>
+          <t>375321</t>
+        </is>
+      </c>
+      <c r="H1031" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I1031" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032" ht="20" customHeight="1">
+      <c r="A1032" s="9" t="n">
+        <v>1028</v>
+      </c>
+      <c r="B1032" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1032" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1032" s="9" t="n">
+        <v>1425</v>
+      </c>
+      <c r="E1032" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F1032" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1032" s="10" t="inlineStr">
+        <is>
+          <t>375324</t>
+        </is>
+      </c>
+      <c r="H1032" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I1032" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033" ht="20" customHeight="1">
+      <c r="A1033" s="9" t="n">
+        <v>1029</v>
+      </c>
+      <c r="B1033" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1033" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1033" s="9" t="n">
+        <v>1426</v>
+      </c>
+      <c r="E1033" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F1033" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1033" s="10" t="inlineStr">
+        <is>
+          <t>375323</t>
+        </is>
+      </c>
+      <c r="H1033" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I1033" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034" ht="20" customHeight="1">
+      <c r="A1034" s="9" t="n">
+        <v>1030</v>
+      </c>
+      <c r="B1034" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1034" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1034" s="9" t="n">
+        <v>1427</v>
+      </c>
+      <c r="E1034" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F1034" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1034" s="10" t="inlineStr">
+        <is>
+          <t>375322</t>
+        </is>
+      </c>
+      <c r="H1034" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1034" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035" ht="20" customHeight="1">
+      <c r="A1035" s="9" t="n">
+        <v>1031</v>
+      </c>
+      <c r="B1035" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1035" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1035" s="9" t="n">
+        <v>1432</v>
+      </c>
+      <c r="E1035" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1035" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1035" s="10" t="inlineStr">
+        <is>
+          <t>375182</t>
+        </is>
+      </c>
+      <c r="H1035" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I1035" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036" ht="20" customHeight="1">
+      <c r="A1036" s="9" t="n">
+        <v>1032</v>
+      </c>
+      <c r="B1036" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1036" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1036" s="9" t="n">
+        <v>1433</v>
+      </c>
+      <c r="E1036" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1036" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1036" s="10" t="inlineStr">
+        <is>
+          <t>375183</t>
+        </is>
+      </c>
+      <c r="H1036" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1036" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037" ht="20" customHeight="1">
+      <c r="A1037" s="9" t="n">
+        <v>1033</v>
+      </c>
+      <c r="B1037" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1037" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1037" s="9" t="n">
+        <v>1436</v>
+      </c>
+      <c r="E1037" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F1037" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G1037" s="10" t="inlineStr">
+        <is>
+          <t>376605</t>
+        </is>
+      </c>
+      <c r="H1037" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1037" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038" ht="20" customHeight="1">
+      <c r="A1038" s="9" t="n">
+        <v>1034</v>
+      </c>
+      <c r="B1038" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1038" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1038" s="9" t="n">
+        <v>1437</v>
+      </c>
+      <c r="E1038" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F1038" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G1038" s="10" t="inlineStr">
+        <is>
+          <t>376603</t>
+        </is>
+      </c>
+      <c r="H1038" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1038" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039" ht="20" customHeight="1">
+      <c r="A1039" s="9" t="n">
+        <v>1035</v>
+      </c>
+      <c r="B1039" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1039" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1039" s="9" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E1039" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F1039" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="G1039" s="10" t="inlineStr">
+        <is>
+          <t>376604</t>
+        </is>
+      </c>
+      <c r="H1039" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1039" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040" ht="20" customHeight="1">
+      <c r="A1040" s="9" t="n">
+        <v>1036</v>
+      </c>
+      <c r="B1040" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1040" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1040" s="9" t="n">
+        <v>1439</v>
+      </c>
+      <c r="E1040" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F1040" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G1040" s="10" t="inlineStr">
+        <is>
+          <t>376602</t>
+        </is>
+      </c>
+      <c r="H1040" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1040" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041" ht="20" customHeight="1">
+      <c r="A1041" s="9" t="n">
+        <v>1037</v>
+      </c>
+      <c r="B1041" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1041" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1041" s="9" t="n">
+        <v>1445</v>
+      </c>
+      <c r="E1041" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1041" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1041" s="10" t="inlineStr">
+        <is>
+          <t>375187</t>
+        </is>
+      </c>
+      <c r="H1041" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I1041" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042" ht="20" customHeight="1">
+      <c r="A1042" s="9" t="n">
+        <v>1038</v>
+      </c>
+      <c r="B1042" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1042" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1042" s="9" t="n">
+        <v>1446</v>
+      </c>
+      <c r="E1042" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1042" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1042" s="10" t="inlineStr">
+        <is>
+          <t>375184</t>
+        </is>
+      </c>
+      <c r="H1042" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I1042" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043" ht="20" customHeight="1">
+      <c r="A1043" s="9" t="n">
+        <v>1039</v>
+      </c>
+      <c r="B1043" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1043" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1043" s="9" t="n">
+        <v>1447</v>
+      </c>
+      <c r="E1043" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1043" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1043" s="10" t="inlineStr">
+        <is>
+          <t>375186</t>
+        </is>
+      </c>
+      <c r="H1043" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1043" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044" ht="20" customHeight="1">
+      <c r="A1044" s="9" t="n">
+        <v>1040</v>
+      </c>
+      <c r="B1044" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1044" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1044" s="9" t="n">
+        <v>1448</v>
+      </c>
+      <c r="E1044" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1044" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1044" s="10" t="inlineStr">
+        <is>
+          <t>375185</t>
+        </is>
+      </c>
+      <c r="H1044" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1044" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045" ht="20" customHeight="1">
+      <c r="A1045" s="9" t="n">
+        <v>1041</v>
+      </c>
+      <c r="B1045" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1045" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1045" s="9" t="n">
+        <v>1449</v>
+      </c>
+      <c r="E1045" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1045" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G1045" s="10" t="inlineStr">
+        <is>
+          <t>376271</t>
+        </is>
+      </c>
+      <c r="H1045" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1045" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046" ht="20" customHeight="1">
+      <c r="A1046" s="9" t="n">
+        <v>1042</v>
+      </c>
+      <c r="B1046" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1046" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1046" s="9" t="n">
+        <v>1450</v>
+      </c>
+      <c r="E1046" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1046" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1046" s="10" t="inlineStr">
+        <is>
+          <t>375190</t>
+        </is>
+      </c>
+      <c r="H1046" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1046" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047" ht="20" customHeight="1">
+      <c r="A1047" s="9" t="n">
+        <v>1043</v>
+      </c>
+      <c r="B1047" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1047" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1047" s="9" t="n">
+        <v>1451</v>
+      </c>
+      <c r="E1047" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1047" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1047" s="10" t="inlineStr">
+        <is>
+          <t>376272</t>
+        </is>
+      </c>
+      <c r="H1047" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I1047" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048" ht="20" customHeight="1">
+      <c r="A1048" s="9" t="n">
+        <v>1044</v>
+      </c>
+      <c r="B1048" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1048" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1048" s="9" t="n">
+        <v>1453</v>
+      </c>
+      <c r="E1048" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1048" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1048" s="10" t="inlineStr">
+        <is>
+          <t>375189</t>
+        </is>
+      </c>
+      <c r="H1048" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1048" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049" ht="20" customHeight="1">
+      <c r="A1049" s="9" t="n">
+        <v>1045</v>
+      </c>
+      <c r="B1049" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1049" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1049" s="9" t="n">
+        <v>1454</v>
+      </c>
+      <c r="E1049" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1049" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1049" s="10" t="inlineStr">
+        <is>
+          <t>375188</t>
+        </is>
+      </c>
+      <c r="H1049" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1049" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050" ht="20" customHeight="1">
+      <c r="A1050" s="9" t="n">
+        <v>1046</v>
+      </c>
+      <c r="B1050" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1050" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1050" s="9" t="n">
+        <v>1455</v>
+      </c>
+      <c r="E1050" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1050" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1050" s="10" t="inlineStr">
+        <is>
+          <t>376274</t>
+        </is>
+      </c>
+      <c r="H1050" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1050" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051" ht="20" customHeight="1">
+      <c r="A1051" s="9" t="n">
+        <v>1047</v>
+      </c>
+      <c r="B1051" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1051" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1051" s="9" t="n">
+        <v>1456</v>
+      </c>
+      <c r="E1051" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F1051" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1051" s="10" t="inlineStr">
+        <is>
+          <t>376276</t>
+        </is>
+      </c>
+      <c r="H1051" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1051" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052" ht="20" customHeight="1">
+      <c r="A1052" s="9" t="n">
+        <v>1048</v>
+      </c>
+      <c r="B1052" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1052" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1052" s="9" t="n">
+        <v>1457</v>
+      </c>
+      <c r="E1052" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1052" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1052" s="10" t="inlineStr">
+        <is>
+          <t>376275</t>
+        </is>
+      </c>
+      <c r="H1052" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I1052" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053" ht="20" customHeight="1">
+      <c r="A1053" s="9" t="n">
+        <v>1049</v>
+      </c>
+      <c r="B1053" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1053" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1053" s="9" t="n">
+        <v>1458</v>
+      </c>
+      <c r="E1053" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1053" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1053" s="10" t="inlineStr">
+        <is>
+          <t>376273</t>
+        </is>
+      </c>
+      <c r="H1053" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1053" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054" ht="20" customHeight="1">
+      <c r="A1054" s="9" t="n">
+        <v>1050</v>
+      </c>
+      <c r="B1054" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1054" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1054" s="9" t="n">
+        <v>1460</v>
+      </c>
+      <c r="E1054" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F1054" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1054" s="10" t="inlineStr">
+        <is>
+          <t>375193</t>
+        </is>
+      </c>
+      <c r="H1054" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1054" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055" ht="20" customHeight="1">
+      <c r="A1055" s="9" t="n">
+        <v>1051</v>
+      </c>
+      <c r="B1055" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1055" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1055" s="9" t="n">
+        <v>1470</v>
+      </c>
+      <c r="E1055" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F1055" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1055" s="10" t="inlineStr">
+        <is>
+          <t>376349</t>
+        </is>
+      </c>
+      <c r="H1055" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I1055" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056" ht="20" customHeight="1">
+      <c r="A1056" s="9" t="n">
+        <v>1052</v>
+      </c>
+      <c r="B1056" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1056" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1056" s="9" t="n">
+        <v>1471</v>
+      </c>
+      <c r="E1056" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F1056" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1056" s="10" t="inlineStr">
+        <is>
+          <t>376348</t>
+        </is>
+      </c>
+      <c r="H1056" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I1056" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057" ht="20" customHeight="1">
+      <c r="A1057" s="9" t="n">
+        <v>1053</v>
+      </c>
+      <c r="B1057" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1057" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1057" s="9" t="n">
+        <v>1474</v>
+      </c>
+      <c r="E1057" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F1057" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G1057" s="10" t="inlineStr">
+        <is>
+          <t>375319</t>
+        </is>
+      </c>
+      <c r="H1057" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1057" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058" ht="20" customHeight="1">
+      <c r="A1058" s="9" t="n">
+        <v>1054</v>
+      </c>
+      <c r="B1058" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1058" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1058" s="9" t="n">
+        <v>1475</v>
+      </c>
+      <c r="E1058" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F1058" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G1058" s="10" t="inlineStr">
+        <is>
+          <t>375318</t>
+        </is>
+      </c>
+      <c r="H1058" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I1058" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059" ht="20" customHeight="1">
+      <c r="A1059" s="9" t="n">
+        <v>1055</v>
+      </c>
+      <c r="B1059" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1059" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1059" s="9" t="n">
+        <v>1476</v>
+      </c>
+      <c r="E1059" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="F1059" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G1059" s="10" t="inlineStr">
+        <is>
+          <t>376606</t>
+        </is>
+      </c>
+      <c r="H1059" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I1059" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060" ht="20" customHeight="1">
+      <c r="A1060" s="9" t="n">
+        <v>1056</v>
+      </c>
+      <c r="B1060" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1060" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D1060" s="9" t="n">
+        <v>1477</v>
+      </c>
+      <c r="E1060" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="F1060" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G1060" s="10" t="inlineStr">
+        <is>
+          <t>376607</t>
+        </is>
+      </c>
+      <c r="H1060" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I1060" s="11" t="inlineStr">
+        <is>
+          <t>grade 22 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (1056 BAL)</t>
+        </is>
+      </c>
+      <c r="B1061" s="4" t="n"/>
+      <c r="C1061" s="4" t="n"/>
+      <c r="D1061" s="4" t="n"/>
+      <c r="E1061" s="4" t="n"/>
+      <c r="F1061" s="4" t="n"/>
+      <c r="G1061" s="4" t="n"/>
+      <c r="H1061" s="4">
+        <f>SUM(H5:H1060)</f>
         <v/>
       </c>
-      <c r="I1003" s="4" t="inlineStr">
+      <c r="I1061" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -57620,7 +60926,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A1003:G1003"/>
+    <mergeCell ref="A1061:G1061"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -57633,7 +60939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -58537,37 +61843,66 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>2537</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>43.74</v>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>1376 - 1477</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4">
-        <f>SUM(D5:D33)</f>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4">
+        <f>SUM(D5:D34)</f>
         <v/>
       </c>
-      <c r="E34" s="4">
-        <f>SUM(E5:E33)</f>
+      <c r="E35" s="4">
+        <f>SUM(E5:E34)</f>
         <v/>
       </c>
-      <c r="F34" s="4">
-        <f>AVERAGE(F5:F33)</f>
+      <c r="F35" s="4">
+        <f>AVERAGE(F5:F34)</f>
         <v/>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>3 - 1374</t>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>3 - 1477</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A35:C35"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A34:C34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update data bal tembakau tanggal 29 September 2026 (87 bal, 3723.0 kg, No Gud 1844-1995), sync Supabase, update rekap excel, dan bump cache version v=7.5
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -28849,7 +28849,9 @@
           <t>381362</t>
         </is>
       </c>
-      <c r="E1417" s="5" t="n"/>
+      <c r="E1417" s="5" t="n">
+        <v>45</v>
+      </c>
       <c r="F1417" s="5" t="n"/>
     </row>
     <row r="1418" ht="20.25" customHeight="1">
@@ -29707,7 +29709,9 @@
           <t>381098</t>
         </is>
       </c>
-      <c r="E1460" s="5" t="n"/>
+      <c r="E1460" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1460" s="5" t="n"/>
     </row>
     <row r="1461" ht="20.25" customHeight="1">
@@ -29825,7 +29829,9 @@
           <t>381099</t>
         </is>
       </c>
-      <c r="E1466" s="5" t="n"/>
+      <c r="E1466" s="5" t="n">
+        <v>46</v>
+      </c>
       <c r="F1466" s="5" t="n"/>
     </row>
     <row r="1467" ht="20.25" customHeight="1">
@@ -29843,7 +29849,9 @@
           <t>381097</t>
         </is>
       </c>
-      <c r="E1467" s="5" t="n"/>
+      <c r="E1467" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1467" s="5" t="n"/>
     </row>
     <row r="1468" ht="20.25" customHeight="1">
@@ -29861,7 +29869,9 @@
           <t>381372</t>
         </is>
       </c>
-      <c r="E1468" s="5" t="n"/>
+      <c r="E1468" s="5" t="n">
+        <v>37</v>
+      </c>
       <c r="F1468" s="5" t="n"/>
     </row>
     <row r="1469" ht="20.25" customHeight="1">
@@ -29879,7 +29889,9 @@
           <t>381083</t>
         </is>
       </c>
-      <c r="E1469" s="5" t="n"/>
+      <c r="E1469" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1469" s="5" t="n"/>
     </row>
     <row r="1470" ht="20.25" customHeight="1">
@@ -29897,7 +29909,9 @@
           <t>381087</t>
         </is>
       </c>
-      <c r="E1470" s="5" t="n"/>
+      <c r="E1470" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1470" s="5" t="n"/>
     </row>
     <row r="1471" ht="20.25" customHeight="1">
@@ -29915,7 +29929,9 @@
           <t>381084</t>
         </is>
       </c>
-      <c r="E1471" s="5" t="n"/>
+      <c r="E1471" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1471" s="5" t="n"/>
     </row>
     <row r="1472" ht="20.25" customHeight="1">
@@ -29933,7 +29949,9 @@
           <t>381361</t>
         </is>
       </c>
-      <c r="E1472" s="5" t="n"/>
+      <c r="E1472" s="5" t="n">
+        <v>30</v>
+      </c>
       <c r="F1472" s="5" t="n"/>
     </row>
     <row r="1473" ht="20.25" customHeight="1">
@@ -29951,7 +29969,9 @@
           <t>381085</t>
         </is>
       </c>
-      <c r="E1473" s="5" t="n"/>
+      <c r="E1473" s="5" t="n">
+        <v>48</v>
+      </c>
       <c r="F1473" s="5" t="n"/>
     </row>
     <row r="1474" ht="20.25" customHeight="1">
@@ -29969,7 +29989,9 @@
           <t>381088</t>
         </is>
       </c>
-      <c r="E1474" s="5" t="n"/>
+      <c r="E1474" s="5" t="n">
+        <v>48</v>
+      </c>
       <c r="F1474" s="5" t="n"/>
     </row>
     <row r="1475" ht="20.25" customHeight="1">
@@ -29987,7 +30009,9 @@
           <t>381089</t>
         </is>
       </c>
-      <c r="E1475" s="5" t="n"/>
+      <c r="E1475" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1475" s="5" t="n"/>
     </row>
     <row r="1476" ht="20.25" customHeight="1">
@@ -30005,7 +30029,9 @@
           <t>381086</t>
         </is>
       </c>
-      <c r="E1476" s="5" t="n"/>
+      <c r="E1476" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1476" s="5" t="n"/>
     </row>
     <row r="1477" ht="20.25" customHeight="1">
@@ -30023,7 +30049,9 @@
           <t>381360</t>
         </is>
       </c>
-      <c r="E1477" s="5" t="n"/>
+      <c r="E1477" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1477" s="5" t="n"/>
     </row>
     <row r="1478" ht="20.25" customHeight="1">
@@ -30041,7 +30069,9 @@
           <t>381365</t>
         </is>
       </c>
-      <c r="E1478" s="5" t="n"/>
+      <c r="E1478" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1478" s="5" t="n"/>
     </row>
     <row r="1479" ht="20.25" customHeight="1">
@@ -30059,7 +30089,9 @@
           <t>381364</t>
         </is>
       </c>
-      <c r="E1479" s="5" t="n"/>
+      <c r="E1479" s="5" t="n">
+        <v>35</v>
+      </c>
       <c r="F1479" s="5" t="n"/>
     </row>
     <row r="1480" ht="20.25" customHeight="1">
@@ -30077,7 +30109,9 @@
           <t>381363</t>
         </is>
       </c>
-      <c r="E1480" s="5" t="n"/>
+      <c r="E1480" s="5" t="n">
+        <v>48</v>
+      </c>
       <c r="F1480" s="5" t="n"/>
     </row>
     <row r="1481" ht="20.25" customHeight="1">
@@ -30095,7 +30129,9 @@
           <t>381366</t>
         </is>
       </c>
-      <c r="E1481" s="5" t="n"/>
+      <c r="E1481" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1481" s="5" t="n"/>
     </row>
     <row r="1482" ht="20.25" customHeight="1">
@@ -30113,7 +30149,9 @@
           <t>381284</t>
         </is>
       </c>
-      <c r="E1482" s="5" t="n"/>
+      <c r="E1482" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1482" s="5" t="n"/>
     </row>
     <row r="1483" ht="20.25" customHeight="1">
@@ -30131,7 +30169,9 @@
           <t>381283</t>
         </is>
       </c>
-      <c r="E1483" s="5" t="n"/>
+      <c r="E1483" s="5" t="n">
+        <v>45</v>
+      </c>
       <c r="F1483" s="5" t="n"/>
     </row>
     <row r="1484" ht="20.25" customHeight="1">
@@ -30149,7 +30189,9 @@
           <t>381367</t>
         </is>
       </c>
-      <c r="E1484" s="5" t="n"/>
+      <c r="E1484" s="5" t="n">
+        <v>40</v>
+      </c>
       <c r="F1484" s="5" t="n"/>
     </row>
     <row r="1485" ht="20.25" customHeight="1">
@@ -30167,7 +30209,9 @@
           <t>381092</t>
         </is>
       </c>
-      <c r="E1485" s="5" t="n"/>
+      <c r="E1485" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1485" s="5" t="n"/>
     </row>
     <row r="1486" ht="20.25" customHeight="1">
@@ -30185,7 +30229,9 @@
           <t>381091</t>
         </is>
       </c>
-      <c r="E1486" s="5" t="n"/>
+      <c r="E1486" s="5" t="n">
+        <v>48</v>
+      </c>
       <c r="F1486" s="5" t="n"/>
     </row>
     <row r="1487" ht="20.25" customHeight="1">
@@ -30203,7 +30249,9 @@
           <t>381708</t>
         </is>
       </c>
-      <c r="E1487" s="5" t="n"/>
+      <c r="E1487" s="5" t="n">
+        <v>46</v>
+      </c>
       <c r="F1487" s="5" t="n"/>
     </row>
     <row r="1488" ht="20.25" customHeight="1">
@@ -30221,7 +30269,9 @@
           <t>381804</t>
         </is>
       </c>
-      <c r="E1488" s="5" t="n"/>
+      <c r="E1488" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1488" s="5" t="n"/>
     </row>
     <row r="1489" ht="20.25" customHeight="1">
@@ -30239,7 +30289,9 @@
           <t>381294</t>
         </is>
       </c>
-      <c r="E1489" s="5" t="n"/>
+      <c r="E1489" s="5" t="n">
+        <v>43</v>
+      </c>
       <c r="F1489" s="5" t="n"/>
     </row>
     <row r="1490" ht="20.25" customHeight="1">
@@ -30257,7 +30309,9 @@
           <t>381402</t>
         </is>
       </c>
-      <c r="E1490" s="5" t="n"/>
+      <c r="E1490" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1490" s="5" t="n"/>
     </row>
     <row r="1491" ht="20.25" customHeight="1">
@@ -30275,7 +30329,9 @@
           <t>381377</t>
         </is>
       </c>
-      <c r="E1491" s="5" t="n"/>
+      <c r="E1491" s="5" t="n">
+        <v>49</v>
+      </c>
       <c r="F1491" s="5" t="n"/>
     </row>
     <row r="1492" ht="20.25" customHeight="1">
@@ -30293,7 +30349,9 @@
           <t>381287</t>
         </is>
       </c>
-      <c r="E1492" s="5" t="n"/>
+      <c r="E1492" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1492" s="5" t="n"/>
     </row>
     <row r="1493" ht="20.25" customHeight="1">
@@ -30311,7 +30369,9 @@
           <t>381286</t>
         </is>
       </c>
-      <c r="E1493" s="5" t="n"/>
+      <c r="E1493" s="5" t="n">
+        <v>39</v>
+      </c>
       <c r="F1493" s="5" t="n"/>
     </row>
     <row r="1494" ht="20.25" customHeight="1">
@@ -30329,7 +30389,9 @@
           <t>381285</t>
         </is>
       </c>
-      <c r="E1494" s="5" t="n"/>
+      <c r="E1494" s="5" t="n">
+        <v>37</v>
+      </c>
       <c r="F1494" s="5" t="n"/>
     </row>
     <row r="1495" ht="20.25" customHeight="1">
@@ -30347,7 +30409,9 @@
           <t>381636</t>
         </is>
       </c>
-      <c r="E1495" s="5" t="n"/>
+      <c r="E1495" s="5" t="n">
+        <v>49</v>
+      </c>
       <c r="F1495" s="5" t="n"/>
     </row>
     <row r="1496" ht="20.25" customHeight="1">
@@ -30365,7 +30429,9 @@
           <t>381637</t>
         </is>
       </c>
-      <c r="E1496" s="5" t="n"/>
+      <c r="E1496" s="5" t="n">
+        <v>46</v>
+      </c>
       <c r="F1496" s="5" t="n"/>
     </row>
     <row r="1497" ht="20.25" customHeight="1">
@@ -30383,7 +30449,9 @@
           <t>381368</t>
         </is>
       </c>
-      <c r="E1497" s="5" t="n"/>
+      <c r="E1497" s="5" t="n">
+        <v>30</v>
+      </c>
       <c r="F1497" s="5" t="n"/>
     </row>
     <row r="1498" ht="20.25" customHeight="1">
@@ -30401,7 +30469,9 @@
           <t>381288</t>
         </is>
       </c>
-      <c r="E1498" s="5" t="n"/>
+      <c r="E1498" s="5" t="n">
+        <v>30</v>
+      </c>
       <c r="F1498" s="5" t="n"/>
     </row>
     <row r="1499" ht="20.25" customHeight="1">
@@ -30419,7 +30489,9 @@
           <t>381638</t>
         </is>
       </c>
-      <c r="E1499" s="5" t="n"/>
+      <c r="E1499" s="5" t="n">
+        <v>42</v>
+      </c>
       <c r="F1499" s="5" t="n"/>
     </row>
     <row r="1500" ht="20.25" customHeight="1">
@@ -30437,7 +30509,9 @@
           <t>381639</t>
         </is>
       </c>
-      <c r="E1500" s="5" t="n"/>
+      <c r="E1500" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1500" s="5" t="n"/>
     </row>
     <row r="1501" ht="20.25" customHeight="1">
@@ -30455,7 +30529,9 @@
           <t>381371</t>
         </is>
       </c>
-      <c r="E1501" s="5" t="n"/>
+      <c r="E1501" s="5" t="n">
+        <v>35</v>
+      </c>
       <c r="F1501" s="5" t="n"/>
     </row>
     <row r="1502" ht="20.25" customHeight="1">
@@ -30473,7 +30549,9 @@
           <t>381370</t>
         </is>
       </c>
-      <c r="E1502" s="5" t="n"/>
+      <c r="E1502" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1502" s="5" t="n"/>
     </row>
     <row r="1503" ht="20.25" customHeight="1">
@@ -30491,7 +30569,9 @@
           <t>381369</t>
         </is>
       </c>
-      <c r="E1503" s="5" t="n"/>
+      <c r="E1503" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1503" s="5" t="n"/>
     </row>
     <row r="1504" ht="20.25" customHeight="1">
@@ -30509,7 +30589,9 @@
           <t>381094</t>
         </is>
       </c>
-      <c r="E1504" s="5" t="n"/>
+      <c r="E1504" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1504" s="5" t="n"/>
     </row>
     <row r="1505" ht="20.25" customHeight="1">
@@ -30527,7 +30609,9 @@
           <t>381095</t>
         </is>
       </c>
-      <c r="E1505" s="5" t="n"/>
+      <c r="E1505" s="5" t="n">
+        <v>46</v>
+      </c>
       <c r="F1505" s="5" t="n"/>
     </row>
     <row r="1506" ht="20.25" customHeight="1">
@@ -30545,7 +30629,9 @@
           <t>381373</t>
         </is>
       </c>
-      <c r="E1506" s="5" t="n"/>
+      <c r="E1506" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1506" s="5" t="n"/>
     </row>
     <row r="1507" ht="20.25" customHeight="1">
@@ -30563,7 +30649,9 @@
           <t>381712</t>
         </is>
       </c>
-      <c r="E1507" s="5" t="n"/>
+      <c r="E1507" s="5" t="n">
+        <v>39</v>
+      </c>
       <c r="F1507" s="5" t="n"/>
     </row>
     <row r="1508" ht="20.25" customHeight="1">
@@ -30581,7 +30669,9 @@
           <t>381096</t>
         </is>
       </c>
-      <c r="E1508" s="5" t="n"/>
+      <c r="E1508" s="5" t="n">
+        <v>42</v>
+      </c>
       <c r="F1508" s="5" t="n"/>
     </row>
     <row r="1509" ht="20.25" customHeight="1">
@@ -30599,7 +30689,9 @@
           <t>381379</t>
         </is>
       </c>
-      <c r="E1509" s="5" t="n"/>
+      <c r="E1509" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1509" s="5" t="n"/>
     </row>
     <row r="1510" ht="20.25" customHeight="1">
@@ -30617,7 +30709,9 @@
           <t>381807</t>
         </is>
       </c>
-      <c r="E1510" s="5" t="n"/>
+      <c r="E1510" s="5" t="n">
+        <v>48</v>
+      </c>
       <c r="F1510" s="5" t="n"/>
     </row>
     <row r="1511" ht="20.25" customHeight="1">
@@ -30635,7 +30729,9 @@
           <t>381713</t>
         </is>
       </c>
-      <c r="E1511" s="5" t="n"/>
+      <c r="E1511" s="5" t="n">
+        <v>41</v>
+      </c>
       <c r="F1511" s="5" t="n"/>
     </row>
     <row r="1512" ht="20.25" customHeight="1">
@@ -30653,7 +30749,9 @@
           <t>381378</t>
         </is>
       </c>
-      <c r="E1512" s="5" t="n"/>
+      <c r="E1512" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1512" s="5" t="n"/>
     </row>
     <row r="1513" ht="20.25" customHeight="1">
@@ -30671,7 +30769,9 @@
           <t>381290</t>
         </is>
       </c>
-      <c r="E1513" s="5" t="n"/>
+      <c r="E1513" s="5" t="n">
+        <v>42</v>
+      </c>
       <c r="F1513" s="5" t="n"/>
     </row>
     <row r="1514" ht="20.25" customHeight="1">
@@ -30689,7 +30789,9 @@
           <t>381100</t>
         </is>
       </c>
-      <c r="E1514" s="5" t="n"/>
+      <c r="E1514" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1514" s="5" t="n"/>
     </row>
     <row r="1515" ht="20.25" customHeight="1">
@@ -30707,7 +30809,9 @@
           <t>381291</t>
         </is>
       </c>
-      <c r="E1515" s="5" t="n"/>
+      <c r="E1515" s="5" t="n">
+        <v>40</v>
+      </c>
       <c r="F1515" s="5" t="n"/>
     </row>
     <row r="1516" ht="20.25" customHeight="1">
@@ -30725,7 +30829,9 @@
           <t>381701</t>
         </is>
       </c>
-      <c r="E1516" s="5" t="n"/>
+      <c r="E1516" s="5" t="n">
+        <v>45</v>
+      </c>
       <c r="F1516" s="5" t="n"/>
     </row>
     <row r="1517" ht="20.25" customHeight="1">
@@ -30743,7 +30849,9 @@
           <t>381289</t>
         </is>
       </c>
-      <c r="E1517" s="5" t="n"/>
+      <c r="E1517" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1517" s="5" t="n"/>
     </row>
     <row r="1518" ht="20.25" customHeight="1">
@@ -30761,7 +30869,9 @@
           <t>381292</t>
         </is>
       </c>
-      <c r="E1518" s="5" t="n"/>
+      <c r="E1518" s="5" t="n">
+        <v>35</v>
+      </c>
       <c r="F1518" s="5" t="n"/>
     </row>
     <row r="1519" ht="20.25" customHeight="1">
@@ -30779,7 +30889,9 @@
           <t>381293</t>
         </is>
       </c>
-      <c r="E1519" s="5" t="n"/>
+      <c r="E1519" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1519" s="5" t="n"/>
     </row>
     <row r="1520" ht="20.25" customHeight="1">
@@ -30797,7 +30909,9 @@
           <t>381803</t>
         </is>
       </c>
-      <c r="E1520" s="5" t="n"/>
+      <c r="E1520" s="5" t="n">
+        <v>38</v>
+      </c>
       <c r="F1520" s="5" t="n"/>
     </row>
     <row r="1521" ht="20.25" customHeight="1">
@@ -30815,7 +30929,9 @@
           <t>381808</t>
         </is>
       </c>
-      <c r="E1521" s="5" t="n"/>
+      <c r="E1521" s="5" t="n">
+        <v>41</v>
+      </c>
       <c r="F1521" s="5" t="n"/>
     </row>
     <row r="1522" ht="20.25" customHeight="1">
@@ -30833,7 +30949,9 @@
           <t>381295</t>
         </is>
       </c>
-      <c r="E1522" s="5" t="n"/>
+      <c r="E1522" s="5" t="n">
+        <v>34</v>
+      </c>
       <c r="F1522" s="5" t="n"/>
     </row>
     <row r="1523" ht="20.25" customHeight="1">
@@ -30851,7 +30969,9 @@
           <t>381296</t>
         </is>
       </c>
-      <c r="E1523" s="5" t="n"/>
+      <c r="E1523" s="5" t="n">
+        <v>37</v>
+      </c>
       <c r="F1523" s="5" t="n"/>
     </row>
     <row r="1524" ht="20.25" customHeight="1">
@@ -30869,7 +30989,9 @@
           <t>381299</t>
         </is>
       </c>
-      <c r="E1524" s="5" t="n"/>
+      <c r="E1524" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1524" s="5" t="n"/>
     </row>
     <row r="1525" ht="20.25" customHeight="1">
@@ -30887,7 +31009,9 @@
           <t>381375</t>
         </is>
       </c>
-      <c r="E1525" s="5" t="n"/>
+      <c r="E1525" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1525" s="5" t="n"/>
     </row>
     <row r="1526" ht="20.25" customHeight="1">
@@ -30905,7 +31029,9 @@
           <t>381376</t>
         </is>
       </c>
-      <c r="E1526" s="5" t="n"/>
+      <c r="E1526" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1526" s="5" t="n"/>
     </row>
     <row r="1527" ht="20.25" customHeight="1">
@@ -30923,7 +31049,9 @@
           <t>381374</t>
         </is>
       </c>
-      <c r="E1527" s="5" t="n"/>
+      <c r="E1527" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1527" s="5" t="n"/>
     </row>
     <row r="1528" ht="20.25" customHeight="1">
@@ -30941,7 +31069,9 @@
           <t>381703</t>
         </is>
       </c>
-      <c r="E1528" s="5" t="n"/>
+      <c r="E1528" s="5" t="n">
+        <v>46</v>
+      </c>
       <c r="F1528" s="5" t="n"/>
     </row>
     <row r="1529" ht="20.25" customHeight="1">
@@ -30959,7 +31089,9 @@
           <t>381704</t>
         </is>
       </c>
-      <c r="E1529" s="5" t="n"/>
+      <c r="E1529" s="5" t="n">
+        <v>42</v>
+      </c>
       <c r="F1529" s="5" t="n"/>
     </row>
     <row r="1530" ht="20.25" customHeight="1">
@@ -30977,7 +31109,9 @@
           <t>381702</t>
         </is>
       </c>
-      <c r="E1530" s="5" t="n"/>
+      <c r="E1530" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1530" s="5" t="n"/>
     </row>
     <row r="1531" ht="20.25" customHeight="1">
@@ -30995,7 +31129,9 @@
           <t>381706</t>
         </is>
       </c>
-      <c r="E1531" s="5" t="n"/>
+      <c r="E1531" s="5" t="n">
+        <v>48</v>
+      </c>
       <c r="F1531" s="5" t="n"/>
     </row>
     <row r="1532" ht="20.25" customHeight="1">
@@ -31013,7 +31149,9 @@
           <t>381707</t>
         </is>
       </c>
-      <c r="E1532" s="5" t="n"/>
+      <c r="E1532" s="5" t="n">
+        <v>41</v>
+      </c>
       <c r="F1532" s="5" t="n"/>
     </row>
     <row r="1533" ht="20.25" customHeight="1">
@@ -31031,7 +31169,9 @@
           <t>381705</t>
         </is>
       </c>
-      <c r="E1533" s="5" t="n"/>
+      <c r="E1533" s="5" t="n">
+        <v>45</v>
+      </c>
       <c r="F1533" s="5" t="n"/>
     </row>
     <row r="1534" ht="20.25" customHeight="1">
@@ -31049,7 +31189,9 @@
           <t>381709</t>
         </is>
       </c>
-      <c r="E1534" s="5" t="n"/>
+      <c r="E1534" s="5" t="n">
+        <v>43</v>
+      </c>
       <c r="F1534" s="5" t="n"/>
     </row>
     <row r="1535" ht="20.25" customHeight="1">
@@ -31067,7 +31209,9 @@
           <t>381710</t>
         </is>
       </c>
-      <c r="E1535" s="5" t="n"/>
+      <c r="E1535" s="5" t="n">
+        <v>39</v>
+      </c>
       <c r="F1535" s="5" t="n"/>
     </row>
     <row r="1536" ht="20.25" customHeight="1">
@@ -31085,7 +31229,9 @@
           <t>381380</t>
         </is>
       </c>
-      <c r="E1536" s="5" t="n"/>
+      <c r="E1536" s="5" t="n">
+        <v>39</v>
+      </c>
       <c r="F1536" s="5" t="n"/>
     </row>
     <row r="1537" ht="20.25" customHeight="1">
@@ -31103,7 +31249,9 @@
           <t>282389</t>
         </is>
       </c>
-      <c r="E1537" s="5" t="n"/>
+      <c r="E1537" s="5" t="n">
+        <v>37</v>
+      </c>
       <c r="F1537" s="5" t="n"/>
     </row>
     <row r="1538" ht="20.25" customHeight="1">
@@ -31121,7 +31269,9 @@
           <t>125889</t>
         </is>
       </c>
-      <c r="E1538" s="5" t="n"/>
+      <c r="E1538" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1538" s="5" t="n"/>
     </row>
     <row r="1539" ht="20.25" customHeight="1">
@@ -31139,7 +31289,9 @@
           <t>381298</t>
         </is>
       </c>
-      <c r="E1539" s="5" t="n"/>
+      <c r="E1539" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1539" s="5" t="n"/>
     </row>
     <row r="1540" ht="20.25" customHeight="1">
@@ -31157,7 +31309,9 @@
           <t>381711</t>
         </is>
       </c>
-      <c r="E1540" s="5" t="n"/>
+      <c r="E1540" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1540" s="5" t="n"/>
     </row>
     <row r="1541" ht="20.25" customHeight="1">
@@ -31175,7 +31329,9 @@
           <t>381297</t>
         </is>
       </c>
-      <c r="E1541" s="5" t="n"/>
+      <c r="E1541" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="F1541" s="5" t="n"/>
     </row>
     <row r="1542" ht="20.25" customHeight="1">
@@ -31193,7 +31349,9 @@
           <t>381802</t>
         </is>
       </c>
-      <c r="E1542" s="5" t="n"/>
+      <c r="E1542" s="5" t="n">
+        <v>47</v>
+      </c>
       <c r="F1542" s="5" t="n"/>
     </row>
     <row r="1543" ht="20.25" customHeight="1">
@@ -31211,7 +31369,9 @@
           <t>381805</t>
         </is>
       </c>
-      <c r="E1543" s="5" t="n"/>
+      <c r="E1543" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1543" s="5" t="n"/>
     </row>
     <row r="1544" ht="20.25" customHeight="1">
@@ -31229,7 +31389,9 @@
           <t>381806</t>
         </is>
       </c>
-      <c r="E1544" s="5" t="n"/>
+      <c r="E1544" s="5" t="n">
+        <v>36</v>
+      </c>
       <c r="F1544" s="5" t="n"/>
     </row>
     <row r="1545" ht="20.25" customHeight="1">
@@ -31247,7 +31409,9 @@
           <t>381300</t>
         </is>
       </c>
-      <c r="E1545" s="5" t="n"/>
+      <c r="E1545" s="5" t="n">
+        <v>30</v>
+      </c>
       <c r="F1545" s="5" t="n"/>
     </row>
     <row r="1546" ht="20.25" customHeight="1">
@@ -31265,7 +31429,9 @@
           <t>381801</t>
         </is>
       </c>
-      <c r="E1546" s="5" t="n"/>
+      <c r="E1546" s="5" t="n">
+        <v>30</v>
+      </c>
       <c r="F1546" s="5" t="n"/>
     </row>
     <row r="1547" ht="20.25" customHeight="1">
@@ -31283,7 +31449,9 @@
           <t>380886</t>
         </is>
       </c>
-      <c r="E1547" s="5" t="n"/>
+      <c r="E1547" s="5" t="n">
+        <v>34</v>
+      </c>
       <c r="F1547" s="5" t="n"/>
     </row>
     <row r="1548" ht="20.25" customHeight="1">
@@ -31301,7 +31469,9 @@
           <t>381403</t>
         </is>
       </c>
-      <c r="E1548" s="5" t="n"/>
+      <c r="E1548" s="5" t="n">
+        <v>37</v>
+      </c>
       <c r="F1548" s="5" t="n"/>
     </row>
     <row r="1549" ht="20.25" customHeight="1">
@@ -31319,7 +31489,9 @@
           <t>381090</t>
         </is>
       </c>
-      <c r="E1549" s="5" t="n"/>
+      <c r="E1549" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1549" s="5" t="n"/>
     </row>
     <row r="1550" ht="20.25" customHeight="1">
@@ -31337,7 +31509,9 @@
           <t>381093</t>
         </is>
       </c>
-      <c r="E1550" s="5" t="n"/>
+      <c r="E1550" s="5" t="n">
+        <v>44</v>
+      </c>
       <c r="F1550" s="5" t="n"/>
     </row>
     <row r="1551" ht="22" customHeight="1">
@@ -83727,7 +83901,9 @@
           <t>381362</t>
         </is>
       </c>
-      <c r="H1417" s="9" t="n"/>
+      <c r="H1417" s="9" t="n">
+        <v>45</v>
+      </c>
       <c r="I1417" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85316,7 +85492,9 @@
           <t>381098</t>
         </is>
       </c>
-      <c r="H1460" s="9" t="n"/>
+      <c r="H1460" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1460" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85536,7 +85714,9 @@
           <t>381099</t>
         </is>
       </c>
-      <c r="H1466" s="9" t="n"/>
+      <c r="H1466" s="9" t="n">
+        <v>46</v>
+      </c>
       <c r="I1466" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85571,7 +85751,9 @@
           <t>381097</t>
         </is>
       </c>
-      <c r="H1467" s="9" t="n"/>
+      <c r="H1467" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1467" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85606,7 +85788,9 @@
           <t>381372</t>
         </is>
       </c>
-      <c r="H1468" s="9" t="n"/>
+      <c r="H1468" s="9" t="n">
+        <v>37</v>
+      </c>
       <c r="I1468" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85641,7 +85825,9 @@
           <t>381083</t>
         </is>
       </c>
-      <c r="H1469" s="9" t="n"/>
+      <c r="H1469" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1469" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85676,7 +85862,9 @@
           <t>381087</t>
         </is>
       </c>
-      <c r="H1470" s="9" t="n"/>
+      <c r="H1470" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1470" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85711,7 +85899,9 @@
           <t>381084</t>
         </is>
       </c>
-      <c r="H1471" s="9" t="n"/>
+      <c r="H1471" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1471" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85746,7 +85936,9 @@
           <t>381361</t>
         </is>
       </c>
-      <c r="H1472" s="9" t="n"/>
+      <c r="H1472" s="9" t="n">
+        <v>30</v>
+      </c>
       <c r="I1472" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85781,7 +85973,9 @@
           <t>381085</t>
         </is>
       </c>
-      <c r="H1473" s="9" t="n"/>
+      <c r="H1473" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="I1473" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85816,7 +86010,9 @@
           <t>381088</t>
         </is>
       </c>
-      <c r="H1474" s="9" t="n"/>
+      <c r="H1474" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="I1474" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85851,7 +86047,9 @@
           <t>381089</t>
         </is>
       </c>
-      <c r="H1475" s="9" t="n"/>
+      <c r="H1475" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1475" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85886,7 +86084,9 @@
           <t>381086</t>
         </is>
       </c>
-      <c r="H1476" s="9" t="n"/>
+      <c r="H1476" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1476" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85921,7 +86121,9 @@
           <t>381360</t>
         </is>
       </c>
-      <c r="H1477" s="9" t="n"/>
+      <c r="H1477" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1477" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85956,7 +86158,9 @@
           <t>381365</t>
         </is>
       </c>
-      <c r="H1478" s="9" t="n"/>
+      <c r="H1478" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1478" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -85991,7 +86195,9 @@
           <t>381364</t>
         </is>
       </c>
-      <c r="H1479" s="9" t="n"/>
+      <c r="H1479" s="9" t="n">
+        <v>35</v>
+      </c>
       <c r="I1479" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86026,7 +86232,9 @@
           <t>381363</t>
         </is>
       </c>
-      <c r="H1480" s="9" t="n"/>
+      <c r="H1480" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="I1480" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86061,7 +86269,9 @@
           <t>381366</t>
         </is>
       </c>
-      <c r="H1481" s="9" t="n"/>
+      <c r="H1481" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1481" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86096,7 +86306,9 @@
           <t>381284</t>
         </is>
       </c>
-      <c r="H1482" s="9" t="n"/>
+      <c r="H1482" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1482" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86131,7 +86343,9 @@
           <t>381283</t>
         </is>
       </c>
-      <c r="H1483" s="9" t="n"/>
+      <c r="H1483" s="9" t="n">
+        <v>45</v>
+      </c>
       <c r="I1483" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86166,7 +86380,9 @@
           <t>381367</t>
         </is>
       </c>
-      <c r="H1484" s="9" t="n"/>
+      <c r="H1484" s="9" t="n">
+        <v>40</v>
+      </c>
       <c r="I1484" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86201,7 +86417,9 @@
           <t>381092</t>
         </is>
       </c>
-      <c r="H1485" s="9" t="n"/>
+      <c r="H1485" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1485" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86236,7 +86454,9 @@
           <t>381091</t>
         </is>
       </c>
-      <c r="H1486" s="9" t="n"/>
+      <c r="H1486" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="I1486" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86271,7 +86491,9 @@
           <t>381708</t>
         </is>
       </c>
-      <c r="H1487" s="9" t="n"/>
+      <c r="H1487" s="9" t="n">
+        <v>46</v>
+      </c>
       <c r="I1487" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86306,7 +86528,9 @@
           <t>381804</t>
         </is>
       </c>
-      <c r="H1488" s="9" t="n"/>
+      <c r="H1488" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1488" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86341,7 +86565,9 @@
           <t>381294</t>
         </is>
       </c>
-      <c r="H1489" s="9" t="n"/>
+      <c r="H1489" s="9" t="n">
+        <v>43</v>
+      </c>
       <c r="I1489" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86376,7 +86602,9 @@
           <t>381402</t>
         </is>
       </c>
-      <c r="H1490" s="9" t="n"/>
+      <c r="H1490" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1490" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86411,7 +86639,9 @@
           <t>381377</t>
         </is>
       </c>
-      <c r="H1491" s="9" t="n"/>
+      <c r="H1491" s="9" t="n">
+        <v>49</v>
+      </c>
       <c r="I1491" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86446,7 +86676,9 @@
           <t>381287</t>
         </is>
       </c>
-      <c r="H1492" s="9" t="n"/>
+      <c r="H1492" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1492" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86481,7 +86713,9 @@
           <t>381286</t>
         </is>
       </c>
-      <c r="H1493" s="9" t="n"/>
+      <c r="H1493" s="9" t="n">
+        <v>39</v>
+      </c>
       <c r="I1493" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86516,7 +86750,9 @@
           <t>381285</t>
         </is>
       </c>
-      <c r="H1494" s="9" t="n"/>
+      <c r="H1494" s="9" t="n">
+        <v>37</v>
+      </c>
       <c r="I1494" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86551,7 +86787,9 @@
           <t>381636</t>
         </is>
       </c>
-      <c r="H1495" s="9" t="n"/>
+      <c r="H1495" s="9" t="n">
+        <v>49</v>
+      </c>
       <c r="I1495" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86586,7 +86824,9 @@
           <t>381637</t>
         </is>
       </c>
-      <c r="H1496" s="9" t="n"/>
+      <c r="H1496" s="9" t="n">
+        <v>46</v>
+      </c>
       <c r="I1496" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86621,7 +86861,9 @@
           <t>381368</t>
         </is>
       </c>
-      <c r="H1497" s="9" t="n"/>
+      <c r="H1497" s="9" t="n">
+        <v>30</v>
+      </c>
       <c r="I1497" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86656,7 +86898,9 @@
           <t>381288</t>
         </is>
       </c>
-      <c r="H1498" s="9" t="n"/>
+      <c r="H1498" s="9" t="n">
+        <v>30</v>
+      </c>
       <c r="I1498" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86691,7 +86935,9 @@
           <t>381638</t>
         </is>
       </c>
-      <c r="H1499" s="9" t="n"/>
+      <c r="H1499" s="9" t="n">
+        <v>42</v>
+      </c>
       <c r="I1499" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86726,7 +86972,9 @@
           <t>381639</t>
         </is>
       </c>
-      <c r="H1500" s="9" t="n"/>
+      <c r="H1500" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1500" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86761,7 +87009,9 @@
           <t>381371</t>
         </is>
       </c>
-      <c r="H1501" s="9" t="n"/>
+      <c r="H1501" s="9" t="n">
+        <v>35</v>
+      </c>
       <c r="I1501" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86796,7 +87046,9 @@
           <t>381370</t>
         </is>
       </c>
-      <c r="H1502" s="9" t="n"/>
+      <c r="H1502" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1502" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86831,7 +87083,9 @@
           <t>381369</t>
         </is>
       </c>
-      <c r="H1503" s="9" t="n"/>
+      <c r="H1503" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1503" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86866,7 +87120,9 @@
           <t>381094</t>
         </is>
       </c>
-      <c r="H1504" s="9" t="n"/>
+      <c r="H1504" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1504" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86901,7 +87157,9 @@
           <t>381095</t>
         </is>
       </c>
-      <c r="H1505" s="9" t="n"/>
+      <c r="H1505" s="9" t="n">
+        <v>46</v>
+      </c>
       <c r="I1505" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86936,7 +87194,9 @@
           <t>381373</t>
         </is>
       </c>
-      <c r="H1506" s="9" t="n"/>
+      <c r="H1506" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1506" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -86971,7 +87231,9 @@
           <t>381712</t>
         </is>
       </c>
-      <c r="H1507" s="9" t="n"/>
+      <c r="H1507" s="9" t="n">
+        <v>39</v>
+      </c>
       <c r="I1507" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87006,7 +87268,9 @@
           <t>381096</t>
         </is>
       </c>
-      <c r="H1508" s="9" t="n"/>
+      <c r="H1508" s="9" t="n">
+        <v>42</v>
+      </c>
       <c r="I1508" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87041,7 +87305,9 @@
           <t>381379</t>
         </is>
       </c>
-      <c r="H1509" s="9" t="n"/>
+      <c r="H1509" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1509" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87076,7 +87342,9 @@
           <t>381807</t>
         </is>
       </c>
-      <c r="H1510" s="9" t="n"/>
+      <c r="H1510" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="I1510" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87111,7 +87379,9 @@
           <t>381713</t>
         </is>
       </c>
-      <c r="H1511" s="9" t="n"/>
+      <c r="H1511" s="9" t="n">
+        <v>41</v>
+      </c>
       <c r="I1511" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87146,7 +87416,9 @@
           <t>381378</t>
         </is>
       </c>
-      <c r="H1512" s="9" t="n"/>
+      <c r="H1512" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1512" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87181,7 +87453,9 @@
           <t>381290</t>
         </is>
       </c>
-      <c r="H1513" s="9" t="n"/>
+      <c r="H1513" s="9" t="n">
+        <v>42</v>
+      </c>
       <c r="I1513" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87216,7 +87490,9 @@
           <t>381100</t>
         </is>
       </c>
-      <c r="H1514" s="9" t="n"/>
+      <c r="H1514" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1514" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87251,7 +87527,9 @@
           <t>381291</t>
         </is>
       </c>
-      <c r="H1515" s="9" t="n"/>
+      <c r="H1515" s="9" t="n">
+        <v>40</v>
+      </c>
       <c r="I1515" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87286,7 +87564,9 @@
           <t>381701</t>
         </is>
       </c>
-      <c r="H1516" s="9" t="n"/>
+      <c r="H1516" s="9" t="n">
+        <v>45</v>
+      </c>
       <c r="I1516" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87321,7 +87601,9 @@
           <t>381289</t>
         </is>
       </c>
-      <c r="H1517" s="9" t="n"/>
+      <c r="H1517" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1517" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87356,7 +87638,9 @@
           <t>381292</t>
         </is>
       </c>
-      <c r="H1518" s="9" t="n"/>
+      <c r="H1518" s="9" t="n">
+        <v>35</v>
+      </c>
       <c r="I1518" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87391,7 +87675,9 @@
           <t>381293</t>
         </is>
       </c>
-      <c r="H1519" s="9" t="n"/>
+      <c r="H1519" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1519" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87426,7 +87712,9 @@
           <t>381803</t>
         </is>
       </c>
-      <c r="H1520" s="9" t="n"/>
+      <c r="H1520" s="9" t="n">
+        <v>38</v>
+      </c>
       <c r="I1520" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87461,7 +87749,9 @@
           <t>381808</t>
         </is>
       </c>
-      <c r="H1521" s="9" t="n"/>
+      <c r="H1521" s="9" t="n">
+        <v>41</v>
+      </c>
       <c r="I1521" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87496,7 +87786,9 @@
           <t>381295</t>
         </is>
       </c>
-      <c r="H1522" s="9" t="n"/>
+      <c r="H1522" s="9" t="n">
+        <v>34</v>
+      </c>
       <c r="I1522" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87531,7 +87823,9 @@
           <t>381296</t>
         </is>
       </c>
-      <c r="H1523" s="9" t="n"/>
+      <c r="H1523" s="9" t="n">
+        <v>37</v>
+      </c>
       <c r="I1523" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87566,7 +87860,9 @@
           <t>381299</t>
         </is>
       </c>
-      <c r="H1524" s="9" t="n"/>
+      <c r="H1524" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1524" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87601,7 +87897,9 @@
           <t>381375</t>
         </is>
       </c>
-      <c r="H1525" s="9" t="n"/>
+      <c r="H1525" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1525" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87636,7 +87934,9 @@
           <t>381376</t>
         </is>
       </c>
-      <c r="H1526" s="9" t="n"/>
+      <c r="H1526" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1526" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87671,7 +87971,9 @@
           <t>381374</t>
         </is>
       </c>
-      <c r="H1527" s="9" t="n"/>
+      <c r="H1527" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1527" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87706,7 +88008,9 @@
           <t>381703</t>
         </is>
       </c>
-      <c r="H1528" s="9" t="n"/>
+      <c r="H1528" s="9" t="n">
+        <v>46</v>
+      </c>
       <c r="I1528" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87741,7 +88045,9 @@
           <t>381704</t>
         </is>
       </c>
-      <c r="H1529" s="9" t="n"/>
+      <c r="H1529" s="9" t="n">
+        <v>42</v>
+      </c>
       <c r="I1529" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87776,7 +88082,9 @@
           <t>381702</t>
         </is>
       </c>
-      <c r="H1530" s="9" t="n"/>
+      <c r="H1530" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1530" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87811,7 +88119,9 @@
           <t>381706</t>
         </is>
       </c>
-      <c r="H1531" s="9" t="n"/>
+      <c r="H1531" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="I1531" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87846,7 +88156,9 @@
           <t>381707</t>
         </is>
       </c>
-      <c r="H1532" s="9" t="n"/>
+      <c r="H1532" s="9" t="n">
+        <v>41</v>
+      </c>
       <c r="I1532" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87881,7 +88193,9 @@
           <t>381705</t>
         </is>
       </c>
-      <c r="H1533" s="9" t="n"/>
+      <c r="H1533" s="9" t="n">
+        <v>45</v>
+      </c>
       <c r="I1533" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87916,7 +88230,9 @@
           <t>381709</t>
         </is>
       </c>
-      <c r="H1534" s="9" t="n"/>
+      <c r="H1534" s="9" t="n">
+        <v>43</v>
+      </c>
       <c r="I1534" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87951,7 +88267,9 @@
           <t>381710</t>
         </is>
       </c>
-      <c r="H1535" s="9" t="n"/>
+      <c r="H1535" s="9" t="n">
+        <v>39</v>
+      </c>
       <c r="I1535" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -87986,7 +88304,9 @@
           <t>381380</t>
         </is>
       </c>
-      <c r="H1536" s="9" t="n"/>
+      <c r="H1536" s="9" t="n">
+        <v>39</v>
+      </c>
       <c r="I1536" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88021,7 +88341,9 @@
           <t>282389</t>
         </is>
       </c>
-      <c r="H1537" s="9" t="n"/>
+      <c r="H1537" s="9" t="n">
+        <v>37</v>
+      </c>
       <c r="I1537" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88056,7 +88378,9 @@
           <t>125889</t>
         </is>
       </c>
-      <c r="H1538" s="9" t="n"/>
+      <c r="H1538" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1538" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88091,7 +88415,9 @@
           <t>381298</t>
         </is>
       </c>
-      <c r="H1539" s="9" t="n"/>
+      <c r="H1539" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1539" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88126,7 +88452,9 @@
           <t>381711</t>
         </is>
       </c>
-      <c r="H1540" s="9" t="n"/>
+      <c r="H1540" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1540" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88161,7 +88489,9 @@
           <t>381297</t>
         </is>
       </c>
-      <c r="H1541" s="9" t="n"/>
+      <c r="H1541" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="I1541" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88196,7 +88526,9 @@
           <t>381802</t>
         </is>
       </c>
-      <c r="H1542" s="9" t="n"/>
+      <c r="H1542" s="9" t="n">
+        <v>47</v>
+      </c>
       <c r="I1542" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88231,7 +88563,9 @@
           <t>381805</t>
         </is>
       </c>
-      <c r="H1543" s="9" t="n"/>
+      <c r="H1543" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1543" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88266,7 +88600,9 @@
           <t>381806</t>
         </is>
       </c>
-      <c r="H1544" s="9" t="n"/>
+      <c r="H1544" s="9" t="n">
+        <v>36</v>
+      </c>
       <c r="I1544" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88301,7 +88637,9 @@
           <t>381300</t>
         </is>
       </c>
-      <c r="H1545" s="9" t="n"/>
+      <c r="H1545" s="9" t="n">
+        <v>30</v>
+      </c>
       <c r="I1545" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88336,7 +88674,9 @@
           <t>381801</t>
         </is>
       </c>
-      <c r="H1546" s="9" t="n"/>
+      <c r="H1546" s="9" t="n">
+        <v>30</v>
+      </c>
       <c r="I1546" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88371,7 +88711,9 @@
           <t>380886</t>
         </is>
       </c>
-      <c r="H1547" s="9" t="n"/>
+      <c r="H1547" s="9" t="n">
+        <v>34</v>
+      </c>
       <c r="I1547" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88406,7 +88748,9 @@
           <t>381403</t>
         </is>
       </c>
-      <c r="H1548" s="9" t="n"/>
+      <c r="H1548" s="9" t="n">
+        <v>37</v>
+      </c>
       <c r="I1548" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88441,7 +88785,9 @@
           <t>381090</t>
         </is>
       </c>
-      <c r="H1549" s="9" t="n"/>
+      <c r="H1549" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1549" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -88476,7 +88822,9 @@
           <t>381093</t>
         </is>
       </c>
-      <c r="H1550" s="9" t="n"/>
+      <c r="H1550" s="9" t="n">
+        <v>44</v>
+      </c>
       <c r="I1550" s="11" t="inlineStr">
         <is>
           <t>grade 29 sep.xlsx</t>
@@ -89645,15 +89993,11 @@
       <c r="D41" s="9" t="n">
         <v>87</v>
       </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E41" s="9" t="n">
+        <v>3723</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>42.79</v>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>

</xml_diff>